<commit_message>
Update board — 0 notes, 0 done (2026-08-17 14:41)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J2"/>
   <cols>
     <col min="1" max="1" width="11.83203125" customWidth="1"/>
     <col min="2" max="2" width="34.83203125" customWidth="1"/>
@@ -447,103 +447,39 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>T-0K2UA58</v>
+        <v/>
       </c>
       <c r="B2" t="str">
-        <v>Open the Activity log sheet</v>
+        <v/>
       </c>
       <c r="C2" t="str">
-        <v>A dated row for every edit, status change and deletion.</v>
+        <v/>
       </c>
       <c r="D2" t="str">
-        <v>To do</v>
-      </c>
-      <c r="E2">
-        <v>0</v>
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v/>
       </c>
       <c r="F2" t="str">
         <v/>
       </c>
       <c r="G2" t="str">
-        <v>2026-08-17</v>
+        <v/>
       </c>
       <c r="H2" t="str">
         <v/>
       </c>
       <c r="I2" t="str">
-        <v>2026-08-17 14:40</v>
+        <v/>
       </c>
       <c r="J2" t="str">
-        <v>--p3</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>T-0K2UA20</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Drag the progress slider</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Reaching 100% marks the note done and stamps the completion date.</v>
-      </c>
-      <c r="D3" t="str">
-        <v>In progress</v>
-      </c>
-      <c r="E3">
-        <v>40</v>
-      </c>
-      <c r="F3" t="str">
-        <v/>
-      </c>
-      <c r="G3" t="str">
-        <v>2026-08-17</v>
-      </c>
-      <c r="H3" t="str">
-        <v/>
-      </c>
-      <c r="I3" t="str">
-        <v>2026-08-17 14:40</v>
-      </c>
-      <c r="J3" t="str">
-        <v>--p2</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>T-0K2UA73</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Welcome to your board</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Write straight onto a note. Everything is stored in the Excel file — no database anywhere.</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Done</v>
-      </c>
-      <c r="E4">
-        <v>100</v>
-      </c>
-      <c r="F4" t="str">
-        <v/>
-      </c>
-      <c r="G4" t="str">
-        <v>2026-08-17</v>
-      </c>
-      <c r="H4" t="str">
-        <v>2026-08-17</v>
-      </c>
-      <c r="I4" t="str">
-        <v>2026-08-17 14:40</v>
-      </c>
-      <c r="J4" t="str">
-        <v>--p1</v>
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -569,7 +505,7 @@
         <v>Total notes</v>
       </c>
       <c r="B2">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -577,7 +513,7 @@
         <v>To do</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -585,7 +521,7 @@
         <v>In progress</v>
       </c>
       <c r="B4">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -593,7 +529,7 @@
         <v>Done</v>
       </c>
       <c r="B5">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -601,7 +537,7 @@
         <v>Overall progress %</v>
       </c>
       <c r="B6">
-        <v>47</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -617,7 +553,7 @@
         <v>Last saved</v>
       </c>
       <c r="B8" t="str">
-        <v>2026-08-17 14:40</v>
+        <v>2026-08-17 14:41</v>
       </c>
     </row>
   </sheetData>
@@ -629,7 +565,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E7"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -706,9 +642,60 @@
         <v/>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>2026-08-17 14:41</v>
+      </c>
+      <c r="B5" t="str">
+        <v>T-0K2UA73</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Welcome to your board</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Deleted</v>
+      </c>
+      <c r="E5" t="str">
+        <v>was Done at 100%</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>2026-08-17 14:41</v>
+      </c>
+      <c r="B6" t="str">
+        <v>T-0K2UA58</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Open the Activity log sheet</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Deleted</v>
+      </c>
+      <c r="E6" t="str">
+        <v>was To do at 0%</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>2026-08-17 14:41</v>
+      </c>
+      <c r="B7" t="str">
+        <v>T-0K2UA20</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Drag the progress slider</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Deleted</v>
+      </c>
+      <c r="E7" t="str">
+        <v>was In progress at 40%</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 1 notes, 0 done (2026-08-17 15:19)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -5,7 +5,8 @@
   <sheets>
     <sheet name="Tasks" sheetId="1" r:id="rId1"/>
     <sheet name="Summary" sheetId="2" r:id="rId2"/>
-    <sheet name="Activity log" sheetId="3" r:id="rId3"/>
+    <sheet name="Bin" sheetId="3" r:id="rId3"/>
+    <sheet name="Activity log" sheetId="4" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
@@ -447,34 +448,34 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v/>
+        <v>T-1X4UW94</v>
       </c>
       <c r="B2" t="str">
-        <v/>
+        <v xml:space="preserve">Coveo RSP- QPM </v>
       </c>
       <c r="C2" t="str">
         <v/>
       </c>
       <c r="D2" t="str">
-        <v/>
-      </c>
-      <c r="E2" t="str">
-        <v/>
+        <v>To do</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
       </c>
       <c r="F2" t="str">
         <v/>
       </c>
       <c r="G2" t="str">
-        <v/>
+        <v>2026-08-17</v>
       </c>
       <c r="H2" t="str">
         <v/>
       </c>
       <c r="I2" t="str">
-        <v/>
+        <v>2026-08-17 15:19</v>
       </c>
       <c r="J2" t="str">
-        <v/>
+        <v>--p1</v>
       </c>
     </row>
   </sheetData>
@@ -486,7 +487,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -505,7 +506,7 @@
         <v>Total notes</v>
       </c>
       <c r="B2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -513,7 +514,7 @@
         <v>To do</v>
       </c>
       <c r="B3">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -550,22 +551,124 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
+        <v>In bin</v>
+      </c>
+      <c r="B8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
         <v>Last saved</v>
       </c>
-      <c r="B8" t="str">
-        <v>2026-08-17 14:41</v>
+      <c r="B9" t="str">
+        <v>2026-08-17 15:19</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B9"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:K2"/>
+  <cols>
+    <col min="1" max="1" width="11.83203125" customWidth="1"/>
+    <col min="2" max="2" width="34.83203125" customWidth="1"/>
+    <col min="3" max="3" width="52.83203125" customWidth="1"/>
+    <col min="4" max="4" width="13.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="12.83203125" customWidth="1"/>
+    <col min="9" max="9" width="17.83203125" customWidth="1"/>
+    <col min="10" max="10" width="8.83203125" customWidth="1"/>
+    <col min="11" max="11" width="17.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Title</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Notes</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Progress %</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Due date</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Created</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Last updated</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Colour</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Deleted at</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v/>
+      </c>
+      <c r="B2" t="str">
+        <v/>
+      </c>
+      <c r="C2" t="str">
+        <v/>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:K2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E35"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -693,9 +796,485 @@
         <v>was In progress at 40%</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>2026-08-17 15:18</v>
+      </c>
+      <c r="B8" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="C8" t="str">
+        <v>(untitled)</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Created</v>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>2026-08-17 15:18</v>
+      </c>
+      <c r="B9" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="C9" t="str">
+        <v>C</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E9" t="str">
+        <v>C</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>2026-08-17 15:18</v>
+      </c>
+      <c r="B10" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Co</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Co</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>2026-08-17 15:18</v>
+      </c>
+      <c r="B11" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Cov</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Cov</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>2026-08-17 15:18</v>
+      </c>
+      <c r="B12" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Cove</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Cove</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>2026-08-17 15:18</v>
+      </c>
+      <c r="B13" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Coveo</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Coveo</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>2026-08-17 15:18</v>
+      </c>
+      <c r="B14" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="C14" t="str">
+        <v xml:space="preserve">Coveo </v>
+      </c>
+      <c r="D14" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E14" t="str">
+        <v xml:space="preserve">Coveo </v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>2026-08-17 15:18</v>
+      </c>
+      <c r="B15" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Coveo R</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Coveo R</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>2026-08-17 15:18</v>
+      </c>
+      <c r="B16" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Coveo RS</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Coveo RS</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>2026-08-17 15:18</v>
+      </c>
+      <c r="B17" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Coveo RSP</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Coveo RSP</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>2026-08-17 15:18</v>
+      </c>
+      <c r="B18" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Coveo RSP-</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Coveo RSP-</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>2026-08-17 15:18</v>
+      </c>
+      <c r="B19" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="C19" t="str">
+        <v xml:space="preserve">Coveo RSP- </v>
+      </c>
+      <c r="D19" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E19" t="str">
+        <v xml:space="preserve">Coveo RSP- </v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>2026-08-17 15:18</v>
+      </c>
+      <c r="B20" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Coveo RSP- Q</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Coveo RSP- Q</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>2026-08-17 15:18</v>
+      </c>
+      <c r="B21" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Coveo RSP- QM</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Coveo RSP- QM</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>2026-08-17 15:18</v>
+      </c>
+      <c r="B22" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Coveo RSP- QMP</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Coveo RSP- QMP</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>2026-08-17 15:18</v>
+      </c>
+      <c r="B23" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Coveo RSP- QM</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Coveo RSP- QM</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>2026-08-17 15:18</v>
+      </c>
+      <c r="B24" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Coveo RSP- Q</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E24" t="str">
+        <v>Coveo RSP- Q</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>2026-08-17 15:18</v>
+      </c>
+      <c r="B25" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Coveo RSP- QP</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E25" t="str">
+        <v>Coveo RSP- QP</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>2026-08-17 15:18</v>
+      </c>
+      <c r="B26" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Coveo RSP- QPM</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E26" t="str">
+        <v>Coveo RSP- QPM</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>2026-08-17 15:18</v>
+      </c>
+      <c r="B27" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="C27" t="str">
+        <v xml:space="preserve">Coveo RSP- QPM </v>
+      </c>
+      <c r="D27" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E27" t="str">
+        <v xml:space="preserve">Coveo RSP- QPM </v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>2026-08-17 15:19</v>
+      </c>
+      <c r="B28" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Coveo RSP- QPM G</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Coveo RSP- QPM G</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>2026-08-17 15:19</v>
+      </c>
+      <c r="B29" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Coveo RSP- QPM Gr</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E29" t="str">
+        <v>Coveo RSP- QPM Gr</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>2026-08-17 15:19</v>
+      </c>
+      <c r="B30" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Coveo RSP- QPM Gra</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E30" t="str">
+        <v>Coveo RSP- QPM Gra</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>2026-08-17 15:19</v>
+      </c>
+      <c r="B31" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Coveo RSP- QPM Gran</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E31" t="str">
+        <v>Coveo RSP- QPM Gran</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>2026-08-17 15:19</v>
+      </c>
+      <c r="B32" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Coveo RSP- QPM Gra</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E32" t="str">
+        <v>Coveo RSP- QPM Gra</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>2026-08-17 15:19</v>
+      </c>
+      <c r="B33" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Coveo RSP- QPM Gr</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Coveo RSP- QPM Gr</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>2026-08-17 15:19</v>
+      </c>
+      <c r="B34" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Coveo RSP- QPM G</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E34" t="str">
+        <v>Coveo RSP- QPM G</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>2026-08-17 15:19</v>
+      </c>
+      <c r="B35" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="C35" t="str">
+        <v xml:space="preserve">Coveo RSP- QPM </v>
+      </c>
+      <c r="D35" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E35" t="str">
+        <v xml:space="preserve">Coveo RSP- QPM </v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E35"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 1 notes, 0 done (2026-08-17 15:20)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -460,7 +460,7 @@
         <v>In progress</v>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="F2" t="str">
         <v>2026-08-14</v>
@@ -538,7 +538,7 @@
         <v>Overall progress %</v>
       </c>
       <c r="B6">
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7">
@@ -562,7 +562,7 @@
         <v>Last saved</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-17 15:19</v>
+        <v>2026-08-17 15:20</v>
       </c>
     </row>
   </sheetData>
@@ -668,7 +668,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E57"/>
+  <dimension ref="A1:E58"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -1646,9 +1646,26 @@
         <v>2026-08-14</v>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>2026-08-17 15:19</v>
+      </c>
+      <c r="B58" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="C58" t="str">
+        <v>Coveo RSP- QPM for V2 calls</v>
+      </c>
+      <c r="D58" t="str">
+        <v>Progress updated</v>
+      </c>
+      <c r="E58" t="str">
+        <v>0% → 50%</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E57"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E58"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 2 notes, 0 done (2026-08-17 15:20)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J3"/>
   <cols>
     <col min="1" max="1" width="11.83203125" customWidth="1"/>
     <col min="2" max="2" width="34.83203125" customWidth="1"/>
@@ -448,22 +448,22 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>T-1X4UW94</v>
+        <v>T-1YYRK56</v>
       </c>
       <c r="B2" t="str">
-        <v>Coveo RSP- QPM for V2 calls</v>
+        <v/>
       </c>
       <c r="C2" t="str">
         <v/>
       </c>
       <c r="D2" t="str">
-        <v>In progress</v>
+        <v>To do</v>
       </c>
       <c r="E2">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-08-14</v>
+        <v/>
       </c>
       <c r="G2" t="str">
         <v>2026-08-17</v>
@@ -472,15 +472,47 @@
         <v/>
       </c>
       <c r="I2" t="str">
-        <v>2026-08-17 15:19</v>
+        <v>2026-08-17 15:20</v>
       </c>
       <c r="J2" t="str">
+        <v>--p2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Coveo RSP- QPM for V2 calls</v>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v>In progress</v>
+      </c>
+      <c r="E3">
+        <v>50</v>
+      </c>
+      <c r="F3" t="str">
+        <v>2026-08-14</v>
+      </c>
+      <c r="G3" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
+        <v>2026-08-17 15:19</v>
+      </c>
+      <c r="J3" t="str">
         <v>--p1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -506,7 +538,7 @@
         <v>Total notes</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
@@ -514,7 +546,7 @@
         <v>To do</v>
       </c>
       <c r="B3">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -538,7 +570,7 @@
         <v>Overall progress %</v>
       </c>
       <c r="B6">
-        <v>50</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7">
@@ -668,7 +700,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E58"/>
+  <dimension ref="A1:E59"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -1663,9 +1695,26 @@
         <v>0% → 50%</v>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>2026-08-17 15:20</v>
+      </c>
+      <c r="B59" t="str">
+        <v>T-1YYRK56</v>
+      </c>
+      <c r="C59" t="str">
+        <v>(untitled)</v>
+      </c>
+      <c r="D59" t="str">
+        <v>Created</v>
+      </c>
+      <c r="E59" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E58"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E59"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 3 notes, 0 done (2026-08-17 15:21)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J4"/>
   <cols>
     <col min="1" max="1" width="11.83203125" customWidth="1"/>
     <col min="2" max="2" width="34.83203125" customWidth="1"/>
@@ -448,13 +448,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>T-1YYRK56</v>
+        <v>T-1ZZXI87</v>
       </c>
       <c r="B2" t="str">
-        <v>Coveo RSP - Recommendation Go-Live for BOC AU store</v>
+        <v/>
       </c>
       <c r="C2" t="str">
-        <v>for Grant</v>
+        <v/>
       </c>
       <c r="D2" t="str">
         <v>To do</v>
@@ -475,27 +475,27 @@
         <v>2026-08-17 15:20</v>
       </c>
       <c r="J2" t="str">
-        <v>--p2</v>
+        <v>--p3</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>T-1X4UW94</v>
+        <v>T-1YYRK56</v>
       </c>
       <c r="B3" t="str">
-        <v>Coveo RSP- QPM for V2 calls</v>
+        <v>Coveo RSP - Recommendation Go-Live for BOC AU store</v>
       </c>
       <c r="C3" t="str">
+        <v>for Grant</v>
+      </c>
+      <c r="D3" t="str">
+        <v>To do</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3" t="str">
         <v/>
-      </c>
-      <c r="D3" t="str">
-        <v>In progress</v>
-      </c>
-      <c r="E3">
-        <v>50</v>
-      </c>
-      <c r="F3" t="str">
-        <v>2026-08-14</v>
       </c>
       <c r="G3" t="str">
         <v>2026-08-17</v>
@@ -504,15 +504,47 @@
         <v/>
       </c>
       <c r="I3" t="str">
-        <v>2026-08-17 15:19</v>
+        <v>2026-08-17 15:20</v>
       </c>
       <c r="J3" t="str">
+        <v>--p2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Coveo RSP- QPM for V2 calls</v>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v>In progress</v>
+      </c>
+      <c r="E4">
+        <v>50</v>
+      </c>
+      <c r="F4" t="str">
+        <v>2026-08-14</v>
+      </c>
+      <c r="G4" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v>2026-08-17 15:19</v>
+      </c>
+      <c r="J4" t="str">
         <v>--p1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -538,7 +570,7 @@
         <v>Total notes</v>
       </c>
       <c r="B2">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -546,7 +578,7 @@
         <v>To do</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -570,7 +602,7 @@
         <v>Overall progress %</v>
       </c>
       <c r="B6">
-        <v>25</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7">
@@ -594,7 +626,7 @@
         <v>Last saved</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-17 15:20</v>
+        <v>2026-08-17 15:21</v>
       </c>
     </row>
   </sheetData>
@@ -700,7 +732,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E123"/>
+  <dimension ref="A1:E124"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -2800,9 +2832,26 @@
         <v>for Grant</v>
       </c>
     </row>
+    <row r="124">
+      <c r="A124" t="str">
+        <v>2026-08-17 15:20</v>
+      </c>
+      <c r="B124" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C124" t="str">
+        <v>(untitled)</v>
+      </c>
+      <c r="D124" t="str">
+        <v>Created</v>
+      </c>
+      <c r="E124" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E123"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E124"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 4 notes, 0 done (2026-08-17 15:21)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J5"/>
   <cols>
     <col min="1" max="1" width="11.83203125" customWidth="1"/>
     <col min="2" max="2" width="34.83203125" customWidth="1"/>
@@ -448,10 +448,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>T-1ZZXI87</v>
+        <v>T-20UNS57</v>
       </c>
       <c r="B2" t="str">
-        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+        <v/>
       </c>
       <c r="C2" t="str">
         <v/>
@@ -475,18 +475,18 @@
         <v>2026-08-17 15:21</v>
       </c>
       <c r="J2" t="str">
-        <v>--p3</v>
+        <v>--p4</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>T-1YYRK56</v>
+        <v>T-1ZZXI87</v>
       </c>
       <c r="B3" t="str">
-        <v>Coveo RSP - Recommendation Go-Live for BOC AU store</v>
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
       </c>
       <c r="C3" t="str">
-        <v>for Grant</v>
+        <v xml:space="preserve">For grant </v>
       </c>
       <c r="D3" t="str">
         <v>To do</v>
@@ -504,30 +504,30 @@
         <v/>
       </c>
       <c r="I3" t="str">
-        <v>2026-08-17 15:20</v>
+        <v>2026-08-17 15:21</v>
       </c>
       <c r="J3" t="str">
-        <v>--p2</v>
+        <v>--p3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>T-1X4UW94</v>
+        <v>T-1YYRK56</v>
       </c>
       <c r="B4" t="str">
-        <v>Coveo RSP- QPM for V2 calls</v>
+        <v>Coveo RSP - Recommendation Go-Live for BOC AU store</v>
       </c>
       <c r="C4" t="str">
+        <v>for Grant</v>
+      </c>
+      <c r="D4" t="str">
+        <v>To do</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4" t="str">
         <v/>
-      </c>
-      <c r="D4" t="str">
-        <v>In progress</v>
-      </c>
-      <c r="E4">
-        <v>50</v>
-      </c>
-      <c r="F4" t="str">
-        <v>2026-08-14</v>
       </c>
       <c r="G4" t="str">
         <v>2026-08-17</v>
@@ -536,15 +536,47 @@
         <v/>
       </c>
       <c r="I4" t="str">
+        <v>2026-08-17 15:20</v>
+      </c>
+      <c r="J4" t="str">
+        <v>--p2</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Coveo RSP- QPM for V2 calls</v>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v>In progress</v>
+      </c>
+      <c r="E5">
+        <v>50</v>
+      </c>
+      <c r="F5" t="str">
+        <v>2026-08-14</v>
+      </c>
+      <c r="G5" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
         <v>2026-08-17 15:19</v>
       </c>
-      <c r="J4" t="str">
+      <c r="J5" t="str">
         <v>--p1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J5"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -570,7 +602,7 @@
         <v>Total notes</v>
       </c>
       <c r="B2">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">
@@ -578,7 +610,7 @@
         <v>To do</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -602,7 +634,7 @@
         <v>Overall progress %</v>
       </c>
       <c r="B6">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7">
@@ -732,7 +764,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E153"/>
+  <dimension ref="A1:E166"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -3342,9 +3374,230 @@
         <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
       </c>
     </row>
+    <row r="154">
+      <c r="A154" t="str">
+        <v>2026-08-17 15:21</v>
+      </c>
+      <c r="B154" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C154" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D154" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E154" t="str">
+        <v>F</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="str">
+        <v>2026-08-17 15:21</v>
+      </c>
+      <c r="B155" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C155" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D155" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E155" t="str">
+        <v>Fo</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="str">
+        <v>2026-08-17 15:21</v>
+      </c>
+      <c r="B156" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C156" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D156" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E156" t="str">
+        <v>For</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="str">
+        <v>2026-08-17 15:21</v>
+      </c>
+      <c r="B157" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C157" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D157" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E157" t="str">
+        <v xml:space="preserve">For </v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="str">
+        <v>2026-08-17 15:21</v>
+      </c>
+      <c r="B158" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C158" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D158" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E158" t="str">
+        <v>For</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="str">
+        <v>2026-08-17 15:21</v>
+      </c>
+      <c r="B159" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C159" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D159" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E159" t="str">
+        <v xml:space="preserve">For </v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="str">
+        <v>2026-08-17 15:21</v>
+      </c>
+      <c r="B160" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C160" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D160" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E160" t="str">
+        <v>For g</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="str">
+        <v>2026-08-17 15:21</v>
+      </c>
+      <c r="B161" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C161" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D161" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E161" t="str">
+        <v>For gr</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="str">
+        <v>2026-08-17 15:21</v>
+      </c>
+      <c r="B162" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C162" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D162" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E162" t="str">
+        <v>For gra</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="str">
+        <v>2026-08-17 15:21</v>
+      </c>
+      <c r="B163" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C163" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D163" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E163" t="str">
+        <v>For gran</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="str">
+        <v>2026-08-17 15:21</v>
+      </c>
+      <c r="B164" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C164" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D164" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E164" t="str">
+        <v>For grant</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="str">
+        <v>2026-08-17 15:21</v>
+      </c>
+      <c r="B165" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C165" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D165" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E165" t="str">
+        <v xml:space="preserve">For grant </v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="str">
+        <v>2026-08-17 15:21</v>
+      </c>
+      <c r="B166" t="str">
+        <v>T-20UNS57</v>
+      </c>
+      <c r="C166" t="str">
+        <v>(untitled)</v>
+      </c>
+      <c r="D166" t="str">
+        <v>Created</v>
+      </c>
+      <c r="E166" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E153"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E166"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 4 notes, 0 done (2026-08-17 15:22)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -451,7 +451,7 @@
         <v>T-20UNS57</v>
       </c>
       <c r="B2" t="str">
-        <v>DF--4191</v>
+        <v>DF--4191 - New Ve</v>
       </c>
       <c r="C2" t="str">
         <v/>
@@ -472,7 +472,7 @@
         <v/>
       </c>
       <c r="I2" t="str">
-        <v>2026-08-17 15:21</v>
+        <v>2026-08-17 15:22</v>
       </c>
       <c r="J2" t="str">
         <v>--p4</v>
@@ -658,7 +658,7 @@
         <v>Last saved</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-17 15:21</v>
+        <v>2026-08-17 15:22</v>
       </c>
     </row>
   </sheetData>
@@ -764,7 +764,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E174"/>
+  <dimension ref="A1:E183"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -3731,9 +3731,162 @@
         <v>DF--4191</v>
       </c>
     </row>
+    <row r="175">
+      <c r="A175" t="str">
+        <v>2026-08-17 15:22</v>
+      </c>
+      <c r="B175" t="str">
+        <v>T-20UNS57</v>
+      </c>
+      <c r="C175" t="str">
+        <v xml:space="preserve">DF--4191 </v>
+      </c>
+      <c r="D175" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E175" t="str">
+        <v xml:space="preserve">DF--4191 </v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="str">
+        <v>2026-08-17 15:22</v>
+      </c>
+      <c r="B176" t="str">
+        <v>T-20UNS57</v>
+      </c>
+      <c r="C176" t="str">
+        <v>DF--4191 -</v>
+      </c>
+      <c r="D176" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E176" t="str">
+        <v>DF--4191 -</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="str">
+        <v>2026-08-17 15:22</v>
+      </c>
+      <c r="B177" t="str">
+        <v>T-20UNS57</v>
+      </c>
+      <c r="C177" t="str">
+        <v xml:space="preserve">DF--4191 - </v>
+      </c>
+      <c r="D177" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E177" t="str">
+        <v xml:space="preserve">DF--4191 - </v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="str">
+        <v>2026-08-17 15:22</v>
+      </c>
+      <c r="B178" t="str">
+        <v>T-20UNS57</v>
+      </c>
+      <c r="C178" t="str">
+        <v>DF--4191 - N</v>
+      </c>
+      <c r="D178" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E178" t="str">
+        <v>DF--4191 - N</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="str">
+        <v>2026-08-17 15:22</v>
+      </c>
+      <c r="B179" t="str">
+        <v>T-20UNS57</v>
+      </c>
+      <c r="C179" t="str">
+        <v>DF--4191 - Ne</v>
+      </c>
+      <c r="D179" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E179" t="str">
+        <v>DF--4191 - Ne</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="str">
+        <v>2026-08-17 15:22</v>
+      </c>
+      <c r="B180" t="str">
+        <v>T-20UNS57</v>
+      </c>
+      <c r="C180" t="str">
+        <v>DF--4191 - New</v>
+      </c>
+      <c r="D180" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E180" t="str">
+        <v>DF--4191 - New</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="str">
+        <v>2026-08-17 15:22</v>
+      </c>
+      <c r="B181" t="str">
+        <v>T-20UNS57</v>
+      </c>
+      <c r="C181" t="str">
+        <v xml:space="preserve">DF--4191 - New </v>
+      </c>
+      <c r="D181" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E181" t="str">
+        <v xml:space="preserve">DF--4191 - New </v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="str">
+        <v>2026-08-17 15:22</v>
+      </c>
+      <c r="B182" t="str">
+        <v>T-20UNS57</v>
+      </c>
+      <c r="C182" t="str">
+        <v>DF--4191 - New V</v>
+      </c>
+      <c r="D182" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E182" t="str">
+        <v>DF--4191 - New V</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="str">
+        <v>2026-08-17 15:22</v>
+      </c>
+      <c r="B183" t="str">
+        <v>T-20UNS57</v>
+      </c>
+      <c r="C183" t="str">
+        <v>DF--4191 - New Ve</v>
+      </c>
+      <c r="D183" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E183" t="str">
+        <v>DF--4191 - New Ve</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E174"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E183"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 5 notes, 0 done (2026-08-17 15:23)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J6"/>
   <cols>
     <col min="1" max="1" width="11.83203125" customWidth="1"/>
     <col min="2" max="2" width="34.83203125" customWidth="1"/>
@@ -446,49 +446,49 @@
         <v>Colour</v>
       </c>
     </row>
-    <row r="2" xml:space="preserve">
+    <row r="2">
       <c r="A2" t="str">
-        <v>T-20UNS57</v>
+        <v>T-22JLI81</v>
       </c>
       <c r="B2" t="str">
+        <v xml:space="preserve">Coveo </v>
+      </c>
+      <c r="C2" t="str">
+        <v/>
+      </c>
+      <c r="D2" t="str">
+        <v>To do</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
+      <c r="I2" t="str">
+        <v>2026-08-17 15:22</v>
+      </c>
+      <c r="J2" t="str">
+        <v>--p5</v>
+      </c>
+    </row>
+    <row r="3" xml:space="preserve">
+      <c r="A3" t="str">
+        <v>T-20UNS57</v>
+      </c>
+      <c r="B3" t="str">
         <v xml:space="preserve">DF--4191 - New Version Recommendation Model Migration </v>
       </c>
-      <c r="C2" t="str" xml:space="preserve">
+      <c r="C3" t="str" xml:space="preserve">
         <v xml:space="preserve">For 
 RGG and RSW (DE and CH store)</v>
       </c>
-      <c r="D2" t="str">
-        <v>To do</v>
-      </c>
-      <c r="E2">
-        <v>0</v>
-      </c>
-      <c r="F2" t="str">
-        <v/>
-      </c>
-      <c r="G2" t="str">
-        <v>2026-08-17</v>
-      </c>
-      <c r="H2" t="str">
-        <v/>
-      </c>
-      <c r="I2" t="str">
-        <v>2026-08-17 15:22</v>
-      </c>
-      <c r="J2" t="str">
-        <v>--p4</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>T-1ZZXI87</v>
-      </c>
-      <c r="B3" t="str">
-        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
-      </c>
-      <c r="C3" t="str">
-        <v xml:space="preserve">For grant </v>
-      </c>
       <c r="D3" t="str">
         <v>To do</v>
       </c>
@@ -505,21 +505,21 @@
         <v/>
       </c>
       <c r="I3" t="str">
-        <v>2026-08-17 15:21</v>
+        <v>2026-08-17 15:22</v>
       </c>
       <c r="J3" t="str">
-        <v>--p3</v>
+        <v>--p4</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>T-1YYRK56</v>
+        <v>T-1ZZXI87</v>
       </c>
       <c r="B4" t="str">
-        <v>Coveo RSP - Recommendation Go-Live for BOC AU store</v>
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
       </c>
       <c r="C4" t="str">
-        <v>for Grant</v>
+        <v xml:space="preserve">For grant </v>
       </c>
       <c r="D4" t="str">
         <v>To do</v>
@@ -537,30 +537,30 @@
         <v/>
       </c>
       <c r="I4" t="str">
-        <v>2026-08-17 15:20</v>
+        <v>2026-08-17 15:21</v>
       </c>
       <c r="J4" t="str">
-        <v>--p2</v>
+        <v>--p3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>T-1X4UW94</v>
+        <v>T-1YYRK56</v>
       </c>
       <c r="B5" t="str">
-        <v>Coveo RSP- QPM for V2 calls</v>
+        <v>Coveo RSP - Recommendation Go-Live for BOC AU store</v>
       </c>
       <c r="C5" t="str">
+        <v>for Grant</v>
+      </c>
+      <c r="D5" t="str">
+        <v>To do</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5" t="str">
         <v/>
-      </c>
-      <c r="D5" t="str">
-        <v>In progress</v>
-      </c>
-      <c r="E5">
-        <v>50</v>
-      </c>
-      <c r="F5" t="str">
-        <v>2026-08-14</v>
       </c>
       <c r="G5" t="str">
         <v>2026-08-17</v>
@@ -569,15 +569,47 @@
         <v/>
       </c>
       <c r="I5" t="str">
+        <v>2026-08-17 15:20</v>
+      </c>
+      <c r="J5" t="str">
+        <v>--p2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Coveo RSP- QPM for V2 calls</v>
+      </c>
+      <c r="C6" t="str">
+        <v/>
+      </c>
+      <c r="D6" t="str">
+        <v>In progress</v>
+      </c>
+      <c r="E6">
+        <v>50</v>
+      </c>
+      <c r="F6" t="str">
+        <v>2026-08-14</v>
+      </c>
+      <c r="G6" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+      <c r="I6" t="str">
         <v>2026-08-17 15:19</v>
       </c>
-      <c r="J5" t="str">
+      <c r="J6" t="str">
         <v>--p1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J6"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -603,7 +635,7 @@
         <v>Total notes</v>
       </c>
       <c r="B2">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
@@ -611,7 +643,7 @@
         <v>To do</v>
       </c>
       <c r="B3">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -635,7 +667,7 @@
         <v>Overall progress %</v>
       </c>
       <c r="B6">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7">
@@ -659,7 +691,7 @@
         <v>Last saved</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-17 15:22</v>
+        <v>2026-08-17 15:23</v>
       </c>
     </row>
   </sheetData>
@@ -765,7 +797,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E256"/>
+  <dimension ref="A1:E263"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -5126,9 +5158,128 @@
         <v>For  RGG and RSW (DE and CH store)</v>
       </c>
     </row>
+    <row r="257">
+      <c r="A257" t="str">
+        <v>2026-08-17 15:22</v>
+      </c>
+      <c r="B257" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C257" t="str">
+        <v>(untitled)</v>
+      </c>
+      <c r="D257" t="str">
+        <v>Created</v>
+      </c>
+      <c r="E257" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="str">
+        <v>2026-08-17 15:22</v>
+      </c>
+      <c r="B258" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C258" t="str">
+        <v>C</v>
+      </c>
+      <c r="D258" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E258" t="str">
+        <v>C</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="str">
+        <v>2026-08-17 15:22</v>
+      </c>
+      <c r="B259" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C259" t="str">
+        <v>Co</v>
+      </c>
+      <c r="D259" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E259" t="str">
+        <v>Co</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="str">
+        <v>2026-08-17 15:22</v>
+      </c>
+      <c r="B260" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C260" t="str">
+        <v>Cov</v>
+      </c>
+      <c r="D260" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E260" t="str">
+        <v>Cov</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="str">
+        <v>2026-08-17 15:22</v>
+      </c>
+      <c r="B261" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C261" t="str">
+        <v>Cove</v>
+      </c>
+      <c r="D261" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E261" t="str">
+        <v>Cove</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="str">
+        <v>2026-08-17 15:22</v>
+      </c>
+      <c r="B262" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C262" t="str">
+        <v>Coveo</v>
+      </c>
+      <c r="D262" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E262" t="str">
+        <v>Coveo</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="str">
+        <v>2026-08-17 15:22</v>
+      </c>
+      <c r="B263" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C263" t="str">
+        <v xml:space="preserve">Coveo </v>
+      </c>
+      <c r="D263" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E263" t="str">
+        <v xml:space="preserve">Coveo </v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E256"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E263"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 5 notes, 0 done (2026-08-17 15:24)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -446,15 +446,16 @@
         <v>Colour</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" xml:space="preserve">
       <c r="A2" t="str">
         <v>T-22JLI81</v>
       </c>
       <c r="B2" t="str">
-        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and </v>
-      </c>
-      <c r="C2" t="str">
-        <v/>
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="C2" t="str" xml:space="preserve">
+        <v xml:space="preserve">For 
+RSP, RGG, RSW, BOCT</v>
       </c>
       <c r="D2" t="str">
         <v>To do</v>
@@ -472,7 +473,7 @@
         <v/>
       </c>
       <c r="I2" t="str">
-        <v>2026-08-17 15:23</v>
+        <v>2026-08-17 15:24</v>
       </c>
       <c r="J2" t="str">
         <v>--p5</v>
@@ -691,7 +692,7 @@
         <v>Last saved</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-17 15:23</v>
+        <v>2026-08-17 15:24</v>
       </c>
     </row>
   </sheetData>
@@ -797,7 +798,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E335"/>
+  <dimension ref="A1:E402"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -6501,9 +6502,1148 @@
         <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and </v>
       </c>
     </row>
+    <row r="336">
+      <c r="A336" t="str">
+        <v>2026-08-17 15:23</v>
+      </c>
+      <c r="B336" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C336" t="str">
+        <v>Coveo Global Configuration API Deprecation Confirmation and C</v>
+      </c>
+      <c r="D336" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E336" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and </v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="str">
+        <v>2026-08-17 15:23</v>
+      </c>
+      <c r="B337" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C337" t="str">
+        <v>Coveo Global Configuration API Deprecation Confirmation and Co</v>
+      </c>
+      <c r="D337" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E337" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and </v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="str">
+        <v>2026-08-17 15:23</v>
+      </c>
+      <c r="B338" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C338" t="str">
+        <v>Coveo Global Configuration API Deprecation Confirmation and Con</v>
+      </c>
+      <c r="D338" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E338" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and </v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="str">
+        <v>2026-08-17 15:23</v>
+      </c>
+      <c r="B339" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C339" t="str">
+        <v>Coveo Global Configuration API Deprecation Confirmation and Conf</v>
+      </c>
+      <c r="D339" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E339" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and </v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="str">
+        <v>2026-08-17 15:23</v>
+      </c>
+      <c r="B340" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C340" t="str">
+        <v>Coveo Global Configuration API Deprecation Confirmation and Confi</v>
+      </c>
+      <c r="D340" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E340" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and </v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="str">
+        <v>2026-08-17 15:23</v>
+      </c>
+      <c r="B341" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C341" t="str">
+        <v>Coveo Global Configuration API Deprecation Confirmation and Confir</v>
+      </c>
+      <c r="D341" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E341" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and </v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="str">
+        <v>2026-08-17 15:23</v>
+      </c>
+      <c r="B342" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C342" t="str">
+        <v>Coveo Global Configuration API Deprecation Confirmation and Confirm</v>
+      </c>
+      <c r="D342" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E342" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and </v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="str">
+        <v>2026-08-17 15:23</v>
+      </c>
+      <c r="B343" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C343" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm </v>
+      </c>
+      <c r="D343" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E343" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and </v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="str">
+        <v>2026-08-17 15:23</v>
+      </c>
+      <c r="B344" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C344" t="str">
+        <v>Coveo Global Configuration API Deprecation Confirmation and Confirm C</v>
+      </c>
+      <c r="D344" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E344" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and </v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="str">
+        <v>2026-08-17 15:23</v>
+      </c>
+      <c r="B345" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C345" t="str">
+        <v>Coveo Global Configuration API Deprecation Confirmation and Confirm Co</v>
+      </c>
+      <c r="D345" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E345" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and </v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="str">
+        <v>2026-08-17 15:23</v>
+      </c>
+      <c r="B346" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C346" t="str">
+        <v>Coveo Global Configuration API Deprecation Confirmation and Confirm Cov</v>
+      </c>
+      <c r="D346" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E346" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and </v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="str">
+        <v>2026-08-17 15:23</v>
+      </c>
+      <c r="B347" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C347" t="str">
+        <v>Coveo Global Configuration API Deprecation Confirmation and Confirm Cove</v>
+      </c>
+      <c r="D347" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E347" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and </v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="str">
+        <v>2026-08-17 15:23</v>
+      </c>
+      <c r="B348" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C348" t="str">
+        <v>Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo</v>
+      </c>
+      <c r="D348" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E348" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and </v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="str">
+        <v>2026-08-17 15:23</v>
+      </c>
+      <c r="B349" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C349" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo </v>
+      </c>
+      <c r="D349" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E349" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and </v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="str">
+        <v>2026-08-17 15:23</v>
+      </c>
+      <c r="B350" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C350" t="str">
+        <v>Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo f</v>
+      </c>
+      <c r="D350" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E350" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and </v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="str">
+        <v>2026-08-17 15:23</v>
+      </c>
+      <c r="B351" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C351" t="str">
+        <v>Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo fo</v>
+      </c>
+      <c r="D351" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E351" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and </v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="str">
+        <v>2026-08-17 15:23</v>
+      </c>
+      <c r="B352" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C352" t="str">
+        <v>Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for</v>
+      </c>
+      <c r="D352" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E352" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and </v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="str">
+        <v>2026-08-17 15:23</v>
+      </c>
+      <c r="B353" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C353" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for </v>
+      </c>
+      <c r="D353" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E353" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and </v>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="str">
+        <v>2026-08-17 15:23</v>
+      </c>
+      <c r="B354" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C354" t="str">
+        <v>Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for P</v>
+      </c>
+      <c r="D354" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E354" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and </v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="str">
+        <v>2026-08-17 15:23</v>
+      </c>
+      <c r="B355" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C355" t="str">
+        <v>Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Pr</v>
+      </c>
+      <c r="D355" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E355" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and </v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="str">
+        <v>2026-08-17 15:23</v>
+      </c>
+      <c r="B356" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C356" t="str">
+        <v>Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Pro</v>
+      </c>
+      <c r="D356" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E356" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and </v>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="str">
+        <v>2026-08-17 15:23</v>
+      </c>
+      <c r="B357" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C357" t="str">
+        <v>Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Prod</v>
+      </c>
+      <c r="D357" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E357" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and </v>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="str">
+        <v>2026-08-17 15:23</v>
+      </c>
+      <c r="B358" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C358" t="str">
+        <v>Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Produ</v>
+      </c>
+      <c r="D358" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E358" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and </v>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="str">
+        <v>2026-08-17 15:23</v>
+      </c>
+      <c r="B359" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C359" t="str">
+        <v>Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Produc</v>
+      </c>
+      <c r="D359" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E359" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and </v>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="str">
+        <v>2026-08-17 15:23</v>
+      </c>
+      <c r="B360" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C360" t="str">
+        <v>Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Product</v>
+      </c>
+      <c r="D360" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E360" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and </v>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="str">
+        <v>2026-08-17 15:23</v>
+      </c>
+      <c r="B361" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C361" t="str">
+        <v>Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Producti</v>
+      </c>
+      <c r="D361" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E361" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and </v>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="str">
+        <v>2026-08-17 15:23</v>
+      </c>
+      <c r="B362" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C362" t="str">
+        <v>Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Productio</v>
+      </c>
+      <c r="D362" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E362" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and </v>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="str">
+        <v>2026-08-17 15:23</v>
+      </c>
+      <c r="B363" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C363" t="str">
+        <v>Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production</v>
+      </c>
+      <c r="D363" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E363" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and </v>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="str">
+        <v>2026-08-17 15:23</v>
+      </c>
+      <c r="B364" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C364" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D364" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E364" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and </v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="str">
+        <v>2026-08-17 15:23</v>
+      </c>
+      <c r="B365" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C365" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D365" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E365" t="str">
+        <v>F</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="str">
+        <v>2026-08-17 15:23</v>
+      </c>
+      <c r="B366" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C366" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D366" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E366" t="str">
+        <v>Fo</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="str">
+        <v>2026-08-17 15:23</v>
+      </c>
+      <c r="B367" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C367" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D367" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E367" t="str">
+        <v>For</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="str">
+        <v>2026-08-17 15:23</v>
+      </c>
+      <c r="B368" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C368" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D368" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E368" t="str">
+        <v xml:space="preserve">For </v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="str">
+        <v>2026-08-17 15:23</v>
+      </c>
+      <c r="B369" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C369" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D369" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E369" t="str">
+        <v xml:space="preserve">For  </v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="str">
+        <v>2026-08-17 15:23</v>
+      </c>
+      <c r="B370" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C370" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D370" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E370" t="str">
+        <v>For  R</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="str">
+        <v>2026-08-17 15:23</v>
+      </c>
+      <c r="B371" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C371" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D371" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E371" t="str">
+        <v>For  RS</v>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B372" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C372" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D372" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E372" t="str">
+        <v>For  RSP</v>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B373" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C373" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D373" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E373" t="str">
+        <v xml:space="preserve">For  RSP </v>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B374" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C374" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D374" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E374" t="str">
+        <v>For  RSP</v>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B375" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C375" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D375" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E375" t="str">
+        <v>For  RSP,</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B376" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C376" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D376" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E376" t="str">
+        <v xml:space="preserve">For  RSP, </v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B377" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C377" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D377" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E377" t="str">
+        <v>For  RSP, R</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B378" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C378" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D378" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E378" t="str">
+        <v>For  RSP, RG</v>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B379" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C379" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D379" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E379" t="str">
+        <v>For  RSP, RGG</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B380" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C380" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D380" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E380" t="str">
+        <v xml:space="preserve">For  RSP, RGG </v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B381" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C381" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D381" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E381" t="str">
+        <v>For  RSP, RGG</v>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B382" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C382" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D382" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E382" t="str">
+        <v>For  RSP, RGG,</v>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B383" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C383" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D383" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E383" t="str">
+        <v xml:space="preserve">For  RSP, RGG, </v>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B384" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C384" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D384" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E384" t="str">
+        <v>For  RSP, RGG, R</v>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B385" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C385" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D385" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E385" t="str">
+        <v>For  RSP, RGG, RS</v>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B386" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C386" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D386" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E386" t="str">
+        <v>For  RSP, RGG, RSW</v>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B387" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C387" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D387" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E387" t="str">
+        <v>For  RSP, RGG, RSW,</v>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B388" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C388" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D388" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E388" t="str">
+        <v xml:space="preserve">For  RSP, RGG, RSW, </v>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B389" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C389" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D389" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E389" t="str">
+        <v>For  RSP, RGG, RSW, C</v>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B390" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C390" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D390" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E390" t="str">
+        <v>For  RSP, RGG, RSW, CB</v>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B391" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C391" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D391" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E391" t="str">
+        <v>For  RSP, RGG, RSW, CBO</v>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B392" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C392" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D392" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E392" t="str">
+        <v>For  RSP, RGG, RSW, CBOC</v>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B393" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C393" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D393" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E393" t="str">
+        <v>For  RSP, RGG, RSW, CBOCT</v>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B394" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C394" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D394" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E394" t="str">
+        <v>For  RSP, RGG, RSW, CBOC</v>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B395" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C395" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D395" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E395" t="str">
+        <v>For  RSP, RGG, RSW, CBO</v>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B396" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C396" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D396" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E396" t="str">
+        <v>For  RSP, RGG, RSW, CB</v>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B397" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C397" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D397" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E397" t="str">
+        <v>For  RSP, RGG, RSW, C</v>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B398" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C398" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D398" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E398" t="str">
+        <v xml:space="preserve">For  RSP, RGG, RSW, </v>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B399" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C399" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D399" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E399" t="str">
+        <v>For  RSP, RGG, RSW, B</v>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B400" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C400" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D400" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E400" t="str">
+        <v>For  RSP, RGG, RSW, BO</v>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B401" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C401" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D401" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E401" t="str">
+        <v>For  RSP, RGG, RSW, BOC</v>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B402" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C402" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D402" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E402" t="str">
+        <v>For  RSP, RGG, RSW, BOCT</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E335"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E402"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 6 notes, 0 done (2026-08-17 15:24)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J7"/>
   <cols>
     <col min="1" max="1" width="11.83203125" customWidth="1"/>
     <col min="2" max="2" width="34.83203125" customWidth="1"/>
@@ -446,82 +446,82 @@
         <v>Colour</v>
       </c>
     </row>
-    <row r="2" xml:space="preserve">
+    <row r="2">
       <c r="A2" t="str">
-        <v>T-22JLI81</v>
+        <v>T-24W7H31</v>
       </c>
       <c r="B2" t="str">
+        <v/>
+      </c>
+      <c r="C2" t="str">
+        <v/>
+      </c>
+      <c r="D2" t="str">
+        <v>To do</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
+      <c r="I2" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="J2" t="str">
+        <v>--p6</v>
+      </c>
+    </row>
+    <row r="3" xml:space="preserve">
+      <c r="A3" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="B3" t="str">
         <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
       </c>
-      <c r="C2" t="str" xml:space="preserve">
+      <c r="C3" t="str" xml:space="preserve">
         <v xml:space="preserve">For 
 RSP, RGG, RSW, BOCT</v>
       </c>
-      <c r="D2" t="str">
+      <c r="D3" t="str">
         <v>To do</v>
       </c>
-      <c r="E2">
+      <c r="E3">
         <v>0</v>
       </c>
-      <c r="F2" t="str">
+      <c r="F3" t="str">
         <v/>
       </c>
-      <c r="G2" t="str">
+      <c r="G3" t="str">
         <v>2026-08-17</v>
       </c>
-      <c r="H2" t="str">
+      <c r="H3" t="str">
         <v/>
       </c>
-      <c r="I2" t="str">
+      <c r="I3" t="str">
         <v>2026-08-17 15:24</v>
       </c>
-      <c r="J2" t="str">
+      <c r="J3" t="str">
         <v>--p5</v>
       </c>
     </row>
-    <row r="3" xml:space="preserve">
-      <c r="A3" t="str">
-        <v>T-20UNS57</v>
-      </c>
-      <c r="B3" t="str">
+    <row r="4" xml:space="preserve">
+      <c r="A4" t="str">
+        <v>T-20UNS57</v>
+      </c>
+      <c r="B4" t="str">
         <v xml:space="preserve">DF--4191 - New Version Recommendation Model Migration </v>
       </c>
-      <c r="C3" t="str" xml:space="preserve">
+      <c r="C4" t="str" xml:space="preserve">
         <v xml:space="preserve">For 
 RGG and RSW (DE and CH store)</v>
       </c>
-      <c r="D3" t="str">
-        <v>To do</v>
-      </c>
-      <c r="E3">
-        <v>0</v>
-      </c>
-      <c r="F3" t="str">
-        <v/>
-      </c>
-      <c r="G3" t="str">
-        <v>2026-08-17</v>
-      </c>
-      <c r="H3" t="str">
-        <v/>
-      </c>
-      <c r="I3" t="str">
-        <v>2026-08-17 15:22</v>
-      </c>
-      <c r="J3" t="str">
-        <v>--p4</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>T-1ZZXI87</v>
-      </c>
-      <c r="B4" t="str">
-        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
-      </c>
-      <c r="C4" t="str">
-        <v xml:space="preserve">For grant </v>
-      </c>
       <c r="D4" t="str">
         <v>To do</v>
       </c>
@@ -538,21 +538,21 @@
         <v/>
       </c>
       <c r="I4" t="str">
-        <v>2026-08-17 15:21</v>
+        <v>2026-08-17 15:22</v>
       </c>
       <c r="J4" t="str">
-        <v>--p3</v>
+        <v>--p4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>T-1YYRK56</v>
+        <v>T-1ZZXI87</v>
       </c>
       <c r="B5" t="str">
-        <v>Coveo RSP - Recommendation Go-Live for BOC AU store</v>
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
       </c>
       <c r="C5" t="str">
-        <v>for Grant</v>
+        <v xml:space="preserve">For grant </v>
       </c>
       <c r="D5" t="str">
         <v>To do</v>
@@ -570,30 +570,30 @@
         <v/>
       </c>
       <c r="I5" t="str">
-        <v>2026-08-17 15:20</v>
+        <v>2026-08-17 15:21</v>
       </c>
       <c r="J5" t="str">
-        <v>--p2</v>
+        <v>--p3</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>T-1X4UW94</v>
+        <v>T-1YYRK56</v>
       </c>
       <c r="B6" t="str">
-        <v>Coveo RSP- QPM for V2 calls</v>
+        <v>Coveo RSP - Recommendation Go-Live for BOC AU store</v>
       </c>
       <c r="C6" t="str">
+        <v>for Grant</v>
+      </c>
+      <c r="D6" t="str">
+        <v>To do</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6" t="str">
         <v/>
-      </c>
-      <c r="D6" t="str">
-        <v>In progress</v>
-      </c>
-      <c r="E6">
-        <v>50</v>
-      </c>
-      <c r="F6" t="str">
-        <v>2026-08-14</v>
       </c>
       <c r="G6" t="str">
         <v>2026-08-17</v>
@@ -602,15 +602,47 @@
         <v/>
       </c>
       <c r="I6" t="str">
+        <v>2026-08-17 15:20</v>
+      </c>
+      <c r="J6" t="str">
+        <v>--p2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Coveo RSP- QPM for V2 calls</v>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+      <c r="D7" t="str">
+        <v>In progress</v>
+      </c>
+      <c r="E7">
+        <v>50</v>
+      </c>
+      <c r="F7" t="str">
+        <v>2026-08-14</v>
+      </c>
+      <c r="G7" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="str">
         <v>2026-08-17 15:19</v>
       </c>
-      <c r="J6" t="str">
+      <c r="J7" t="str">
         <v>--p1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J7"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -636,7 +668,7 @@
         <v>Total notes</v>
       </c>
       <c r="B2">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
@@ -644,7 +676,7 @@
         <v>To do</v>
       </c>
       <c r="B3">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -668,7 +700,7 @@
         <v>Overall progress %</v>
       </c>
       <c r="B6">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7">
@@ -798,7 +830,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E402"/>
+  <dimension ref="A1:E403"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -7641,9 +7673,26 @@
         <v>For  RSP, RGG, RSW, BOCT</v>
       </c>
     </row>
+    <row r="403">
+      <c r="A403" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B403" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C403" t="str">
+        <v>(untitled)</v>
+      </c>
+      <c r="D403" t="str">
+        <v>Created</v>
+      </c>
+      <c r="E403" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E402"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E403"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 6 notes, 0 done (2026-08-17 15:25)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -451,7 +451,7 @@
         <v>T-24W7H31</v>
       </c>
       <c r="B2" t="str">
-        <v/>
+        <v xml:space="preserve">CPD - Follow Up for TBD to matthiew </v>
       </c>
       <c r="C2" t="str">
         <v/>
@@ -472,7 +472,7 @@
         <v/>
       </c>
       <c r="I2" t="str">
-        <v>2026-08-17 15:24</v>
+        <v>2026-08-17 15:25</v>
       </c>
       <c r="J2" t="str">
         <v>--p6</v>
@@ -724,7 +724,7 @@
         <v>Last saved</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-17 15:24</v>
+        <v>2026-08-17 15:25</v>
       </c>
     </row>
   </sheetData>
@@ -830,7 +830,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E403"/>
+  <dimension ref="A1:E455"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -7690,9 +7690,893 @@
         <v/>
       </c>
     </row>
+    <row r="404">
+      <c r="A404" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B404" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C404" t="str">
+        <v>C</v>
+      </c>
+      <c r="D404" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E404" t="str">
+        <v>C</v>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B405" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C405" t="str">
+        <v>CO</v>
+      </c>
+      <c r="D405" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E405" t="str">
+        <v>CO</v>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B406" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C406" t="str">
+        <v>COP</v>
+      </c>
+      <c r="D406" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E406" t="str">
+        <v>COP</v>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B407" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C407" t="str">
+        <v>CO</v>
+      </c>
+      <c r="D407" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E407" t="str">
+        <v>CO</v>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B408" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C408" t="str">
+        <v>C</v>
+      </c>
+      <c r="D408" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E408" t="str">
+        <v>C</v>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B409" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C409" t="str">
+        <v>CP</v>
+      </c>
+      <c r="D409" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E409" t="str">
+        <v>CP</v>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B410" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C410" t="str">
+        <v>CPD</v>
+      </c>
+      <c r="D410" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E410" t="str">
+        <v>CPD</v>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B411" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C411" t="str">
+        <v xml:space="preserve">CPD </v>
+      </c>
+      <c r="D411" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E411" t="str">
+        <v xml:space="preserve">CPD </v>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B412" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C412" t="str">
+        <v>CPD -</v>
+      </c>
+      <c r="D412" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E412" t="str">
+        <v>CPD -</v>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="str">
+        <v>2026-08-17 15:24</v>
+      </c>
+      <c r="B413" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C413" t="str">
+        <v xml:space="preserve">CPD - </v>
+      </c>
+      <c r="D413" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E413" t="str">
+        <v xml:space="preserve">CPD - </v>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B414" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C414" t="str">
+        <v>CPD - F</v>
+      </c>
+      <c r="D414" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E414" t="str">
+        <v>CPD - F</v>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B415" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C415" t="str">
+        <v>CPD - Fo</v>
+      </c>
+      <c r="D415" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E415" t="str">
+        <v>CPD - Fo</v>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B416" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C416" t="str">
+        <v>CPD - Fol</v>
+      </c>
+      <c r="D416" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E416" t="str">
+        <v>CPD - Fol</v>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B417" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C417" t="str">
+        <v>CPD - Foll</v>
+      </c>
+      <c r="D417" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E417" t="str">
+        <v>CPD - Foll</v>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B418" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C418" t="str">
+        <v>CPD - Follo</v>
+      </c>
+      <c r="D418" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E418" t="str">
+        <v>CPD - Follo</v>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B419" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C419" t="str">
+        <v>CPD - Follow</v>
+      </c>
+      <c r="D419" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E419" t="str">
+        <v>CPD - Follow</v>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B420" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C420" t="str">
+        <v xml:space="preserve">CPD - Follow </v>
+      </c>
+      <c r="D420" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E420" t="str">
+        <v xml:space="preserve">CPD - Follow </v>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B421" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C421" t="str">
+        <v>CPD - Follow U</v>
+      </c>
+      <c r="D421" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E421" t="str">
+        <v>CPD - Follow U</v>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B422" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C422" t="str">
+        <v>CPD - Follow Up</v>
+      </c>
+      <c r="D422" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E422" t="str">
+        <v>CPD - Follow Up</v>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B423" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C423" t="str">
+        <v xml:space="preserve">CPD - Follow Up </v>
+      </c>
+      <c r="D423" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E423" t="str">
+        <v xml:space="preserve">CPD - Follow Up </v>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B424" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C424" t="str">
+        <v>CPD - Follow Up f</v>
+      </c>
+      <c r="D424" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E424" t="str">
+        <v>CPD - Follow Up f</v>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B425" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C425" t="str">
+        <v>CPD - Follow Up fr</v>
+      </c>
+      <c r="D425" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E425" t="str">
+        <v>CPD - Follow Up fr</v>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B426" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C426" t="str">
+        <v>CPD - Follow Up fro</v>
+      </c>
+      <c r="D426" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E426" t="str">
+        <v>CPD - Follow Up fro</v>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B427" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C427" t="str">
+        <v xml:space="preserve">CPD - Follow Up fro </v>
+      </c>
+      <c r="D427" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E427" t="str">
+        <v xml:space="preserve">CPD - Follow Up fro </v>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B428" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C428" t="str">
+        <v>CPD - Follow Up fro</v>
+      </c>
+      <c r="D428" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E428" t="str">
+        <v>CPD - Follow Up fro</v>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B429" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C429" t="str">
+        <v>CPD - Follow Up fr</v>
+      </c>
+      <c r="D429" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E429" t="str">
+        <v>CPD - Follow Up fr</v>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B430" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C430" t="str">
+        <v>CPD - Follow Up f</v>
+      </c>
+      <c r="D430" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E430" t="str">
+        <v>CPD - Follow Up f</v>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B431" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C431" t="str">
+        <v>CPD - Follow Up fo</v>
+      </c>
+      <c r="D431" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E431" t="str">
+        <v>CPD - Follow Up fo</v>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B432" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C432" t="str">
+        <v>CPD - Follow Up for</v>
+      </c>
+      <c r="D432" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E432" t="str">
+        <v>CPD - Follow Up for</v>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B433" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C433" t="str">
+        <v xml:space="preserve">CPD - Follow Up for </v>
+      </c>
+      <c r="D433" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E433" t="str">
+        <v xml:space="preserve">CPD - Follow Up for </v>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B434" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C434" t="str">
+        <v>CPD - Follow Up for T</v>
+      </c>
+      <c r="D434" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E434" t="str">
+        <v>CPD - Follow Up for T</v>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B435" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C435" t="str">
+        <v>CPD - Follow Up for TB</v>
+      </c>
+      <c r="D435" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E435" t="str">
+        <v>CPD - Follow Up for TB</v>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B436" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C436" t="str">
+        <v>CPD - Follow Up for TBD</v>
+      </c>
+      <c r="D436" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E436" t="str">
+        <v>CPD - Follow Up for TBD</v>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B437" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C437" t="str">
+        <v xml:space="preserve">CPD - Follow Up for TBD </v>
+      </c>
+      <c r="D437" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E437" t="str">
+        <v xml:space="preserve">CPD - Follow Up for TBD </v>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B438" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C438" t="str">
+        <v>CPD - Follow Up for TBD t</v>
+      </c>
+      <c r="D438" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E438" t="str">
+        <v>CPD - Follow Up for TBD t</v>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B439" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C439" t="str">
+        <v>CPD - Follow Up for TBD to</v>
+      </c>
+      <c r="D439" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E439" t="str">
+        <v>CPD - Follow Up for TBD to</v>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B440" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C440" t="str">
+        <v xml:space="preserve">CPD - Follow Up for TBD to </v>
+      </c>
+      <c r="D440" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E440" t="str">
+        <v xml:space="preserve">CPD - Follow Up for TBD to </v>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B441" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C441" t="str">
+        <v>CPD - Follow Up for TBD to m</v>
+      </c>
+      <c r="D441" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E441" t="str">
+        <v>CPD - Follow Up for TBD to m</v>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B442" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C442" t="str">
+        <v>CPD - Follow Up for TBD to ma</v>
+      </c>
+      <c r="D442" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E442" t="str">
+        <v>CPD - Follow Up for TBD to ma</v>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B443" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C443" t="str">
+        <v>CPD - Follow Up for TBD to mat</v>
+      </c>
+      <c r="D443" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E443" t="str">
+        <v>CPD - Follow Up for TBD to mat</v>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B444" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C444" t="str">
+        <v>CPD - Follow Up for TBD to math</v>
+      </c>
+      <c r="D444" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E444" t="str">
+        <v>CPD - Follow Up for TBD to math</v>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B445" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C445" t="str">
+        <v>CPD - Follow Up for TBD to mathi</v>
+      </c>
+      <c r="D445" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E445" t="str">
+        <v>CPD - Follow Up for TBD to mathi</v>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B446" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C446" t="str">
+        <v>CPD - Follow Up for TBD to mathiw</v>
+      </c>
+      <c r="D446" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E446" t="str">
+        <v>CPD - Follow Up for TBD to mathiw</v>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B447" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C447" t="str">
+        <v>CPD - Follow Up for TBD to mathi</v>
+      </c>
+      <c r="D447" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E447" t="str">
+        <v>CPD - Follow Up for TBD to mathi</v>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B448" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C448" t="str">
+        <v>CPD - Follow Up for TBD to mathie</v>
+      </c>
+      <c r="D448" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E448" t="str">
+        <v>CPD - Follow Up for TBD to mathie</v>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B449" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C449" t="str">
+        <v>CPD - Follow Up for TBD to mathiew</v>
+      </c>
+      <c r="D449" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E449" t="str">
+        <v>CPD - Follow Up for TBD to mathiew</v>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B450" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C450" t="str">
+        <v>CPD - Follow Up for TBD to mathieww</v>
+      </c>
+      <c r="D450" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E450" t="str">
+        <v>CPD - Follow Up for TBD to mathieww</v>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B451" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C451" t="str">
+        <v xml:space="preserve">CPD - Follow Up for TBD to mathieww </v>
+      </c>
+      <c r="D451" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E451" t="str">
+        <v xml:space="preserve">CPD - Follow Up for TBD to mathieww </v>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B452" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C452" t="str">
+        <v>CPD - Follow Up for TBD to mathieww</v>
+      </c>
+      <c r="D452" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E452" t="str">
+        <v>CPD - Follow Up for TBD to mathieww</v>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B453" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C453" t="str">
+        <v>CPD - Follow Up for TBD to mathiew</v>
+      </c>
+      <c r="D453" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E453" t="str">
+        <v>CPD - Follow Up for TBD to mathiew</v>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B454" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C454" t="str">
+        <v xml:space="preserve">CPD - Follow Up for TBD to mathiew </v>
+      </c>
+      <c r="D454" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E454" t="str">
+        <v xml:space="preserve">CPD - Follow Up for TBD to mathiew </v>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B455" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C455" t="str">
+        <v xml:space="preserve">CPD - Follow Up for TBD to matthiew </v>
+      </c>
+      <c r="D455" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E455" t="str">
+        <v xml:space="preserve">CPD - Follow Up for TBD to matthiew </v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E403"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E455"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 13 notes, 0 done (2026-08-17 15:26)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J14"/>
   <cols>
     <col min="1" max="1" width="11.83203125" customWidth="1"/>
     <col min="2" max="2" width="34.83203125" customWidth="1"/>
@@ -448,10 +448,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>T-24W7H31</v>
+        <v>T-26F3171</v>
       </c>
       <c r="B2" t="str">
-        <v xml:space="preserve">CPD - Follow Up for TBD to mathieu </v>
+        <v/>
       </c>
       <c r="C2" t="str">
         <v/>
@@ -475,174 +475,398 @@
         <v>2026-08-17 15:25</v>
       </c>
       <c r="J2" t="str">
+        <v>--p1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>T-26EX299</v>
+      </c>
+      <c r="B3" t="str">
+        <v/>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v>To do</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="J3" t="str">
         <v>--p6</v>
       </c>
     </row>
-    <row r="3" xml:space="preserve">
-      <c r="A3" t="str">
-        <v>T-22JLI81</v>
-      </c>
-      <c r="B3" t="str">
+    <row r="4">
+      <c r="A4" t="str">
+        <v>T-26EEL81</v>
+      </c>
+      <c r="B4" t="str">
+        <v/>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v>To do</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="J4" t="str">
+        <v>--p5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>T-26E9I71</v>
+      </c>
+      <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v>To do</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="J5" t="str">
+        <v>--p4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>T-26D8C38</v>
+      </c>
+      <c r="B6" t="str">
+        <v/>
+      </c>
+      <c r="C6" t="str">
+        <v/>
+      </c>
+      <c r="D6" t="str">
+        <v>To do</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+      <c r="I6" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="J6" t="str">
+        <v>--p3</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>T-26CK499</v>
+      </c>
+      <c r="B7" t="str">
+        <v/>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+      <c r="D7" t="str">
+        <v>To do</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="J7" t="str">
+        <v>--p2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>T-26BWS82</v>
+      </c>
+      <c r="B8" t="str">
+        <v/>
+      </c>
+      <c r="C8" t="str">
+        <v/>
+      </c>
+      <c r="D8" t="str">
+        <v>To do</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H8" t="str">
+        <v/>
+      </c>
+      <c r="I8" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="J8" t="str">
+        <v>--p1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="B9" t="str">
+        <v xml:space="preserve">CPD - Follow Up for TBD to mathieu </v>
+      </c>
+      <c r="C9" t="str">
+        <v/>
+      </c>
+      <c r="D9" t="str">
+        <v>To do</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H9" t="str">
+        <v/>
+      </c>
+      <c r="I9" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="J9" t="str">
+        <v>--p6</v>
+      </c>
+    </row>
+    <row r="10" xml:space="preserve">
+      <c r="A10" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="B10" t="str">
         <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
       </c>
-      <c r="C3" t="str" xml:space="preserve">
+      <c r="C10" t="str" xml:space="preserve">
         <v xml:space="preserve">For 
 RSP, RGG, RSW, BOCT</v>
       </c>
-      <c r="D3" t="str">
+      <c r="D10" t="str">
         <v>To do</v>
       </c>
-      <c r="E3">
+      <c r="E10">
         <v>0</v>
       </c>
-      <c r="F3" t="str">
+      <c r="F10" t="str">
         <v/>
       </c>
-      <c r="G3" t="str">
+      <c r="G10" t="str">
         <v>2026-08-17</v>
       </c>
-      <c r="H3" t="str">
+      <c r="H10" t="str">
         <v/>
       </c>
-      <c r="I3" t="str">
+      <c r="I10" t="str">
         <v>2026-08-17 15:24</v>
       </c>
-      <c r="J3" t="str">
+      <c r="J10" t="str">
         <v>--p5</v>
       </c>
     </row>
-    <row r="4" xml:space="preserve">
-      <c r="A4" t="str">
-        <v>T-20UNS57</v>
-      </c>
-      <c r="B4" t="str">
+    <row r="11" xml:space="preserve">
+      <c r="A11" t="str">
+        <v>T-20UNS57</v>
+      </c>
+      <c r="B11" t="str">
         <v xml:space="preserve">DF--4191 - New Version Recommendation Model Migration </v>
       </c>
-      <c r="C4" t="str" xml:space="preserve">
+      <c r="C11" t="str" xml:space="preserve">
         <v xml:space="preserve">For 
 RGG and RSW (DE and CH store)</v>
       </c>
-      <c r="D4" t="str">
+      <c r="D11" t="str">
         <v>To do</v>
       </c>
-      <c r="E4">
+      <c r="E11">
         <v>0</v>
       </c>
-      <c r="F4" t="str">
+      <c r="F11" t="str">
         <v/>
       </c>
-      <c r="G4" t="str">
+      <c r="G11" t="str">
         <v>2026-08-17</v>
       </c>
-      <c r="H4" t="str">
+      <c r="H11" t="str">
         <v/>
       </c>
-      <c r="I4" t="str">
+      <c r="I11" t="str">
         <v>2026-08-17 15:22</v>
       </c>
-      <c r="J4" t="str">
+      <c r="J11" t="str">
         <v>--p4</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="str">
+    <row r="12">
+      <c r="A12" t="str">
         <v>T-1ZZXI87</v>
       </c>
-      <c r="B5" t="str">
+      <c r="B12" t="str">
         <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
       </c>
-      <c r="C5" t="str">
+      <c r="C12" t="str">
         <v xml:space="preserve">For grant </v>
       </c>
-      <c r="D5" t="str">
+      <c r="D12" t="str">
         <v>To do</v>
       </c>
-      <c r="E5">
+      <c r="E12">
         <v>0</v>
       </c>
-      <c r="F5" t="str">
+      <c r="F12" t="str">
         <v/>
       </c>
-      <c r="G5" t="str">
+      <c r="G12" t="str">
         <v>2026-08-17</v>
       </c>
-      <c r="H5" t="str">
+      <c r="H12" t="str">
         <v/>
       </c>
-      <c r="I5" t="str">
+      <c r="I12" t="str">
         <v>2026-08-17 15:21</v>
       </c>
-      <c r="J5" t="str">
+      <c r="J12" t="str">
         <v>--p3</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="str">
+    <row r="13">
+      <c r="A13" t="str">
         <v>T-1YYRK56</v>
       </c>
-      <c r="B6" t="str">
+      <c r="B13" t="str">
         <v>Coveo RSP - Recommendation Go-Live for BOC AU store</v>
       </c>
-      <c r="C6" t="str">
+      <c r="C13" t="str">
         <v>for Grant</v>
       </c>
-      <c r="D6" t="str">
+      <c r="D13" t="str">
         <v>To do</v>
       </c>
-      <c r="E6">
+      <c r="E13">
         <v>0</v>
       </c>
-      <c r="F6" t="str">
+      <c r="F13" t="str">
         <v/>
       </c>
-      <c r="G6" t="str">
+      <c r="G13" t="str">
         <v>2026-08-17</v>
       </c>
-      <c r="H6" t="str">
+      <c r="H13" t="str">
         <v/>
       </c>
-      <c r="I6" t="str">
+      <c r="I13" t="str">
         <v>2026-08-17 15:20</v>
       </c>
-      <c r="J6" t="str">
+      <c r="J13" t="str">
         <v>--p2</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="str">
+    <row r="14">
+      <c r="A14" t="str">
         <v>T-1X4UW94</v>
       </c>
-      <c r="B7" t="str">
+      <c r="B14" t="str">
         <v>Coveo RSP- QPM for V2 calls</v>
       </c>
-      <c r="C7" t="str">
+      <c r="C14" t="str">
         <v/>
       </c>
-      <c r="D7" t="str">
+      <c r="D14" t="str">
         <v>In progress</v>
       </c>
-      <c r="E7">
+      <c r="E14">
         <v>50</v>
       </c>
-      <c r="F7" t="str">
+      <c r="F14" t="str">
         <v>2026-08-14</v>
       </c>
-      <c r="G7" t="str">
+      <c r="G14" t="str">
         <v>2026-08-17</v>
       </c>
-      <c r="H7" t="str">
+      <c r="H14" t="str">
         <v/>
       </c>
-      <c r="I7" t="str">
+      <c r="I14" t="str">
         <v>2026-08-17 15:19</v>
       </c>
-      <c r="J7" t="str">
+      <c r="J14" t="str">
         <v>--p1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J14"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -668,7 +892,7 @@
         <v>Total notes</v>
       </c>
       <c r="B2">
-        <v>6</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3">
@@ -676,7 +900,7 @@
         <v>To do</v>
       </c>
       <c r="B3">
-        <v>5</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4">
@@ -700,7 +924,7 @@
         <v>Overall progress %</v>
       </c>
       <c r="B6">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
@@ -724,7 +948,7 @@
         <v>Last saved</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-17 15:25</v>
+        <v>2026-08-17 15:26</v>
       </c>
     </row>
   </sheetData>
@@ -830,7 +1054,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E458"/>
+  <dimension ref="A1:E465"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -8625,9 +8849,128 @@
         <v xml:space="preserve">CPD - Follow Up for TBD to mathieu </v>
       </c>
     </row>
+    <row r="459">
+      <c r="A459" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B459" t="str">
+        <v>T-26BWS82</v>
+      </c>
+      <c r="C459" t="str">
+        <v>(untitled)</v>
+      </c>
+      <c r="D459" t="str">
+        <v>Created</v>
+      </c>
+      <c r="E459" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B460" t="str">
+        <v>T-26CK499</v>
+      </c>
+      <c r="C460" t="str">
+        <v>(untitled)</v>
+      </c>
+      <c r="D460" t="str">
+        <v>Created</v>
+      </c>
+      <c r="E460" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B461" t="str">
+        <v>T-26D8C38</v>
+      </c>
+      <c r="C461" t="str">
+        <v>(untitled)</v>
+      </c>
+      <c r="D461" t="str">
+        <v>Created</v>
+      </c>
+      <c r="E461" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B462" t="str">
+        <v>T-26E9I71</v>
+      </c>
+      <c r="C462" t="str">
+        <v>(untitled)</v>
+      </c>
+      <c r="D462" t="str">
+        <v>Created</v>
+      </c>
+      <c r="E462" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B463" t="str">
+        <v>T-26EEL81</v>
+      </c>
+      <c r="C463" t="str">
+        <v>(untitled)</v>
+      </c>
+      <c r="D463" t="str">
+        <v>Created</v>
+      </c>
+      <c r="E463" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B464" t="str">
+        <v>T-26EX299</v>
+      </c>
+      <c r="C464" t="str">
+        <v>(untitled)</v>
+      </c>
+      <c r="D464" t="str">
+        <v>Created</v>
+      </c>
+      <c r="E464" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="B465" t="str">
+        <v>T-26F3171</v>
+      </c>
+      <c r="C465" t="str">
+        <v>(untitled)</v>
+      </c>
+      <c r="D465" t="str">
+        <v>Created</v>
+      </c>
+      <c r="E465" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E458"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E465"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 6 notes, 0 done (2026-08-17 15:26)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J7"/>
   <cols>
     <col min="1" max="1" width="11.83203125" customWidth="1"/>
     <col min="2" max="2" width="34.83203125" customWidth="1"/>
@@ -448,10 +448,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>T-26F3171</v>
+        <v>T-24W7H31</v>
       </c>
       <c r="B2" t="str">
-        <v/>
+        <v xml:space="preserve">CPD - Follow Up for TBD to mathieu </v>
       </c>
       <c r="C2" t="str">
         <v/>
@@ -475,18 +475,19 @@
         <v>2026-08-17 15:25</v>
       </c>
       <c r="J2" t="str">
-        <v>--p1</v>
-      </c>
-    </row>
-    <row r="3">
+        <v>--p6</v>
+      </c>
+    </row>
+    <row r="3" xml:space="preserve">
       <c r="A3" t="str">
-        <v>T-26EX299</v>
+        <v>T-22JLI81</v>
       </c>
       <c r="B3" t="str">
-        <v/>
-      </c>
-      <c r="C3" t="str">
-        <v/>
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="C3" t="str" xml:space="preserve">
+        <v xml:space="preserve">For 
+RSP, RGG, RSW, BOCT</v>
       </c>
       <c r="D3" t="str">
         <v>To do</v>
@@ -504,21 +505,22 @@
         <v/>
       </c>
       <c r="I3" t="str">
-        <v>2026-08-17 15:25</v>
+        <v>2026-08-17 15:24</v>
       </c>
       <c r="J3" t="str">
-        <v>--p6</v>
-      </c>
-    </row>
-    <row r="4">
+        <v>--p5</v>
+      </c>
+    </row>
+    <row r="4" xml:space="preserve">
       <c r="A4" t="str">
-        <v>T-26EEL81</v>
+        <v>T-20UNS57</v>
       </c>
       <c r="B4" t="str">
-        <v/>
-      </c>
-      <c r="C4" t="str">
-        <v/>
+        <v xml:space="preserve">DF--4191 - New Version Recommendation Model Migration </v>
+      </c>
+      <c r="C4" t="str" xml:space="preserve">
+        <v xml:space="preserve">For 
+RGG and RSW (DE and CH store)</v>
       </c>
       <c r="D4" t="str">
         <v>To do</v>
@@ -536,21 +538,21 @@
         <v/>
       </c>
       <c r="I4" t="str">
-        <v>2026-08-17 15:25</v>
+        <v>2026-08-17 15:22</v>
       </c>
       <c r="J4" t="str">
-        <v>--p5</v>
+        <v>--p4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>T-26E9I71</v>
+        <v>T-1ZZXI87</v>
       </c>
       <c r="B5" t="str">
-        <v/>
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
       </c>
       <c r="C5" t="str">
-        <v/>
+        <v xml:space="preserve">For grant </v>
       </c>
       <c r="D5" t="str">
         <v>To do</v>
@@ -568,21 +570,21 @@
         <v/>
       </c>
       <c r="I5" t="str">
-        <v>2026-08-17 15:25</v>
+        <v>2026-08-17 15:21</v>
       </c>
       <c r="J5" t="str">
-        <v>--p4</v>
+        <v>--p3</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>T-26D8C38</v>
+        <v>T-1YYRK56</v>
       </c>
       <c r="B6" t="str">
-        <v/>
+        <v>Coveo RSP - Recommendation Go-Live for BOC AU store</v>
       </c>
       <c r="C6" t="str">
-        <v/>
+        <v>for Grant</v>
       </c>
       <c r="D6" t="str">
         <v>To do</v>
@@ -600,30 +602,30 @@
         <v/>
       </c>
       <c r="I6" t="str">
-        <v>2026-08-17 15:25</v>
+        <v>2026-08-17 15:20</v>
       </c>
       <c r="J6" t="str">
-        <v>--p3</v>
+        <v>--p2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>T-26CK499</v>
+        <v>T-1X4UW94</v>
       </c>
       <c r="B7" t="str">
-        <v/>
+        <v>Coveo RSP- QPM for V2 calls</v>
       </c>
       <c r="C7" t="str">
         <v/>
       </c>
       <c r="D7" t="str">
-        <v>To do</v>
+        <v>In progress</v>
       </c>
       <c r="E7">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="F7" t="str">
-        <v/>
+        <v>2026-08-14</v>
       </c>
       <c r="G7" t="str">
         <v>2026-08-17</v>
@@ -632,241 +634,15 @@
         <v/>
       </c>
       <c r="I7" t="str">
-        <v>2026-08-17 15:25</v>
+        <v>2026-08-17 15:19</v>
       </c>
       <c r="J7" t="str">
-        <v>--p2</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>T-26BWS82</v>
-      </c>
-      <c r="B8" t="str">
-        <v/>
-      </c>
-      <c r="C8" t="str">
-        <v/>
-      </c>
-      <c r="D8" t="str">
-        <v>To do</v>
-      </c>
-      <c r="E8">
-        <v>0</v>
-      </c>
-      <c r="F8" t="str">
-        <v/>
-      </c>
-      <c r="G8" t="str">
-        <v>2026-08-17</v>
-      </c>
-      <c r="H8" t="str">
-        <v/>
-      </c>
-      <c r="I8" t="str">
-        <v>2026-08-17 15:25</v>
-      </c>
-      <c r="J8" t="str">
-        <v>--p1</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>T-24W7H31</v>
-      </c>
-      <c r="B9" t="str">
-        <v xml:space="preserve">CPD - Follow Up for TBD to mathieu </v>
-      </c>
-      <c r="C9" t="str">
-        <v/>
-      </c>
-      <c r="D9" t="str">
-        <v>To do</v>
-      </c>
-      <c r="E9">
-        <v>0</v>
-      </c>
-      <c r="F9" t="str">
-        <v/>
-      </c>
-      <c r="G9" t="str">
-        <v>2026-08-17</v>
-      </c>
-      <c r="H9" t="str">
-        <v/>
-      </c>
-      <c r="I9" t="str">
-        <v>2026-08-17 15:25</v>
-      </c>
-      <c r="J9" t="str">
-        <v>--p6</v>
-      </c>
-    </row>
-    <row r="10" xml:space="preserve">
-      <c r="A10" t="str">
-        <v>T-22JLI81</v>
-      </c>
-      <c r="B10" t="str">
-        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
-      </c>
-      <c r="C10" t="str" xml:space="preserve">
-        <v xml:space="preserve">For 
-RSP, RGG, RSW, BOCT</v>
-      </c>
-      <c r="D10" t="str">
-        <v>To do</v>
-      </c>
-      <c r="E10">
-        <v>0</v>
-      </c>
-      <c r="F10" t="str">
-        <v/>
-      </c>
-      <c r="G10" t="str">
-        <v>2026-08-17</v>
-      </c>
-      <c r="H10" t="str">
-        <v/>
-      </c>
-      <c r="I10" t="str">
-        <v>2026-08-17 15:24</v>
-      </c>
-      <c r="J10" t="str">
-        <v>--p5</v>
-      </c>
-    </row>
-    <row r="11" xml:space="preserve">
-      <c r="A11" t="str">
-        <v>T-20UNS57</v>
-      </c>
-      <c r="B11" t="str">
-        <v xml:space="preserve">DF--4191 - New Version Recommendation Model Migration </v>
-      </c>
-      <c r="C11" t="str" xml:space="preserve">
-        <v xml:space="preserve">For 
-RGG and RSW (DE and CH store)</v>
-      </c>
-      <c r="D11" t="str">
-        <v>To do</v>
-      </c>
-      <c r="E11">
-        <v>0</v>
-      </c>
-      <c r="F11" t="str">
-        <v/>
-      </c>
-      <c r="G11" t="str">
-        <v>2026-08-17</v>
-      </c>
-      <c r="H11" t="str">
-        <v/>
-      </c>
-      <c r="I11" t="str">
-        <v>2026-08-17 15:22</v>
-      </c>
-      <c r="J11" t="str">
-        <v>--p4</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>T-1ZZXI87</v>
-      </c>
-      <c r="B12" t="str">
-        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
-      </c>
-      <c r="C12" t="str">
-        <v xml:space="preserve">For grant </v>
-      </c>
-      <c r="D12" t="str">
-        <v>To do</v>
-      </c>
-      <c r="E12">
-        <v>0</v>
-      </c>
-      <c r="F12" t="str">
-        <v/>
-      </c>
-      <c r="G12" t="str">
-        <v>2026-08-17</v>
-      </c>
-      <c r="H12" t="str">
-        <v/>
-      </c>
-      <c r="I12" t="str">
-        <v>2026-08-17 15:21</v>
-      </c>
-      <c r="J12" t="str">
-        <v>--p3</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>T-1YYRK56</v>
-      </c>
-      <c r="B13" t="str">
-        <v>Coveo RSP - Recommendation Go-Live for BOC AU store</v>
-      </c>
-      <c r="C13" t="str">
-        <v>for Grant</v>
-      </c>
-      <c r="D13" t="str">
-        <v>To do</v>
-      </c>
-      <c r="E13">
-        <v>0</v>
-      </c>
-      <c r="F13" t="str">
-        <v/>
-      </c>
-      <c r="G13" t="str">
-        <v>2026-08-17</v>
-      </c>
-      <c r="H13" t="str">
-        <v/>
-      </c>
-      <c r="I13" t="str">
-        <v>2026-08-17 15:20</v>
-      </c>
-      <c r="J13" t="str">
-        <v>--p2</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>T-1X4UW94</v>
-      </c>
-      <c r="B14" t="str">
-        <v>Coveo RSP- QPM for V2 calls</v>
-      </c>
-      <c r="C14" t="str">
-        <v/>
-      </c>
-      <c r="D14" t="str">
-        <v>In progress</v>
-      </c>
-      <c r="E14">
-        <v>50</v>
-      </c>
-      <c r="F14" t="str">
-        <v>2026-08-14</v>
-      </c>
-      <c r="G14" t="str">
-        <v>2026-08-17</v>
-      </c>
-      <c r="H14" t="str">
-        <v/>
-      </c>
-      <c r="I14" t="str">
-        <v>2026-08-17 15:19</v>
-      </c>
-      <c r="J14" t="str">
         <v>--p1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J7"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -892,7 +668,7 @@
         <v>Total notes</v>
       </c>
       <c r="B2">
-        <v>13</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
@@ -900,7 +676,7 @@
         <v>To do</v>
       </c>
       <c r="B3">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -924,7 +700,7 @@
         <v>Overall progress %</v>
       </c>
       <c r="B6">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7">
@@ -940,7 +716,7 @@
         <v>In bin</v>
       </c>
       <c r="B8">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9">
@@ -960,7 +736,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K8"/>
   <cols>
     <col min="1" max="1" width="11.83203125" customWidth="1"/>
     <col min="2" max="2" width="34.83203125" customWidth="1"/>
@@ -1012,7 +788,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v/>
+        <v>T-26BWS82</v>
       </c>
       <c r="B2" t="str">
         <v/>
@@ -1021,40 +797,250 @@
         <v/>
       </c>
       <c r="D2" t="str">
-        <v/>
-      </c>
-      <c r="E2" t="str">
-        <v/>
+        <v>To do</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
       </c>
       <c r="F2" t="str">
         <v/>
       </c>
       <c r="G2" t="str">
-        <v/>
+        <v>2026-08-17</v>
       </c>
       <c r="H2" t="str">
         <v/>
       </c>
       <c r="I2" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="J2" t="str">
+        <v>--p1</v>
+      </c>
+      <c r="K2" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>T-26CK499</v>
+      </c>
+      <c r="B3" t="str">
         <v/>
       </c>
-      <c r="J2" t="str">
+      <c r="C3" t="str">
         <v/>
       </c>
-      <c r="K2" t="str">
+      <c r="D3" t="str">
+        <v>To do</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3" t="str">
         <v/>
+      </c>
+      <c r="G3" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="J3" t="str">
+        <v>--p2</v>
+      </c>
+      <c r="K3" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>T-26D8C38</v>
+      </c>
+      <c r="B4" t="str">
+        <v/>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v>To do</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="J4" t="str">
+        <v>--p3</v>
+      </c>
+      <c r="K4" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>T-26E9I71</v>
+      </c>
+      <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v>To do</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="J5" t="str">
+        <v>--p4</v>
+      </c>
+      <c r="K5" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>T-26EEL81</v>
+      </c>
+      <c r="B6" t="str">
+        <v/>
+      </c>
+      <c r="C6" t="str">
+        <v/>
+      </c>
+      <c r="D6" t="str">
+        <v>To do</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+      <c r="I6" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="J6" t="str">
+        <v>--p5</v>
+      </c>
+      <c r="K6" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>T-26EX299</v>
+      </c>
+      <c r="B7" t="str">
+        <v/>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+      <c r="D7" t="str">
+        <v>To do</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="J7" t="str">
+        <v>--p6</v>
+      </c>
+      <c r="K7" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>T-26F3171</v>
+      </c>
+      <c r="B8" t="str">
+        <v/>
+      </c>
+      <c r="C8" t="str">
+        <v/>
+      </c>
+      <c r="D8" t="str">
+        <v>To do</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H8" t="str">
+        <v/>
+      </c>
+      <c r="I8" t="str">
+        <v>2026-08-17 15:25</v>
+      </c>
+      <c r="J8" t="str">
+        <v>--p1</v>
+      </c>
+      <c r="K8" t="str">
+        <v>2026-08-17 15:26</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K8"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E465"/>
+  <dimension ref="A1:E472"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -8968,9 +8954,128 @@
         <v/>
       </c>
     </row>
+    <row r="466">
+      <c r="A466" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B466" t="str">
+        <v>T-26F3171</v>
+      </c>
+      <c r="C466" t="str">
+        <v>(untitled)</v>
+      </c>
+      <c r="D466" t="str">
+        <v>Moved to bin</v>
+      </c>
+      <c r="E466" t="str">
+        <v>was To do at 0%</v>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B467" t="str">
+        <v>T-26EX299</v>
+      </c>
+      <c r="C467" t="str">
+        <v>(untitled)</v>
+      </c>
+      <c r="D467" t="str">
+        <v>Moved to bin</v>
+      </c>
+      <c r="E467" t="str">
+        <v>was To do at 0%</v>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B468" t="str">
+        <v>T-26EEL81</v>
+      </c>
+      <c r="C468" t="str">
+        <v>(untitled)</v>
+      </c>
+      <c r="D468" t="str">
+        <v>Moved to bin</v>
+      </c>
+      <c r="E468" t="str">
+        <v>was To do at 0%</v>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B469" t="str">
+        <v>T-26E9I71</v>
+      </c>
+      <c r="C469" t="str">
+        <v>(untitled)</v>
+      </c>
+      <c r="D469" t="str">
+        <v>Moved to bin</v>
+      </c>
+      <c r="E469" t="str">
+        <v>was To do at 0%</v>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B470" t="str">
+        <v>T-26D8C38</v>
+      </c>
+      <c r="C470" t="str">
+        <v>(untitled)</v>
+      </c>
+      <c r="D470" t="str">
+        <v>Moved to bin</v>
+      </c>
+      <c r="E470" t="str">
+        <v>was To do at 0%</v>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B471" t="str">
+        <v>T-26CK499</v>
+      </c>
+      <c r="C471" t="str">
+        <v>(untitled)</v>
+      </c>
+      <c r="D471" t="str">
+        <v>Moved to bin</v>
+      </c>
+      <c r="E471" t="str">
+        <v>was To do at 0%</v>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B472" t="str">
+        <v>T-26BWS82</v>
+      </c>
+      <c r="C472" t="str">
+        <v>(untitled)</v>
+      </c>
+      <c r="D472" t="str">
+        <v>Moved to bin</v>
+      </c>
+      <c r="E472" t="str">
+        <v>was To do at 0%</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E465"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E472"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 7 notes, 0 done (2026-08-17 15:27)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J8"/>
   <cols>
     <col min="1" max="1" width="11.83203125" customWidth="1"/>
     <col min="2" max="2" width="34.83203125" customWidth="1"/>
@@ -448,22 +448,22 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>T-24W7H31</v>
+        <v>T-27I6K43</v>
       </c>
       <c r="B2" t="str">
-        <v xml:space="preserve">CPD - Follow Up for TBD to mathieu </v>
+        <v>Coveo CPD Keys and Configuration</v>
       </c>
       <c r="C2" t="str">
         <v/>
       </c>
       <c r="D2" t="str">
-        <v>To do</v>
+        <v>In progress</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
       <c r="F2" t="str">
-        <v/>
+        <v>2026-08-17</v>
       </c>
       <c r="G2" t="str">
         <v>2026-08-17</v>
@@ -472,88 +472,88 @@
         <v/>
       </c>
       <c r="I2" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="J2" t="str">
+        <v>--p1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="B3" t="str">
+        <v xml:space="preserve">CPD - Follow Up for TBD to mathieu </v>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v>To do</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
         <v>2026-08-17 15:25</v>
       </c>
-      <c r="J2" t="str">
+      <c r="J3" t="str">
         <v>--p6</v>
       </c>
     </row>
-    <row r="3" xml:space="preserve">
-      <c r="A3" t="str">
-        <v>T-22JLI81</v>
-      </c>
-      <c r="B3" t="str">
+    <row r="4" xml:space="preserve">
+      <c r="A4" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="B4" t="str">
         <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
       </c>
-      <c r="C3" t="str" xml:space="preserve">
+      <c r="C4" t="str" xml:space="preserve">
         <v xml:space="preserve">For 
 RSP, RGG, RSW, BOCT</v>
       </c>
-      <c r="D3" t="str">
+      <c r="D4" t="str">
         <v>To do</v>
       </c>
-      <c r="E3">
+      <c r="E4">
         <v>0</v>
       </c>
-      <c r="F3" t="str">
+      <c r="F4" t="str">
         <v/>
       </c>
-      <c r="G3" t="str">
+      <c r="G4" t="str">
         <v>2026-08-17</v>
       </c>
-      <c r="H3" t="str">
+      <c r="H4" t="str">
         <v/>
       </c>
-      <c r="I3" t="str">
+      <c r="I4" t="str">
         <v>2026-08-17 15:24</v>
       </c>
-      <c r="J3" t="str">
+      <c r="J4" t="str">
         <v>--p5</v>
       </c>
     </row>
-    <row r="4" xml:space="preserve">
-      <c r="A4" t="str">
+    <row r="5" xml:space="preserve">
+      <c r="A5" t="str">
         <v>T-20UNS57</v>
       </c>
-      <c r="B4" t="str">
+      <c r="B5" t="str">
         <v xml:space="preserve">DF--4191 - New Version Recommendation Model Migration </v>
       </c>
-      <c r="C4" t="str" xml:space="preserve">
+      <c r="C5" t="str" xml:space="preserve">
         <v xml:space="preserve">For 
 RGG and RSW (DE and CH store)</v>
       </c>
-      <c r="D4" t="str">
-        <v>To do</v>
-      </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-      <c r="F4" t="str">
-        <v/>
-      </c>
-      <c r="G4" t="str">
-        <v>2026-08-17</v>
-      </c>
-      <c r="H4" t="str">
-        <v/>
-      </c>
-      <c r="I4" t="str">
-        <v>2026-08-17 15:22</v>
-      </c>
-      <c r="J4" t="str">
-        <v>--p4</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>T-1ZZXI87</v>
-      </c>
-      <c r="B5" t="str">
-        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
-      </c>
-      <c r="C5" t="str">
-        <v xml:space="preserve">For grant </v>
-      </c>
       <c r="D5" t="str">
         <v>To do</v>
       </c>
@@ -570,21 +570,21 @@
         <v/>
       </c>
       <c r="I5" t="str">
-        <v>2026-08-17 15:21</v>
+        <v>2026-08-17 15:22</v>
       </c>
       <c r="J5" t="str">
-        <v>--p3</v>
+        <v>--p4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>T-1YYRK56</v>
+        <v>T-1ZZXI87</v>
       </c>
       <c r="B6" t="str">
-        <v>Coveo RSP - Recommendation Go-Live for BOC AU store</v>
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
       </c>
       <c r="C6" t="str">
-        <v>for Grant</v>
+        <v xml:space="preserve">For grant </v>
       </c>
       <c r="D6" t="str">
         <v>To do</v>
@@ -602,30 +602,30 @@
         <v/>
       </c>
       <c r="I6" t="str">
-        <v>2026-08-17 15:20</v>
+        <v>2026-08-17 15:21</v>
       </c>
       <c r="J6" t="str">
-        <v>--p2</v>
+        <v>--p3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>T-1X4UW94</v>
+        <v>T-1YYRK56</v>
       </c>
       <c r="B7" t="str">
-        <v>Coveo RSP- QPM for V2 calls</v>
+        <v>Coveo RSP - Recommendation Go-Live for BOC AU store</v>
       </c>
       <c r="C7" t="str">
+        <v>for Grant</v>
+      </c>
+      <c r="D7" t="str">
+        <v>To do</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7" t="str">
         <v/>
-      </c>
-      <c r="D7" t="str">
-        <v>In progress</v>
-      </c>
-      <c r="E7">
-        <v>50</v>
-      </c>
-      <c r="F7" t="str">
-        <v>2026-08-14</v>
       </c>
       <c r="G7" t="str">
         <v>2026-08-17</v>
@@ -634,15 +634,47 @@
         <v/>
       </c>
       <c r="I7" t="str">
+        <v>2026-08-17 15:20</v>
+      </c>
+      <c r="J7" t="str">
+        <v>--p2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Coveo RSP- QPM for V2 calls</v>
+      </c>
+      <c r="C8" t="str">
+        <v/>
+      </c>
+      <c r="D8" t="str">
+        <v>In progress</v>
+      </c>
+      <c r="E8">
+        <v>50</v>
+      </c>
+      <c r="F8" t="str">
+        <v>2026-08-14</v>
+      </c>
+      <c r="G8" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H8" t="str">
+        <v/>
+      </c>
+      <c r="I8" t="str">
         <v>2026-08-17 15:19</v>
       </c>
-      <c r="J7" t="str">
+      <c r="J8" t="str">
         <v>--p1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J8"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -668,7 +700,7 @@
         <v>Total notes</v>
       </c>
       <c r="B2">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3">
@@ -684,7 +716,7 @@
         <v>In progress</v>
       </c>
       <c r="B4">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -700,7 +732,7 @@
         <v>Overall progress %</v>
       </c>
       <c r="B6">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7">
@@ -716,7 +748,7 @@
         <v>In bin</v>
       </c>
       <c r="B8">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -724,7 +756,7 @@
         <v>Last saved</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-17 15:26</v>
+        <v>2026-08-17 15:27</v>
       </c>
     </row>
   </sheetData>
@@ -736,7 +768,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K2"/>
   <cols>
     <col min="1" max="1" width="11.83203125" customWidth="1"/>
     <col min="2" max="2" width="34.83203125" customWidth="1"/>
@@ -788,7 +820,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>T-26BWS82</v>
+        <v/>
       </c>
       <c r="B2" t="str">
         <v/>
@@ -797,250 +829,40 @@
         <v/>
       </c>
       <c r="D2" t="str">
-        <v>To do</v>
-      </c>
-      <c r="E2">
-        <v>0</v>
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v/>
       </c>
       <c r="F2" t="str">
         <v/>
       </c>
       <c r="G2" t="str">
-        <v>2026-08-17</v>
+        <v/>
       </c>
       <c r="H2" t="str">
         <v/>
       </c>
       <c r="I2" t="str">
-        <v>2026-08-17 15:25</v>
+        <v/>
       </c>
       <c r="J2" t="str">
-        <v>--p1</v>
+        <v/>
       </c>
       <c r="K2" t="str">
-        <v>2026-08-17 15:26</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>T-26CK499</v>
-      </c>
-      <c r="B3" t="str">
         <v/>
-      </c>
-      <c r="C3" t="str">
-        <v/>
-      </c>
-      <c r="D3" t="str">
-        <v>To do</v>
-      </c>
-      <c r="E3">
-        <v>0</v>
-      </c>
-      <c r="F3" t="str">
-        <v/>
-      </c>
-      <c r="G3" t="str">
-        <v>2026-08-17</v>
-      </c>
-      <c r="H3" t="str">
-        <v/>
-      </c>
-      <c r="I3" t="str">
-        <v>2026-08-17 15:25</v>
-      </c>
-      <c r="J3" t="str">
-        <v>--p2</v>
-      </c>
-      <c r="K3" t="str">
-        <v>2026-08-17 15:26</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>T-26D8C38</v>
-      </c>
-      <c r="B4" t="str">
-        <v/>
-      </c>
-      <c r="C4" t="str">
-        <v/>
-      </c>
-      <c r="D4" t="str">
-        <v>To do</v>
-      </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-      <c r="F4" t="str">
-        <v/>
-      </c>
-      <c r="G4" t="str">
-        <v>2026-08-17</v>
-      </c>
-      <c r="H4" t="str">
-        <v/>
-      </c>
-      <c r="I4" t="str">
-        <v>2026-08-17 15:25</v>
-      </c>
-      <c r="J4" t="str">
-        <v>--p3</v>
-      </c>
-      <c r="K4" t="str">
-        <v>2026-08-17 15:26</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>T-26E9I71</v>
-      </c>
-      <c r="B5" t="str">
-        <v/>
-      </c>
-      <c r="C5" t="str">
-        <v/>
-      </c>
-      <c r="D5" t="str">
-        <v>To do</v>
-      </c>
-      <c r="E5">
-        <v>0</v>
-      </c>
-      <c r="F5" t="str">
-        <v/>
-      </c>
-      <c r="G5" t="str">
-        <v>2026-08-17</v>
-      </c>
-      <c r="H5" t="str">
-        <v/>
-      </c>
-      <c r="I5" t="str">
-        <v>2026-08-17 15:25</v>
-      </c>
-      <c r="J5" t="str">
-        <v>--p4</v>
-      </c>
-      <c r="K5" t="str">
-        <v>2026-08-17 15:26</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>T-26EEL81</v>
-      </c>
-      <c r="B6" t="str">
-        <v/>
-      </c>
-      <c r="C6" t="str">
-        <v/>
-      </c>
-      <c r="D6" t="str">
-        <v>To do</v>
-      </c>
-      <c r="E6">
-        <v>0</v>
-      </c>
-      <c r="F6" t="str">
-        <v/>
-      </c>
-      <c r="G6" t="str">
-        <v>2026-08-17</v>
-      </c>
-      <c r="H6" t="str">
-        <v/>
-      </c>
-      <c r="I6" t="str">
-        <v>2026-08-17 15:25</v>
-      </c>
-      <c r="J6" t="str">
-        <v>--p5</v>
-      </c>
-      <c r="K6" t="str">
-        <v>2026-08-17 15:26</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>T-26EX299</v>
-      </c>
-      <c r="B7" t="str">
-        <v/>
-      </c>
-      <c r="C7" t="str">
-        <v/>
-      </c>
-      <c r="D7" t="str">
-        <v>To do</v>
-      </c>
-      <c r="E7">
-        <v>0</v>
-      </c>
-      <c r="F7" t="str">
-        <v/>
-      </c>
-      <c r="G7" t="str">
-        <v>2026-08-17</v>
-      </c>
-      <c r="H7" t="str">
-        <v/>
-      </c>
-      <c r="I7" t="str">
-        <v>2026-08-17 15:25</v>
-      </c>
-      <c r="J7" t="str">
-        <v>--p6</v>
-      </c>
-      <c r="K7" t="str">
-        <v>2026-08-17 15:26</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>T-26F3171</v>
-      </c>
-      <c r="B8" t="str">
-        <v/>
-      </c>
-      <c r="C8" t="str">
-        <v/>
-      </c>
-      <c r="D8" t="str">
-        <v>To do</v>
-      </c>
-      <c r="E8">
-        <v>0</v>
-      </c>
-      <c r="F8" t="str">
-        <v/>
-      </c>
-      <c r="G8" t="str">
-        <v>2026-08-17</v>
-      </c>
-      <c r="H8" t="str">
-        <v/>
-      </c>
-      <c r="I8" t="str">
-        <v>2026-08-17 15:25</v>
-      </c>
-      <c r="J8" t="str">
-        <v>--p1</v>
-      </c>
-      <c r="K8" t="str">
-        <v>2026-08-17 15:26</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E472"/>
+  <dimension ref="A1:E514"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -9073,9 +8895,723 @@
         <v>was To do at 0%</v>
       </c>
     </row>
+    <row r="473">
+      <c r="A473" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B473" t="str">
+        <v>T-26BWS82</v>
+      </c>
+      <c r="C473" t="str">
+        <v>(untitled)</v>
+      </c>
+      <c r="D473" t="str">
+        <v>Deleted permanently</v>
+      </c>
+      <c r="E473" t="str">
+        <v>binned 2026-08-17 15:26</v>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B474" t="str">
+        <v>T-26CK499</v>
+      </c>
+      <c r="C474" t="str">
+        <v>(untitled)</v>
+      </c>
+      <c r="D474" t="str">
+        <v>Deleted permanently</v>
+      </c>
+      <c r="E474" t="str">
+        <v>binned 2026-08-17 15:26</v>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B475" t="str">
+        <v>T-26D8C38</v>
+      </c>
+      <c r="C475" t="str">
+        <v>(untitled)</v>
+      </c>
+      <c r="D475" t="str">
+        <v>Deleted permanently</v>
+      </c>
+      <c r="E475" t="str">
+        <v>binned 2026-08-17 15:26</v>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B476" t="str">
+        <v>T-26E9I71</v>
+      </c>
+      <c r="C476" t="str">
+        <v>(untitled)</v>
+      </c>
+      <c r="D476" t="str">
+        <v>Deleted permanently</v>
+      </c>
+      <c r="E476" t="str">
+        <v>binned 2026-08-17 15:26</v>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B477" t="str">
+        <v>T-26EEL81</v>
+      </c>
+      <c r="C477" t="str">
+        <v>(untitled)</v>
+      </c>
+      <c r="D477" t="str">
+        <v>Deleted permanently</v>
+      </c>
+      <c r="E477" t="str">
+        <v>binned 2026-08-17 15:26</v>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B478" t="str">
+        <v>T-26EX299</v>
+      </c>
+      <c r="C478" t="str">
+        <v>(untitled)</v>
+      </c>
+      <c r="D478" t="str">
+        <v>Deleted permanently</v>
+      </c>
+      <c r="E478" t="str">
+        <v>binned 2026-08-17 15:26</v>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B479" t="str">
+        <v>T-26F3171</v>
+      </c>
+      <c r="C479" t="str">
+        <v>(untitled)</v>
+      </c>
+      <c r="D479" t="str">
+        <v>Deleted permanently</v>
+      </c>
+      <c r="E479" t="str">
+        <v>binned 2026-08-17 15:26</v>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B480" t="str">
+        <v>T-27I6K43</v>
+      </c>
+      <c r="C480" t="str">
+        <v>(untitled)</v>
+      </c>
+      <c r="D480" t="str">
+        <v>Created</v>
+      </c>
+      <c r="E480" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B481" t="str">
+        <v>T-27I6K43</v>
+      </c>
+      <c r="C481" t="str">
+        <v>C</v>
+      </c>
+      <c r="D481" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E481" t="str">
+        <v>C</v>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B482" t="str">
+        <v>T-27I6K43</v>
+      </c>
+      <c r="C482" t="str">
+        <v>Co</v>
+      </c>
+      <c r="D482" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E482" t="str">
+        <v>Co</v>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B483" t="str">
+        <v>T-27I6K43</v>
+      </c>
+      <c r="C483" t="str">
+        <v>Cov</v>
+      </c>
+      <c r="D483" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E483" t="str">
+        <v>Cov</v>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B484" t="str">
+        <v>T-27I6K43</v>
+      </c>
+      <c r="C484" t="str">
+        <v>Cove</v>
+      </c>
+      <c r="D484" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E484" t="str">
+        <v>Cove</v>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B485" t="str">
+        <v>T-27I6K43</v>
+      </c>
+      <c r="C485" t="str">
+        <v>Coveo</v>
+      </c>
+      <c r="D485" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E485" t="str">
+        <v>Coveo</v>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B486" t="str">
+        <v>T-27I6K43</v>
+      </c>
+      <c r="C486" t="str">
+        <v xml:space="preserve">Coveo </v>
+      </c>
+      <c r="D486" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E486" t="str">
+        <v xml:space="preserve">Coveo </v>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B487" t="str">
+        <v>T-27I6K43</v>
+      </c>
+      <c r="C487" t="str">
+        <v>Coveo C</v>
+      </c>
+      <c r="D487" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E487" t="str">
+        <v>Coveo C</v>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B488" t="str">
+        <v>T-27I6K43</v>
+      </c>
+      <c r="C488" t="str">
+        <v>Coveo CP</v>
+      </c>
+      <c r="D488" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E488" t="str">
+        <v>Coveo CP</v>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B489" t="str">
+        <v>T-27I6K43</v>
+      </c>
+      <c r="C489" t="str">
+        <v>Coveo CPD</v>
+      </c>
+      <c r="D489" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E489" t="str">
+        <v>Coveo CPD</v>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B490" t="str">
+        <v>T-27I6K43</v>
+      </c>
+      <c r="C490" t="str">
+        <v xml:space="preserve">Coveo CPD </v>
+      </c>
+      <c r="D490" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E490" t="str">
+        <v xml:space="preserve">Coveo CPD </v>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B491" t="str">
+        <v>T-27I6K43</v>
+      </c>
+      <c r="C491" t="str">
+        <v>Coveo CPD K</v>
+      </c>
+      <c r="D491" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E491" t="str">
+        <v>Coveo CPD K</v>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B492" t="str">
+        <v>T-27I6K43</v>
+      </c>
+      <c r="C492" t="str">
+        <v>Coveo CPD Ke</v>
+      </c>
+      <c r="D492" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E492" t="str">
+        <v>Coveo CPD Ke</v>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B493" t="str">
+        <v>T-27I6K43</v>
+      </c>
+      <c r="C493" t="str">
+        <v>Coveo CPD Key</v>
+      </c>
+      <c r="D493" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E493" t="str">
+        <v>Coveo CPD Key</v>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B494" t="str">
+        <v>T-27I6K43</v>
+      </c>
+      <c r="C494" t="str">
+        <v>Coveo CPD Keys</v>
+      </c>
+      <c r="D494" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E494" t="str">
+        <v>Coveo CPD Keys</v>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B495" t="str">
+        <v>T-27I6K43</v>
+      </c>
+      <c r="C495" t="str">
+        <v xml:space="preserve">Coveo CPD Keys </v>
+      </c>
+      <c r="D495" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E495" t="str">
+        <v xml:space="preserve">Coveo CPD Keys </v>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B496" t="str">
+        <v>T-27I6K43</v>
+      </c>
+      <c r="C496" t="str">
+        <v>Coveo CPD Keys a</v>
+      </c>
+      <c r="D496" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E496" t="str">
+        <v>Coveo CPD Keys a</v>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B497" t="str">
+        <v>T-27I6K43</v>
+      </c>
+      <c r="C497" t="str">
+        <v>Coveo CPD Keys an</v>
+      </c>
+      <c r="D497" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E497" t="str">
+        <v>Coveo CPD Keys an</v>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B498" t="str">
+        <v>T-27I6K43</v>
+      </c>
+      <c r="C498" t="str">
+        <v>Coveo CPD Keys and</v>
+      </c>
+      <c r="D498" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E498" t="str">
+        <v>Coveo CPD Keys and</v>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B499" t="str">
+        <v>T-27I6K43</v>
+      </c>
+      <c r="C499" t="str">
+        <v xml:space="preserve">Coveo CPD Keys and </v>
+      </c>
+      <c r="D499" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E499" t="str">
+        <v xml:space="preserve">Coveo CPD Keys and </v>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B500" t="str">
+        <v>T-27I6K43</v>
+      </c>
+      <c r="C500" t="str">
+        <v>Coveo CPD Keys and C</v>
+      </c>
+      <c r="D500" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E500" t="str">
+        <v>Coveo CPD Keys and C</v>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B501" t="str">
+        <v>T-27I6K43</v>
+      </c>
+      <c r="C501" t="str">
+        <v>Coveo CPD Keys and Co</v>
+      </c>
+      <c r="D501" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E501" t="str">
+        <v>Coveo CPD Keys and Co</v>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B502" t="str">
+        <v>T-27I6K43</v>
+      </c>
+      <c r="C502" t="str">
+        <v>Coveo CPD Keys and Con</v>
+      </c>
+      <c r="D502" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E502" t="str">
+        <v>Coveo CPD Keys and Con</v>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B503" t="str">
+        <v>T-27I6K43</v>
+      </c>
+      <c r="C503" t="str">
+        <v>Coveo CPD Keys and Conf</v>
+      </c>
+      <c r="D503" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E503" t="str">
+        <v>Coveo CPD Keys and Conf</v>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B504" t="str">
+        <v>T-27I6K43</v>
+      </c>
+      <c r="C504" t="str">
+        <v>Coveo CPD Keys and Confi</v>
+      </c>
+      <c r="D504" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E504" t="str">
+        <v>Coveo CPD Keys and Confi</v>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B505" t="str">
+        <v>T-27I6K43</v>
+      </c>
+      <c r="C505" t="str">
+        <v>Coveo CPD Keys and Config</v>
+      </c>
+      <c r="D505" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E505" t="str">
+        <v>Coveo CPD Keys and Config</v>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B506" t="str">
+        <v>T-27I6K43</v>
+      </c>
+      <c r="C506" t="str">
+        <v>Coveo CPD Keys and Configu</v>
+      </c>
+      <c r="D506" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E506" t="str">
+        <v>Coveo CPD Keys and Configu</v>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B507" t="str">
+        <v>T-27I6K43</v>
+      </c>
+      <c r="C507" t="str">
+        <v>Coveo CPD Keys and Configur</v>
+      </c>
+      <c r="D507" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E507" t="str">
+        <v>Coveo CPD Keys and Configur</v>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="str">
+        <v>2026-08-17 15:26</v>
+      </c>
+      <c r="B508" t="str">
+        <v>T-27I6K43</v>
+      </c>
+      <c r="C508" t="str">
+        <v>Coveo CPD Keys and Configura</v>
+      </c>
+      <c r="D508" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E508" t="str">
+        <v>Coveo CPD Keys and Configura</v>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B509" t="str">
+        <v>T-27I6K43</v>
+      </c>
+      <c r="C509" t="str">
+        <v>Coveo CPD Keys and Configurat</v>
+      </c>
+      <c r="D509" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E509" t="str">
+        <v>Coveo CPD Keys and Configurat</v>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B510" t="str">
+        <v>T-27I6K43</v>
+      </c>
+      <c r="C510" t="str">
+        <v>Coveo CPD Keys and Configurati</v>
+      </c>
+      <c r="D510" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E510" t="str">
+        <v>Coveo CPD Keys and Configurati</v>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B511" t="str">
+        <v>T-27I6K43</v>
+      </c>
+      <c r="C511" t="str">
+        <v>Coveo CPD Keys and Configuratio</v>
+      </c>
+      <c r="D511" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E511" t="str">
+        <v>Coveo CPD Keys and Configuratio</v>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B512" t="str">
+        <v>T-27I6K43</v>
+      </c>
+      <c r="C512" t="str">
+        <v>Coveo CPD Keys and Configuration</v>
+      </c>
+      <c r="D512" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E512" t="str">
+        <v>Coveo CPD Keys and Configuration</v>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B513" t="str">
+        <v>T-27I6K43</v>
+      </c>
+      <c r="C513" t="str">
+        <v>Coveo CPD Keys and Configuration</v>
+      </c>
+      <c r="D513" t="str">
+        <v>Status changed</v>
+      </c>
+      <c r="E513" t="str">
+        <v>To do → In progress</v>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B514" t="str">
+        <v>T-27I6K43</v>
+      </c>
+      <c r="C514" t="str">
+        <v>Coveo CPD Keys and Configuration</v>
+      </c>
+      <c r="D514" t="str">
+        <v>Due date set</v>
+      </c>
+      <c r="E514" t="str">
+        <v>2026-08-17</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E472"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E514"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 8 notes, 0 done (2026-08-17 15:27)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J9"/>
   <cols>
     <col min="1" max="1" width="11.83203125" customWidth="1"/>
     <col min="2" max="2" width="34.83203125" customWidth="1"/>
@@ -448,22 +448,22 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>T-27I6K43</v>
+        <v>T-28A0V57</v>
       </c>
       <c r="B2" t="str">
-        <v>Coveo CPD Keys and Configuration</v>
+        <v>Coveo - CPD explanation to Mohan</v>
       </c>
       <c r="C2" t="str">
         <v/>
       </c>
       <c r="D2" t="str">
-        <v>In progress</v>
+        <v>To do</v>
       </c>
       <c r="E2">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-08-17</v>
+        <v/>
       </c>
       <c r="G2" t="str">
         <v>2026-08-17</v>
@@ -475,27 +475,27 @@
         <v>2026-08-17 15:27</v>
       </c>
       <c r="J2" t="str">
-        <v>--p1</v>
+        <v>--p2</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>T-24W7H31</v>
+        <v>T-27I6K43</v>
       </c>
       <c r="B3" t="str">
-        <v xml:space="preserve">CPD - Follow Up for TBD to mathieu </v>
+        <v>Coveo CPD Keys and Configuration</v>
       </c>
       <c r="C3" t="str">
         <v/>
       </c>
       <c r="D3" t="str">
-        <v>To do</v>
+        <v>In progress</v>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="F3" t="str">
-        <v/>
+        <v>2026-08-17</v>
       </c>
       <c r="G3" t="str">
         <v>2026-08-17</v>
@@ -504,88 +504,88 @@
         <v/>
       </c>
       <c r="I3" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="J3" t="str">
+        <v>--p1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="B4" t="str">
+        <v xml:space="preserve">CPD - Follow Up for TBD to mathieu </v>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v>To do</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
         <v>2026-08-17 15:25</v>
       </c>
-      <c r="J3" t="str">
+      <c r="J4" t="str">
         <v>--p6</v>
       </c>
     </row>
-    <row r="4" xml:space="preserve">
-      <c r="A4" t="str">
-        <v>T-22JLI81</v>
-      </c>
-      <c r="B4" t="str">
+    <row r="5" xml:space="preserve">
+      <c r="A5" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="B5" t="str">
         <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
       </c>
-      <c r="C4" t="str" xml:space="preserve">
+      <c r="C5" t="str" xml:space="preserve">
         <v xml:space="preserve">For 
 RSP, RGG, RSW, BOCT</v>
       </c>
-      <c r="D4" t="str">
+      <c r="D5" t="str">
         <v>To do</v>
       </c>
-      <c r="E4">
+      <c r="E5">
         <v>0</v>
       </c>
-      <c r="F4" t="str">
+      <c r="F5" t="str">
         <v/>
       </c>
-      <c r="G4" t="str">
+      <c r="G5" t="str">
         <v>2026-08-17</v>
       </c>
-      <c r="H4" t="str">
+      <c r="H5" t="str">
         <v/>
       </c>
-      <c r="I4" t="str">
+      <c r="I5" t="str">
         <v>2026-08-17 15:24</v>
       </c>
-      <c r="J4" t="str">
+      <c r="J5" t="str">
         <v>--p5</v>
       </c>
     </row>
-    <row r="5" xml:space="preserve">
-      <c r="A5" t="str">
+    <row r="6" xml:space="preserve">
+      <c r="A6" t="str">
         <v>T-20UNS57</v>
       </c>
-      <c r="B5" t="str">
+      <c r="B6" t="str">
         <v xml:space="preserve">DF--4191 - New Version Recommendation Model Migration </v>
       </c>
-      <c r="C5" t="str" xml:space="preserve">
+      <c r="C6" t="str" xml:space="preserve">
         <v xml:space="preserve">For 
 RGG and RSW (DE and CH store)</v>
       </c>
-      <c r="D5" t="str">
-        <v>To do</v>
-      </c>
-      <c r="E5">
-        <v>0</v>
-      </c>
-      <c r="F5" t="str">
-        <v/>
-      </c>
-      <c r="G5" t="str">
-        <v>2026-08-17</v>
-      </c>
-      <c r="H5" t="str">
-        <v/>
-      </c>
-      <c r="I5" t="str">
-        <v>2026-08-17 15:22</v>
-      </c>
-      <c r="J5" t="str">
-        <v>--p4</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>T-1ZZXI87</v>
-      </c>
-      <c r="B6" t="str">
-        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
-      </c>
-      <c r="C6" t="str">
-        <v xml:space="preserve">For grant </v>
-      </c>
       <c r="D6" t="str">
         <v>To do</v>
       </c>
@@ -602,21 +602,21 @@
         <v/>
       </c>
       <c r="I6" t="str">
-        <v>2026-08-17 15:21</v>
+        <v>2026-08-17 15:22</v>
       </c>
       <c r="J6" t="str">
-        <v>--p3</v>
+        <v>--p4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>T-1YYRK56</v>
+        <v>T-1ZZXI87</v>
       </c>
       <c r="B7" t="str">
-        <v>Coveo RSP - Recommendation Go-Live for BOC AU store</v>
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
       </c>
       <c r="C7" t="str">
-        <v>for Grant</v>
+        <v xml:space="preserve">For grant </v>
       </c>
       <c r="D7" t="str">
         <v>To do</v>
@@ -634,30 +634,30 @@
         <v/>
       </c>
       <c r="I7" t="str">
-        <v>2026-08-17 15:20</v>
+        <v>2026-08-17 15:21</v>
       </c>
       <c r="J7" t="str">
-        <v>--p2</v>
+        <v>--p3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>T-1X4UW94</v>
+        <v>T-1YYRK56</v>
       </c>
       <c r="B8" t="str">
-        <v>Coveo RSP- QPM for V2 calls</v>
+        <v>Coveo RSP - Recommendation Go-Live for BOC AU store</v>
       </c>
       <c r="C8" t="str">
+        <v>for Grant</v>
+      </c>
+      <c r="D8" t="str">
+        <v>To do</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8" t="str">
         <v/>
-      </c>
-      <c r="D8" t="str">
-        <v>In progress</v>
-      </c>
-      <c r="E8">
-        <v>50</v>
-      </c>
-      <c r="F8" t="str">
-        <v>2026-08-14</v>
       </c>
       <c r="G8" t="str">
         <v>2026-08-17</v>
@@ -666,15 +666,47 @@
         <v/>
       </c>
       <c r="I8" t="str">
+        <v>2026-08-17 15:20</v>
+      </c>
+      <c r="J8" t="str">
+        <v>--p2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Coveo RSP- QPM for V2 calls</v>
+      </c>
+      <c r="C9" t="str">
+        <v/>
+      </c>
+      <c r="D9" t="str">
+        <v>In progress</v>
+      </c>
+      <c r="E9">
+        <v>50</v>
+      </c>
+      <c r="F9" t="str">
+        <v>2026-08-14</v>
+      </c>
+      <c r="G9" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H9" t="str">
+        <v/>
+      </c>
+      <c r="I9" t="str">
         <v>2026-08-17 15:19</v>
       </c>
-      <c r="J8" t="str">
+      <c r="J9" t="str">
         <v>--p1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J9"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -700,7 +732,7 @@
         <v>Total notes</v>
       </c>
       <c r="B2">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3">
@@ -708,7 +740,7 @@
         <v>To do</v>
       </c>
       <c r="B3">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4">
@@ -732,7 +764,7 @@
         <v>Overall progress %</v>
       </c>
       <c r="B6">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7">
@@ -862,7 +894,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E515"/>
+  <dimension ref="A1:E566"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -9626,9 +9658,876 @@
         <v>0% → 70%</v>
       </c>
     </row>
+    <row r="516">
+      <c r="A516" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B516" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C516" t="str">
+        <v>(untitled)</v>
+      </c>
+      <c r="D516" t="str">
+        <v>Created</v>
+      </c>
+      <c r="E516" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B517" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C517" t="str">
+        <v>C</v>
+      </c>
+      <c r="D517" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E517" t="str">
+        <v>C</v>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B518" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C518" t="str">
+        <v>CD</v>
+      </c>
+      <c r="D518" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E518" t="str">
+        <v>CD</v>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B519" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C519" t="str">
+        <v>CDP</v>
+      </c>
+      <c r="D519" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E519" t="str">
+        <v>CDP</v>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B520" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C520" t="str">
+        <v>CD</v>
+      </c>
+      <c r="D520" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E520" t="str">
+        <v>CD</v>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B521" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C521" t="str">
+        <v>C</v>
+      </c>
+      <c r="D521" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E521" t="str">
+        <v>C</v>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B522" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C522" t="str">
+        <v>CP</v>
+      </c>
+      <c r="D522" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E522" t="str">
+        <v>CP</v>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B523" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C523" t="str">
+        <v>CPD</v>
+      </c>
+      <c r="D523" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E523" t="str">
+        <v>CPD</v>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B524" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C524" t="str">
+        <v xml:space="preserve">CPD </v>
+      </c>
+      <c r="D524" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E524" t="str">
+        <v xml:space="preserve">CPD </v>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B525" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C525" t="str">
+        <v>CPD M</v>
+      </c>
+      <c r="D525" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E525" t="str">
+        <v>CPD M</v>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B526" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C526" t="str">
+        <v>CPD Mo</v>
+      </c>
+      <c r="D526" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E526" t="str">
+        <v>CPD Mo</v>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B527" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C527" t="str">
+        <v>CPD M</v>
+      </c>
+      <c r="D527" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E527" t="str">
+        <v>CPD M</v>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B528" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C528" t="str">
+        <v xml:space="preserve">CPD </v>
+      </c>
+      <c r="D528" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E528" t="str">
+        <v xml:space="preserve">CPD </v>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B529" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C529" t="str">
+        <v>CPD</v>
+      </c>
+      <c r="D529" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E529" t="str">
+        <v>CPD</v>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B530" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C530" t="str">
+        <v>CP</v>
+      </c>
+      <c r="D530" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E530" t="str">
+        <v>CP</v>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B531" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C531" t="str">
+        <v>C</v>
+      </c>
+      <c r="D531" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E531" t="str">
+        <v>C</v>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B532" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C532" t="str">
+        <v>(untitled)</v>
+      </c>
+      <c r="D532" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E532" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B533" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C533" t="str">
+        <v>C</v>
+      </c>
+      <c r="D533" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E533" t="str">
+        <v>C</v>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B534" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C534" t="str">
+        <v>Co</v>
+      </c>
+      <c r="D534" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E534" t="str">
+        <v>Co</v>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B535" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C535" t="str">
+        <v>Cov</v>
+      </c>
+      <c r="D535" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E535" t="str">
+        <v>Cov</v>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B536" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C536" t="str">
+        <v>Cove</v>
+      </c>
+      <c r="D536" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E536" t="str">
+        <v>Cove</v>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B537" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C537" t="str">
+        <v>Coveo</v>
+      </c>
+      <c r="D537" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E537" t="str">
+        <v>Coveo</v>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B538" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C538" t="str">
+        <v xml:space="preserve">Coveo </v>
+      </c>
+      <c r="D538" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E538" t="str">
+        <v xml:space="preserve">Coveo </v>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B539" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C539" t="str">
+        <v>Coveo -</v>
+      </c>
+      <c r="D539" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E539" t="str">
+        <v>Coveo -</v>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B540" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C540" t="str">
+        <v xml:space="preserve">Coveo - </v>
+      </c>
+      <c r="D540" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E540" t="str">
+        <v xml:space="preserve">Coveo - </v>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B541" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C541" t="str">
+        <v>Coveo - C</v>
+      </c>
+      <c r="D541" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E541" t="str">
+        <v>Coveo - C</v>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B542" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C542" t="str">
+        <v>Coveo - CP</v>
+      </c>
+      <c r="D542" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E542" t="str">
+        <v>Coveo - CP</v>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B543" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C543" t="str">
+        <v>Coveo - CPD</v>
+      </c>
+      <c r="D543" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E543" t="str">
+        <v>Coveo - CPD</v>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B544" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C544" t="str">
+        <v xml:space="preserve">Coveo - CPD </v>
+      </c>
+      <c r="D544" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E544" t="str">
+        <v xml:space="preserve">Coveo - CPD </v>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B545" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C545" t="str">
+        <v>Coveo - CPD e</v>
+      </c>
+      <c r="D545" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E545" t="str">
+        <v>Coveo - CPD e</v>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B546" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C546" t="str">
+        <v>Coveo - CPD ex</v>
+      </c>
+      <c r="D546" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E546" t="str">
+        <v>Coveo - CPD ex</v>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B547" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C547" t="str">
+        <v>Coveo - CPD exp</v>
+      </c>
+      <c r="D547" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E547" t="str">
+        <v>Coveo - CPD exp</v>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B548" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C548" t="str">
+        <v>Coveo - CPD expl</v>
+      </c>
+      <c r="D548" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E548" t="str">
+        <v>Coveo - CPD expl</v>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B549" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C549" t="str">
+        <v>Coveo - CPD expla</v>
+      </c>
+      <c r="D549" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E549" t="str">
+        <v>Coveo - CPD expla</v>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B550" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C550" t="str">
+        <v>Coveo - CPD explan</v>
+      </c>
+      <c r="D550" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E550" t="str">
+        <v>Coveo - CPD explan</v>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B551" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C551" t="str">
+        <v>Coveo - CPD explana</v>
+      </c>
+      <c r="D551" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E551" t="str">
+        <v>Coveo - CPD explana</v>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B552" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C552" t="str">
+        <v>Coveo - CPD explanat</v>
+      </c>
+      <c r="D552" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E552" t="str">
+        <v>Coveo - CPD explanat</v>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B553" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C553" t="str">
+        <v>Coveo - CPD explanati</v>
+      </c>
+      <c r="D553" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E553" t="str">
+        <v>Coveo - CPD explanati</v>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B554" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C554" t="str">
+        <v>Coveo - CPD explanatio</v>
+      </c>
+      <c r="D554" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E554" t="str">
+        <v>Coveo - CPD explanatio</v>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B555" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C555" t="str">
+        <v>Coveo - CPD explanation</v>
+      </c>
+      <c r="D555" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E555" t="str">
+        <v>Coveo - CPD explanation</v>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B556" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C556" t="str">
+        <v xml:space="preserve">Coveo - CPD explanation </v>
+      </c>
+      <c r="D556" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E556" t="str">
+        <v xml:space="preserve">Coveo - CPD explanation </v>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B557" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C557" t="str">
+        <v>Coveo - CPD explanation t</v>
+      </c>
+      <c r="D557" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E557" t="str">
+        <v>Coveo - CPD explanation t</v>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B558" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C558" t="str">
+        <v>Coveo - CPD explanation to</v>
+      </c>
+      <c r="D558" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E558" t="str">
+        <v>Coveo - CPD explanation to</v>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B559" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C559" t="str">
+        <v xml:space="preserve">Coveo - CPD explanation to </v>
+      </c>
+      <c r="D559" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E559" t="str">
+        <v xml:space="preserve">Coveo - CPD explanation to </v>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B560" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C560" t="str">
+        <v>Coveo - CPD explanation to M</v>
+      </c>
+      <c r="D560" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E560" t="str">
+        <v>Coveo - CPD explanation to M</v>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B561" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C561" t="str">
+        <v>Coveo - CPD explanation to Mo</v>
+      </c>
+      <c r="D561" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E561" t="str">
+        <v>Coveo - CPD explanation to Mo</v>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B562" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C562" t="str">
+        <v>Coveo - CPD explanation to Moh</v>
+      </c>
+      <c r="D562" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E562" t="str">
+        <v>Coveo - CPD explanation to Moh</v>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B563" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C563" t="str">
+        <v>Coveo - CPD explanation to Moha</v>
+      </c>
+      <c r="D563" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E563" t="str">
+        <v>Coveo - CPD explanation to Moha</v>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B564" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C564" t="str">
+        <v>Coveo - CPD explanation to Mohab</v>
+      </c>
+      <c r="D564" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E564" t="str">
+        <v>Coveo - CPD explanation to Mohab</v>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B565" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C565" t="str">
+        <v>Coveo - CPD explanation to Moha</v>
+      </c>
+      <c r="D565" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E565" t="str">
+        <v>Coveo - CPD explanation to Moha</v>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="B566" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C566" t="str">
+        <v>Coveo - CPD explanation to Mohan</v>
+      </c>
+      <c r="D566" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E566" t="str">
+        <v>Coveo - CPD explanation to Mohan</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E515"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E566"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 9 notes, 0 done (2026-08-17 15:28)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J10"/>
   <cols>
     <col min="1" max="1" width="11.83203125" customWidth="1"/>
     <col min="2" max="2" width="34.83203125" customWidth="1"/>
@@ -448,10 +448,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>T-28A0V57</v>
+        <v>T-292O348</v>
       </c>
       <c r="B2" t="str">
-        <v>Coveo - CPD explanation to Mohan</v>
+        <v xml:space="preserve">Sonar Qube </v>
       </c>
       <c r="C2" t="str">
         <v/>
@@ -472,30 +472,30 @@
         <v/>
       </c>
       <c r="I2" t="str">
-        <v>2026-08-17 15:27</v>
+        <v>2026-08-17 15:28</v>
       </c>
       <c r="J2" t="str">
-        <v>--p2</v>
+        <v>--p3</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>T-27I6K43</v>
+        <v>T-28A0V57</v>
       </c>
       <c r="B3" t="str">
-        <v>Coveo CPD Keys and Configuration</v>
+        <v>Coveo - CPD explanation to Mohan</v>
       </c>
       <c r="C3" t="str">
         <v/>
       </c>
       <c r="D3" t="str">
-        <v>In progress</v>
+        <v>To do</v>
       </c>
       <c r="E3">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="F3" t="str">
-        <v>2026-08-17</v>
+        <v/>
       </c>
       <c r="G3" t="str">
         <v>2026-08-17</v>
@@ -507,27 +507,27 @@
         <v>2026-08-17 15:27</v>
       </c>
       <c r="J3" t="str">
-        <v>--p1</v>
+        <v>--p2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>T-24W7H31</v>
+        <v>T-27I6K43</v>
       </c>
       <c r="B4" t="str">
-        <v xml:space="preserve">CPD - Follow Up for TBD to mathieu </v>
+        <v>Coveo CPD Keys and Configuration</v>
       </c>
       <c r="C4" t="str">
         <v/>
       </c>
       <c r="D4" t="str">
-        <v>To do</v>
+        <v>In progress</v>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="F4" t="str">
-        <v/>
+        <v>2026-08-17</v>
       </c>
       <c r="G4" t="str">
         <v>2026-08-17</v>
@@ -536,88 +536,88 @@
         <v/>
       </c>
       <c r="I4" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="J4" t="str">
+        <v>--p1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="B5" t="str">
+        <v xml:space="preserve">CPD - Follow Up for TBD to mathieu </v>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v>To do</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
         <v>2026-08-17 15:25</v>
       </c>
-      <c r="J4" t="str">
+      <c r="J5" t="str">
         <v>--p6</v>
       </c>
     </row>
-    <row r="5" xml:space="preserve">
-      <c r="A5" t="str">
-        <v>T-22JLI81</v>
-      </c>
-      <c r="B5" t="str">
+    <row r="6" xml:space="preserve">
+      <c r="A6" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="B6" t="str">
         <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
       </c>
-      <c r="C5" t="str" xml:space="preserve">
+      <c r="C6" t="str" xml:space="preserve">
         <v xml:space="preserve">For 
 RSP, RGG, RSW, BOCT</v>
       </c>
-      <c r="D5" t="str">
+      <c r="D6" t="str">
         <v>To do</v>
       </c>
-      <c r="E5">
+      <c r="E6">
         <v>0</v>
       </c>
-      <c r="F5" t="str">
+      <c r="F6" t="str">
         <v/>
       </c>
-      <c r="G5" t="str">
+      <c r="G6" t="str">
         <v>2026-08-17</v>
       </c>
-      <c r="H5" t="str">
+      <c r="H6" t="str">
         <v/>
       </c>
-      <c r="I5" t="str">
+      <c r="I6" t="str">
         <v>2026-08-17 15:24</v>
       </c>
-      <c r="J5" t="str">
+      <c r="J6" t="str">
         <v>--p5</v>
       </c>
     </row>
-    <row r="6" xml:space="preserve">
-      <c r="A6" t="str">
+    <row r="7" xml:space="preserve">
+      <c r="A7" t="str">
         <v>T-20UNS57</v>
       </c>
-      <c r="B6" t="str">
+      <c r="B7" t="str">
         <v xml:space="preserve">DF--4191 - New Version Recommendation Model Migration </v>
       </c>
-      <c r="C6" t="str" xml:space="preserve">
+      <c r="C7" t="str" xml:space="preserve">
         <v xml:space="preserve">For 
 RGG and RSW (DE and CH store)</v>
       </c>
-      <c r="D6" t="str">
-        <v>To do</v>
-      </c>
-      <c r="E6">
-        <v>0</v>
-      </c>
-      <c r="F6" t="str">
-        <v/>
-      </c>
-      <c r="G6" t="str">
-        <v>2026-08-17</v>
-      </c>
-      <c r="H6" t="str">
-        <v/>
-      </c>
-      <c r="I6" t="str">
-        <v>2026-08-17 15:22</v>
-      </c>
-      <c r="J6" t="str">
-        <v>--p4</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>T-1ZZXI87</v>
-      </c>
-      <c r="B7" t="str">
-        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
-      </c>
-      <c r="C7" t="str">
-        <v xml:space="preserve">For grant </v>
-      </c>
       <c r="D7" t="str">
         <v>To do</v>
       </c>
@@ -634,21 +634,21 @@
         <v/>
       </c>
       <c r="I7" t="str">
-        <v>2026-08-17 15:21</v>
+        <v>2026-08-17 15:22</v>
       </c>
       <c r="J7" t="str">
-        <v>--p3</v>
+        <v>--p4</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>T-1YYRK56</v>
+        <v>T-1ZZXI87</v>
       </c>
       <c r="B8" t="str">
-        <v>Coveo RSP - Recommendation Go-Live for BOC AU store</v>
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
       </c>
       <c r="C8" t="str">
-        <v>for Grant</v>
+        <v xml:space="preserve">For grant </v>
       </c>
       <c r="D8" t="str">
         <v>To do</v>
@@ -666,30 +666,30 @@
         <v/>
       </c>
       <c r="I8" t="str">
-        <v>2026-08-17 15:20</v>
+        <v>2026-08-17 15:21</v>
       </c>
       <c r="J8" t="str">
-        <v>--p2</v>
+        <v>--p3</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>T-1X4UW94</v>
+        <v>T-1YYRK56</v>
       </c>
       <c r="B9" t="str">
-        <v>Coveo RSP- QPM for V2 calls</v>
+        <v>Coveo RSP - Recommendation Go-Live for BOC AU store</v>
       </c>
       <c r="C9" t="str">
+        <v>for Grant</v>
+      </c>
+      <c r="D9" t="str">
+        <v>To do</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9" t="str">
         <v/>
-      </c>
-      <c r="D9" t="str">
-        <v>In progress</v>
-      </c>
-      <c r="E9">
-        <v>50</v>
-      </c>
-      <c r="F9" t="str">
-        <v>2026-08-14</v>
       </c>
       <c r="G9" t="str">
         <v>2026-08-17</v>
@@ -698,15 +698,47 @@
         <v/>
       </c>
       <c r="I9" t="str">
+        <v>2026-08-17 15:20</v>
+      </c>
+      <c r="J9" t="str">
+        <v>--p2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Coveo RSP- QPM for V2 calls</v>
+      </c>
+      <c r="C10" t="str">
+        <v/>
+      </c>
+      <c r="D10" t="str">
+        <v>In progress</v>
+      </c>
+      <c r="E10">
+        <v>50</v>
+      </c>
+      <c r="F10" t="str">
+        <v>2026-08-14</v>
+      </c>
+      <c r="G10" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H10" t="str">
+        <v/>
+      </c>
+      <c r="I10" t="str">
         <v>2026-08-17 15:19</v>
       </c>
-      <c r="J9" t="str">
+      <c r="J10" t="str">
         <v>--p1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J10"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -732,7 +764,7 @@
         <v>Total notes</v>
       </c>
       <c r="B2">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3">
@@ -740,7 +772,7 @@
         <v>To do</v>
       </c>
       <c r="B3">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4">
@@ -764,7 +796,7 @@
         <v>Overall progress %</v>
       </c>
       <c r="B6">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7">
@@ -788,7 +820,7 @@
         <v>Last saved</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-17 15:27</v>
+        <v>2026-08-17 15:28</v>
       </c>
     </row>
   </sheetData>
@@ -894,7 +926,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E566"/>
+  <dimension ref="A1:E582"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -10525,9 +10557,281 @@
         <v>Coveo - CPD explanation to Mohan</v>
       </c>
     </row>
+    <row r="567">
+      <c r="A567" t="str">
+        <v>2026-08-17 15:28</v>
+      </c>
+      <c r="B567" t="str">
+        <v>T-292O348</v>
+      </c>
+      <c r="C567" t="str">
+        <v>(untitled)</v>
+      </c>
+      <c r="D567" t="str">
+        <v>Created</v>
+      </c>
+      <c r="E567" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="str">
+        <v>2026-08-17 15:28</v>
+      </c>
+      <c r="B568" t="str">
+        <v>T-292O348</v>
+      </c>
+      <c r="C568" t="str">
+        <v>S</v>
+      </c>
+      <c r="D568" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E568" t="str">
+        <v>S</v>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="str">
+        <v>2026-08-17 15:28</v>
+      </c>
+      <c r="B569" t="str">
+        <v>T-292O348</v>
+      </c>
+      <c r="C569" t="str">
+        <v>So</v>
+      </c>
+      <c r="D569" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E569" t="str">
+        <v>So</v>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="str">
+        <v>2026-08-17 15:28</v>
+      </c>
+      <c r="B570" t="str">
+        <v>T-292O348</v>
+      </c>
+      <c r="C570" t="str">
+        <v>Son</v>
+      </c>
+      <c r="D570" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E570" t="str">
+        <v>Son</v>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="str">
+        <v>2026-08-17 15:28</v>
+      </c>
+      <c r="B571" t="str">
+        <v>T-292O348</v>
+      </c>
+      <c r="C571" t="str">
+        <v>Sona</v>
+      </c>
+      <c r="D571" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E571" t="str">
+        <v>Sona</v>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="str">
+        <v>2026-08-17 15:28</v>
+      </c>
+      <c r="B572" t="str">
+        <v>T-292O348</v>
+      </c>
+      <c r="C572" t="str">
+        <v>Sonar</v>
+      </c>
+      <c r="D572" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E572" t="str">
+        <v>Sonar</v>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="str">
+        <v>2026-08-17 15:28</v>
+      </c>
+      <c r="B573" t="str">
+        <v>T-292O348</v>
+      </c>
+      <c r="C573" t="str">
+        <v xml:space="preserve">Sonar </v>
+      </c>
+      <c r="D573" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E573" t="str">
+        <v xml:space="preserve">Sonar </v>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="str">
+        <v>2026-08-17 15:28</v>
+      </c>
+      <c r="B574" t="str">
+        <v>T-292O348</v>
+      </c>
+      <c r="C574" t="str">
+        <v>Sonar Q</v>
+      </c>
+      <c r="D574" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E574" t="str">
+        <v>Sonar Q</v>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="str">
+        <v>2026-08-17 15:28</v>
+      </c>
+      <c r="B575" t="str">
+        <v>T-292O348</v>
+      </c>
+      <c r="C575" t="str">
+        <v>Sonar Qu</v>
+      </c>
+      <c r="D575" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E575" t="str">
+        <v>Sonar Qu</v>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="str">
+        <v>2026-08-17 15:28</v>
+      </c>
+      <c r="B576" t="str">
+        <v>T-292O348</v>
+      </c>
+      <c r="C576" t="str">
+        <v>Sonar Qub</v>
+      </c>
+      <c r="D576" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E576" t="str">
+        <v>Sonar Qub</v>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="str">
+        <v>2026-08-17 15:28</v>
+      </c>
+      <c r="B577" t="str">
+        <v>T-292O348</v>
+      </c>
+      <c r="C577" t="str">
+        <v>Sonar Qube</v>
+      </c>
+      <c r="D577" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E577" t="str">
+        <v>Sonar Qube</v>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="str">
+        <v>2026-08-17 15:28</v>
+      </c>
+      <c r="B578" t="str">
+        <v>T-292O348</v>
+      </c>
+      <c r="C578" t="str">
+        <v xml:space="preserve">Sonar Qube </v>
+      </c>
+      <c r="D578" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E578" t="str">
+        <v xml:space="preserve">Sonar Qube </v>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="str">
+        <v>2026-08-17 15:28</v>
+      </c>
+      <c r="B579" t="str">
+        <v>T-292O348</v>
+      </c>
+      <c r="C579" t="str">
+        <v>Sonar Qube</v>
+      </c>
+      <c r="D579" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E579" t="str">
+        <v>Sonar Qube</v>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="str">
+        <v>2026-08-17 15:28</v>
+      </c>
+      <c r="B580" t="str">
+        <v>T-292O348</v>
+      </c>
+      <c r="C580" t="str">
+        <v>Sonar Qub</v>
+      </c>
+      <c r="D580" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E580" t="str">
+        <v>Sonar Qub</v>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="str">
+        <v>2026-08-17 15:28</v>
+      </c>
+      <c r="B581" t="str">
+        <v>T-292O348</v>
+      </c>
+      <c r="C581" t="str">
+        <v>Sonar Qube</v>
+      </c>
+      <c r="D581" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E581" t="str">
+        <v>Sonar Qube</v>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="str">
+        <v>2026-08-17 15:28</v>
+      </c>
+      <c r="B582" t="str">
+        <v>T-292O348</v>
+      </c>
+      <c r="C582" t="str">
+        <v xml:space="preserve">Sonar Qube </v>
+      </c>
+      <c r="D582" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E582" t="str">
+        <v xml:space="preserve">Sonar Qube </v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E566"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E582"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 9 notes, 0 done (2026-08-17 15:30)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -592,7 +592,7 @@
         <v>0</v>
       </c>
       <c r="F6" t="str">
-        <v/>
+        <v>2026-08-21</v>
       </c>
       <c r="G6" t="str">
         <v>2026-08-17</v>
@@ -601,7 +601,7 @@
         <v/>
       </c>
       <c r="I6" t="str">
-        <v>2026-08-17 15:24</v>
+        <v>2026-08-17 15:30</v>
       </c>
       <c r="J6" t="str">
         <v>--p5</v>
@@ -820,7 +820,7 @@
         <v>Last saved</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-17 15:28</v>
+        <v>2026-08-17 15:30</v>
       </c>
     </row>
   </sheetData>
@@ -926,7 +926,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E593"/>
+  <dimension ref="A1:E594"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -11016,9 +11016,26 @@
         <v>Sonarqube Resolve</v>
       </c>
     </row>
+    <row r="594">
+      <c r="A594" t="str">
+        <v>2026-08-17 15:30</v>
+      </c>
+      <c r="B594" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C594" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D594" t="str">
+        <v>Due date set</v>
+      </c>
+      <c r="E594" t="str">
+        <v>2026-08-21</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E593"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E594"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 9 notes, 0 done (2026-08-17 15:31)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -579,7 +579,7 @@
         <v>T-22JLI81</v>
       </c>
       <c r="B6" t="str">
-        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation mail and Confirm Coveo for Production </v>
       </c>
       <c r="C6" t="str" xml:space="preserve">
         <v xml:space="preserve">For 
@@ -601,7 +601,7 @@
         <v/>
       </c>
       <c r="I6" t="str">
-        <v>2026-08-17 15:30</v>
+        <v>2026-08-17 15:31</v>
       </c>
       <c r="J6" t="str">
         <v>--p5</v>
@@ -820,7 +820,7 @@
         <v>Last saved</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-17 15:30</v>
+        <v>2026-08-17 15:31</v>
       </c>
     </row>
   </sheetData>
@@ -926,7 +926,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E594"/>
+  <dimension ref="A1:E599"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -11033,9 +11033,94 @@
         <v>2026-08-21</v>
       </c>
     </row>
+    <row r="595">
+      <c r="A595" t="str">
+        <v>2026-08-17 15:30</v>
+      </c>
+      <c r="B595" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C595" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation  and Confirm Coveo for Production </v>
+      </c>
+      <c r="D595" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E595" t="str">
+        <v>Coveo Global Configuration API Deprecation Confirmation  and</v>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="str">
+        <v>2026-08-17 15:31</v>
+      </c>
+      <c r="B596" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C596" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation m and Confirm Coveo for Production </v>
+      </c>
+      <c r="D596" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E596" t="str">
+        <v>Coveo Global Configuration API Deprecation Confirmation m an</v>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="str">
+        <v>2026-08-17 15:31</v>
+      </c>
+      <c r="B597" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C597" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation ma and Confirm Coveo for Production </v>
+      </c>
+      <c r="D597" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E597" t="str">
+        <v>Coveo Global Configuration API Deprecation Confirmation ma a</v>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="str">
+        <v>2026-08-17 15:31</v>
+      </c>
+      <c r="B598" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C598" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation mai and Confirm Coveo for Production </v>
+      </c>
+      <c r="D598" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E598" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation mai </v>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="str">
+        <v>2026-08-17 15:31</v>
+      </c>
+      <c r="B599" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C599" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation mail and Confirm Coveo for Production </v>
+      </c>
+      <c r="D599" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E599" t="str">
+        <v>Coveo Global Configuration API Deprecation Confirmation mail</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E594"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E599"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 10 notes, 0 done (2026-08-17 15:31)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J11"/>
   <cols>
     <col min="1" max="1" width="11.83203125" customWidth="1"/>
     <col min="2" max="2" width="34.83203125" customWidth="1"/>
@@ -448,10 +448,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>T-292O348</v>
+        <v>T-2D24I52</v>
       </c>
       <c r="B2" t="str">
-        <v>Sonarqube Resolve</v>
+        <v xml:space="preserve">TASK -- Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
       </c>
       <c r="C2" t="str">
         <v/>
@@ -472,18 +472,18 @@
         <v/>
       </c>
       <c r="I2" t="str">
-        <v>2026-08-17 15:28</v>
+        <v>2026-08-17 15:31</v>
       </c>
       <c r="J2" t="str">
-        <v>--p3</v>
+        <v>--p4</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>T-28A0V57</v>
+        <v>T-292O348</v>
       </c>
       <c r="B3" t="str">
-        <v>Coveo - CPD explanation to Mohan</v>
+        <v>Sonarqube Resolve</v>
       </c>
       <c r="C3" t="str">
         <v/>
@@ -504,30 +504,30 @@
         <v/>
       </c>
       <c r="I3" t="str">
-        <v>2026-08-17 15:27</v>
+        <v>2026-08-17 15:28</v>
       </c>
       <c r="J3" t="str">
-        <v>--p2</v>
+        <v>--p3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>T-27I6K43</v>
+        <v>T-28A0V57</v>
       </c>
       <c r="B4" t="str">
-        <v>Coveo CPD Keys and Configuration</v>
+        <v>Coveo - CPD explanation to Mohan</v>
       </c>
       <c r="C4" t="str">
         <v/>
       </c>
       <c r="D4" t="str">
-        <v>In progress</v>
+        <v>To do</v>
       </c>
       <c r="E4">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="F4" t="str">
-        <v>2026-08-17</v>
+        <v/>
       </c>
       <c r="G4" t="str">
         <v>2026-08-17</v>
@@ -539,27 +539,27 @@
         <v>2026-08-17 15:27</v>
       </c>
       <c r="J4" t="str">
-        <v>--p1</v>
+        <v>--p2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>T-24W7H31</v>
+        <v>T-27I6K43</v>
       </c>
       <c r="B5" t="str">
-        <v xml:space="preserve">CPD - Follow Up for TBD to mathieu </v>
+        <v>Coveo CPD Keys and Configuration</v>
       </c>
       <c r="C5" t="str">
         <v/>
       </c>
       <c r="D5" t="str">
-        <v>To do</v>
+        <v>In progress</v>
       </c>
       <c r="E5">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="F5" t="str">
-        <v/>
+        <v>2026-08-17</v>
       </c>
       <c r="G5" t="str">
         <v>2026-08-17</v>
@@ -568,88 +568,88 @@
         <v/>
       </c>
       <c r="I5" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="J5" t="str">
+        <v>--p1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="B6" t="str">
+        <v xml:space="preserve">CPD - Follow Up for TBD to mathieu </v>
+      </c>
+      <c r="C6" t="str">
+        <v/>
+      </c>
+      <c r="D6" t="str">
+        <v>To do</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+      <c r="I6" t="str">
         <v>2026-08-17 15:25</v>
       </c>
-      <c r="J5" t="str">
+      <c r="J6" t="str">
         <v>--p6</v>
       </c>
     </row>
-    <row r="6" xml:space="preserve">
-      <c r="A6" t="str">
-        <v>T-22JLI81</v>
-      </c>
-      <c r="B6" t="str">
+    <row r="7" xml:space="preserve">
+      <c r="A7" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="B7" t="str">
         <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation mail and Confirm Coveo for Production </v>
       </c>
-      <c r="C6" t="str" xml:space="preserve">
+      <c r="C7" t="str" xml:space="preserve">
         <v xml:space="preserve">For 
 RSP, RGG, RSW, BOCT</v>
       </c>
-      <c r="D6" t="str">
+      <c r="D7" t="str">
         <v>To do</v>
       </c>
-      <c r="E6">
+      <c r="E7">
         <v>0</v>
       </c>
-      <c r="F6" t="str">
+      <c r="F7" t="str">
         <v>2026-08-21</v>
       </c>
-      <c r="G6" t="str">
+      <c r="G7" t="str">
         <v>2026-08-17</v>
       </c>
-      <c r="H6" t="str">
+      <c r="H7" t="str">
         <v/>
       </c>
-      <c r="I6" t="str">
+      <c r="I7" t="str">
         <v>2026-08-17 15:31</v>
       </c>
-      <c r="J6" t="str">
+      <c r="J7" t="str">
         <v>--p5</v>
       </c>
     </row>
-    <row r="7" xml:space="preserve">
-      <c r="A7" t="str">
+    <row r="8" xml:space="preserve">
+      <c r="A8" t="str">
         <v>T-20UNS57</v>
       </c>
-      <c r="B7" t="str">
+      <c r="B8" t="str">
         <v xml:space="preserve">DF--4191 - New Version Recommendation Model Migration </v>
       </c>
-      <c r="C7" t="str" xml:space="preserve">
+      <c r="C8" t="str" xml:space="preserve">
         <v xml:space="preserve">For 
 RGG and RSW (DE and CH store)</v>
       </c>
-      <c r="D7" t="str">
-        <v>To do</v>
-      </c>
-      <c r="E7">
-        <v>0</v>
-      </c>
-      <c r="F7" t="str">
-        <v/>
-      </c>
-      <c r="G7" t="str">
-        <v>2026-08-17</v>
-      </c>
-      <c r="H7" t="str">
-        <v/>
-      </c>
-      <c r="I7" t="str">
-        <v>2026-08-17 15:22</v>
-      </c>
-      <c r="J7" t="str">
-        <v>--p4</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>T-1ZZXI87</v>
-      </c>
-      <c r="B8" t="str">
-        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
-      </c>
-      <c r="C8" t="str">
-        <v xml:space="preserve">For grant </v>
-      </c>
       <c r="D8" t="str">
         <v>To do</v>
       </c>
@@ -666,21 +666,21 @@
         <v/>
       </c>
       <c r="I8" t="str">
-        <v>2026-08-17 15:21</v>
+        <v>2026-08-17 15:22</v>
       </c>
       <c r="J8" t="str">
-        <v>--p3</v>
+        <v>--p4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>T-1YYRK56</v>
+        <v>T-1ZZXI87</v>
       </c>
       <c r="B9" t="str">
-        <v>Coveo RSP - Recommendation Go-Live for BOC AU store</v>
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
       </c>
       <c r="C9" t="str">
-        <v>for Grant</v>
+        <v xml:space="preserve">For grant </v>
       </c>
       <c r="D9" t="str">
         <v>To do</v>
@@ -698,30 +698,30 @@
         <v/>
       </c>
       <c r="I9" t="str">
-        <v>2026-08-17 15:20</v>
+        <v>2026-08-17 15:21</v>
       </c>
       <c r="J9" t="str">
-        <v>--p2</v>
+        <v>--p3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>T-1X4UW94</v>
+        <v>T-1YYRK56</v>
       </c>
       <c r="B10" t="str">
-        <v>Coveo RSP- QPM for V2 calls</v>
+        <v>Coveo RSP - Recommendation Go-Live for BOC AU store</v>
       </c>
       <c r="C10" t="str">
+        <v>for Grant</v>
+      </c>
+      <c r="D10" t="str">
+        <v>To do</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10" t="str">
         <v/>
-      </c>
-      <c r="D10" t="str">
-        <v>In progress</v>
-      </c>
-      <c r="E10">
-        <v>50</v>
-      </c>
-      <c r="F10" t="str">
-        <v>2026-08-14</v>
       </c>
       <c r="G10" t="str">
         <v>2026-08-17</v>
@@ -730,15 +730,47 @@
         <v/>
       </c>
       <c r="I10" t="str">
+        <v>2026-08-17 15:20</v>
+      </c>
+      <c r="J10" t="str">
+        <v>--p2</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Coveo RSP- QPM for V2 calls</v>
+      </c>
+      <c r="C11" t="str">
+        <v/>
+      </c>
+      <c r="D11" t="str">
+        <v>In progress</v>
+      </c>
+      <c r="E11">
+        <v>50</v>
+      </c>
+      <c r="F11" t="str">
+        <v>2026-08-14</v>
+      </c>
+      <c r="G11" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H11" t="str">
+        <v/>
+      </c>
+      <c r="I11" t="str">
         <v>2026-08-17 15:19</v>
       </c>
-      <c r="J10" t="str">
+      <c r="J11" t="str">
         <v>--p1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J11"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -764,7 +796,7 @@
         <v>Total notes</v>
       </c>
       <c r="B2">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3">
@@ -772,7 +804,7 @@
         <v>To do</v>
       </c>
       <c r="B3">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4">
@@ -796,7 +828,7 @@
         <v>Overall progress %</v>
       </c>
       <c r="B6">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7">
@@ -926,7 +958,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E599"/>
+  <dimension ref="A1:E609"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -11118,9 +11150,179 @@
         <v>Coveo Global Configuration API Deprecation Confirmation mail</v>
       </c>
     </row>
+    <row r="600">
+      <c r="A600" t="str">
+        <v>2026-08-17 15:31</v>
+      </c>
+      <c r="B600" t="str">
+        <v>T-2D24I52</v>
+      </c>
+      <c r="C600" t="str">
+        <v>(untitled)</v>
+      </c>
+      <c r="D600" t="str">
+        <v>Created</v>
+      </c>
+      <c r="E600" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="str">
+        <v>2026-08-17 15:31</v>
+      </c>
+      <c r="B601" t="str">
+        <v>T-2D24I52</v>
+      </c>
+      <c r="C601" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D601" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E601" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation and </v>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="str">
+        <v>2026-08-17 15:31</v>
+      </c>
+      <c r="B602" t="str">
+        <v>T-2D24I52</v>
+      </c>
+      <c r="C602" t="str">
+        <v xml:space="preserve">TCoveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D602" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E602" t="str">
+        <v>TCoveo Global Configuration API Deprecation Confirmation and</v>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="str">
+        <v>2026-08-17 15:31</v>
+      </c>
+      <c r="B603" t="str">
+        <v>T-2D24I52</v>
+      </c>
+      <c r="C603" t="str">
+        <v xml:space="preserve">TACoveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D603" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E603" t="str">
+        <v>TACoveo Global Configuration API Deprecation Confirmation an</v>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="str">
+        <v>2026-08-17 15:31</v>
+      </c>
+      <c r="B604" t="str">
+        <v>T-2D24I52</v>
+      </c>
+      <c r="C604" t="str">
+        <v xml:space="preserve">TASCoveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D604" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E604" t="str">
+        <v>TASCoveo Global Configuration API Deprecation Confirmation a</v>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="str">
+        <v>2026-08-17 15:31</v>
+      </c>
+      <c r="B605" t="str">
+        <v>T-2D24I52</v>
+      </c>
+      <c r="C605" t="str">
+        <v xml:space="preserve">TASKCoveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D605" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E605" t="str">
+        <v xml:space="preserve">TASKCoveo Global Configuration API Deprecation Confirmation </v>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="str">
+        <v>2026-08-17 15:31</v>
+      </c>
+      <c r="B606" t="str">
+        <v>T-2D24I52</v>
+      </c>
+      <c r="C606" t="str">
+        <v xml:space="preserve">TASK-Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D606" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E606" t="str">
+        <v>TASK-Coveo Global Configuration API Deprecation Confirmation</v>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="str">
+        <v>2026-08-17 15:31</v>
+      </c>
+      <c r="B607" t="str">
+        <v>T-2D24I52</v>
+      </c>
+      <c r="C607" t="str">
+        <v xml:space="preserve">TASK--Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D607" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E607" t="str">
+        <v>TASK--Coveo Global Configuration API Deprecation Confirmatio</v>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="str">
+        <v>2026-08-17 15:31</v>
+      </c>
+      <c r="B608" t="str">
+        <v>T-2D24I52</v>
+      </c>
+      <c r="C608" t="str">
+        <v xml:space="preserve">TASK-- Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D608" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E608" t="str">
+        <v>TASK-- Coveo Global Configuration API Deprecation Confirmati</v>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="str">
+        <v>2026-08-17 15:31</v>
+      </c>
+      <c r="B609" t="str">
+        <v>T-2D24I52</v>
+      </c>
+      <c r="C609" t="str">
+        <v xml:space="preserve">TASK -- Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D609" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E609" t="str">
+        <v>TASK -- Coveo Global Configuration API Deprecation Confirmat</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E599"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E609"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 9 notes, 0 done (2026-08-17 15:44)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -586,7 +586,7 @@
 RSP, RGG, RSW, BOCT</v>
       </c>
       <c r="D6" t="str">
-        <v>To do</v>
+        <v>In progress</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -601,7 +601,7 @@
         <v/>
       </c>
       <c r="I6" t="str">
-        <v>2026-08-17 15:31</v>
+        <v>2026-08-17 15:44</v>
       </c>
       <c r="J6" t="str">
         <v>--p5</v>
@@ -772,7 +772,7 @@
         <v>To do</v>
       </c>
       <c r="B3">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4">
@@ -780,7 +780,7 @@
         <v>In progress</v>
       </c>
       <c r="B4">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -820,7 +820,7 @@
         <v>Last saved</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-17 15:31</v>
+        <v>2026-08-17 15:44</v>
       </c>
     </row>
   </sheetData>
@@ -926,7 +926,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E616"/>
+  <dimension ref="A1:E617"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -11407,9 +11407,26 @@
         <v>SonarQube Resolve</v>
       </c>
     </row>
+    <row r="617">
+      <c r="A617" t="str">
+        <v>2026-08-17 15:44</v>
+      </c>
+      <c r="B617" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C617" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation mail and Confirm Coveo for Production </v>
+      </c>
+      <c r="D617" t="str">
+        <v>Status changed</v>
+      </c>
+      <c r="E617" t="str">
+        <v>To do → In progress</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E616"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E617"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 10 notes, 0 done (2026-08-17 15:50)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J11"/>
   <cols>
     <col min="1" max="1" width="11.83203125" customWidth="1"/>
     <col min="2" max="2" width="34.83203125" customWidth="1"/>
@@ -448,10 +448,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>T-292O348</v>
+        <v>T-31URD46</v>
       </c>
       <c r="B2" t="str">
-        <v>SonarQube Resolve</v>
+        <v>Coveo RSW(</v>
       </c>
       <c r="C2" t="str">
         <v/>
@@ -472,18 +472,18 @@
         <v/>
       </c>
       <c r="I2" t="str">
-        <v>2026-08-17 15:31</v>
+        <v>2026-08-17 15:50</v>
       </c>
       <c r="J2" t="str">
-        <v>--p3</v>
+        <v>--p4</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>T-28A0V57</v>
+        <v>T-292O348</v>
       </c>
       <c r="B3" t="str">
-        <v>Coveo - CPD explanation to Mohan</v>
+        <v>SonarQube Resolve</v>
       </c>
       <c r="C3" t="str">
         <v/>
@@ -504,30 +504,30 @@
         <v/>
       </c>
       <c r="I3" t="str">
-        <v>2026-08-17 15:27</v>
+        <v>2026-08-17 15:31</v>
       </c>
       <c r="J3" t="str">
-        <v>--p2</v>
+        <v>--p3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>T-27I6K43</v>
+        <v>T-28A0V57</v>
       </c>
       <c r="B4" t="str">
-        <v>Coveo CPD Keys and Configuration</v>
+        <v>Coveo - CPD explanation to Mohan</v>
       </c>
       <c r="C4" t="str">
         <v/>
       </c>
       <c r="D4" t="str">
-        <v>In progress</v>
+        <v>To do</v>
       </c>
       <c r="E4">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="F4" t="str">
-        <v>2026-08-17</v>
+        <v/>
       </c>
       <c r="G4" t="str">
         <v>2026-08-17</v>
@@ -539,27 +539,27 @@
         <v>2026-08-17 15:27</v>
       </c>
       <c r="J4" t="str">
-        <v>--p1</v>
+        <v>--p2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>T-24W7H31</v>
+        <v>T-27I6K43</v>
       </c>
       <c r="B5" t="str">
-        <v xml:space="preserve">CPD - Follow Up for TBD to mathieu </v>
+        <v>Coveo CPD Keys and Configuration</v>
       </c>
       <c r="C5" t="str">
         <v/>
       </c>
       <c r="D5" t="str">
-        <v>To do</v>
+        <v>In progress</v>
       </c>
       <c r="E5">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="F5" t="str">
-        <v/>
+        <v>2026-08-17</v>
       </c>
       <c r="G5" t="str">
         <v>2026-08-17</v>
@@ -568,88 +568,88 @@
         <v/>
       </c>
       <c r="I5" t="str">
+        <v>2026-08-17 15:27</v>
+      </c>
+      <c r="J5" t="str">
+        <v>--p1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="B6" t="str">
+        <v xml:space="preserve">CPD - Follow Up for TBD to mathieu </v>
+      </c>
+      <c r="C6" t="str">
+        <v/>
+      </c>
+      <c r="D6" t="str">
+        <v>To do</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+      <c r="I6" t="str">
         <v>2026-08-17 15:25</v>
       </c>
-      <c r="J5" t="str">
+      <c r="J6" t="str">
         <v>--p6</v>
       </c>
     </row>
-    <row r="6" xml:space="preserve">
-      <c r="A6" t="str">
-        <v>T-22JLI81</v>
-      </c>
-      <c r="B6" t="str">
+    <row r="7" xml:space="preserve">
+      <c r="A7" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="B7" t="str">
         <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation mail and Confirm Coveo for Production </v>
       </c>
-      <c r="C6" t="str" xml:space="preserve">
+      <c r="C7" t="str" xml:space="preserve">
         <v xml:space="preserve">For 
 RSP, RGG, RSW, BOCT</v>
       </c>
-      <c r="D6" t="str">
+      <c r="D7" t="str">
         <v>In progress</v>
       </c>
-      <c r="E6">
+      <c r="E7">
         <v>0</v>
       </c>
-      <c r="F6" t="str">
+      <c r="F7" t="str">
         <v>2026-08-21</v>
       </c>
-      <c r="G6" t="str">
+      <c r="G7" t="str">
         <v>2026-08-17</v>
       </c>
-      <c r="H6" t="str">
+      <c r="H7" t="str">
         <v/>
       </c>
-      <c r="I6" t="str">
+      <c r="I7" t="str">
         <v>2026-08-17 15:44</v>
       </c>
-      <c r="J6" t="str">
+      <c r="J7" t="str">
         <v>--p5</v>
       </c>
     </row>
-    <row r="7" xml:space="preserve">
-      <c r="A7" t="str">
+    <row r="8" xml:space="preserve">
+      <c r="A8" t="str">
         <v>T-20UNS57</v>
       </c>
-      <c r="B7" t="str">
+      <c r="B8" t="str">
         <v xml:space="preserve">DF--4191 - New Version Recommendation Model Migration </v>
       </c>
-      <c r="C7" t="str" xml:space="preserve">
+      <c r="C8" t="str" xml:space="preserve">
         <v xml:space="preserve">For 
 RGG and RSW (DE and CH store)</v>
       </c>
-      <c r="D7" t="str">
-        <v>To do</v>
-      </c>
-      <c r="E7">
-        <v>0</v>
-      </c>
-      <c r="F7" t="str">
-        <v/>
-      </c>
-      <c r="G7" t="str">
-        <v>2026-08-17</v>
-      </c>
-      <c r="H7" t="str">
-        <v/>
-      </c>
-      <c r="I7" t="str">
-        <v>2026-08-17 15:22</v>
-      </c>
-      <c r="J7" t="str">
-        <v>--p4</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>T-1ZZXI87</v>
-      </c>
-      <c r="B8" t="str">
-        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
-      </c>
-      <c r="C8" t="str">
-        <v xml:space="preserve">For grant </v>
-      </c>
       <c r="D8" t="str">
         <v>To do</v>
       </c>
@@ -666,21 +666,21 @@
         <v/>
       </c>
       <c r="I8" t="str">
-        <v>2026-08-17 15:21</v>
+        <v>2026-08-17 15:22</v>
       </c>
       <c r="J8" t="str">
-        <v>--p3</v>
+        <v>--p4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>T-1YYRK56</v>
+        <v>T-1ZZXI87</v>
       </c>
       <c r="B9" t="str">
-        <v>Coveo RSP - Recommendation Go-Live for BOC AU store</v>
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
       </c>
       <c r="C9" t="str">
-        <v>for Grant</v>
+        <v xml:space="preserve">For grant </v>
       </c>
       <c r="D9" t="str">
         <v>To do</v>
@@ -698,30 +698,30 @@
         <v/>
       </c>
       <c r="I9" t="str">
-        <v>2026-08-17 15:20</v>
+        <v>2026-08-17 15:21</v>
       </c>
       <c r="J9" t="str">
-        <v>--p2</v>
+        <v>--p3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>T-1X4UW94</v>
+        <v>T-1YYRK56</v>
       </c>
       <c r="B10" t="str">
-        <v>Coveo RSP- QPM for V2 calls</v>
+        <v>Coveo RSP - Recommendation Go-Live for BOC AU store</v>
       </c>
       <c r="C10" t="str">
+        <v>for Grant</v>
+      </c>
+      <c r="D10" t="str">
+        <v>To do</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10" t="str">
         <v/>
-      </c>
-      <c r="D10" t="str">
-        <v>In progress</v>
-      </c>
-      <c r="E10">
-        <v>50</v>
-      </c>
-      <c r="F10" t="str">
-        <v>2026-08-14</v>
       </c>
       <c r="G10" t="str">
         <v>2026-08-17</v>
@@ -730,15 +730,47 @@
         <v/>
       </c>
       <c r="I10" t="str">
+        <v>2026-08-17 15:20</v>
+      </c>
+      <c r="J10" t="str">
+        <v>--p2</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Coveo RSP- QPM for V2 calls</v>
+      </c>
+      <c r="C11" t="str">
+        <v/>
+      </c>
+      <c r="D11" t="str">
+        <v>In progress</v>
+      </c>
+      <c r="E11">
+        <v>50</v>
+      </c>
+      <c r="F11" t="str">
+        <v>2026-08-14</v>
+      </c>
+      <c r="G11" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H11" t="str">
+        <v/>
+      </c>
+      <c r="I11" t="str">
         <v>2026-08-17 15:19</v>
       </c>
-      <c r="J10" t="str">
+      <c r="J11" t="str">
         <v>--p1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J11"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -764,7 +796,7 @@
         <v>Total notes</v>
       </c>
       <c r="B2">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3">
@@ -772,7 +804,7 @@
         <v>To do</v>
       </c>
       <c r="B3">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4">
@@ -796,7 +828,7 @@
         <v>Overall progress %</v>
       </c>
       <c r="B6">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7">
@@ -820,7 +852,7 @@
         <v>Last saved</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-17 15:44</v>
+        <v>2026-08-17 15:50</v>
       </c>
     </row>
   </sheetData>
@@ -926,7 +958,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E617"/>
+  <dimension ref="A1:E648"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -11424,9 +11456,536 @@
         <v>To do → In progress</v>
       </c>
     </row>
+    <row r="618">
+      <c r="A618" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B618" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C618" t="str">
+        <v>(untitled)</v>
+      </c>
+      <c r="D618" t="str">
+        <v>Created</v>
+      </c>
+      <c r="E618" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B619" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C619" t="str">
+        <v>C</v>
+      </c>
+      <c r="D619" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E619" t="str">
+        <v>C</v>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B620" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C620" t="str">
+        <v>Co</v>
+      </c>
+      <c r="D620" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E620" t="str">
+        <v>Co</v>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B621" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C621" t="str">
+        <v>Cov</v>
+      </c>
+      <c r="D621" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E621" t="str">
+        <v>Cov</v>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B622" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C622" t="str">
+        <v>Cove</v>
+      </c>
+      <c r="D622" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E622" t="str">
+        <v>Cove</v>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B623" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C623" t="str">
+        <v>Cov</v>
+      </c>
+      <c r="D623" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E623" t="str">
+        <v>Cov</v>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B624" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C624" t="str">
+        <v>Covc</v>
+      </c>
+      <c r="D624" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E624" t="str">
+        <v>Covc</v>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B625" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C625" t="str">
+        <v>Covce</v>
+      </c>
+      <c r="D625" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E625" t="str">
+        <v>Covce</v>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B626" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C626" t="str">
+        <v>Covc</v>
+      </c>
+      <c r="D626" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E626" t="str">
+        <v>Covc</v>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B627" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C627" t="str">
+        <v>Cov</v>
+      </c>
+      <c r="D627" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E627" t="str">
+        <v>Cov</v>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B628" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C628" t="str">
+        <v>Cove</v>
+      </c>
+      <c r="D628" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E628" t="str">
+        <v>Cove</v>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B629" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C629" t="str">
+        <v xml:space="preserve">Cove </v>
+      </c>
+      <c r="D629" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E629" t="str">
+        <v xml:space="preserve">Cove </v>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B630" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C630" t="str">
+        <v>Cove</v>
+      </c>
+      <c r="D630" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E630" t="str">
+        <v>Cove</v>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B631" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C631" t="str">
+        <v>Cov</v>
+      </c>
+      <c r="D631" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E631" t="str">
+        <v>Cov</v>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B632" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C632" t="str">
+        <v>Co</v>
+      </c>
+      <c r="D632" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E632" t="str">
+        <v>Co</v>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B633" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C633" t="str">
+        <v>CoV</v>
+      </c>
+      <c r="D633" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E633" t="str">
+        <v>CoV</v>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B634" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C634" t="str">
+        <v>CoVe</v>
+      </c>
+      <c r="D634" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E634" t="str">
+        <v>CoVe</v>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B635" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C635" t="str">
+        <v>CoV</v>
+      </c>
+      <c r="D635" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E635" t="str">
+        <v>CoV</v>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B636" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C636" t="str">
+        <v>Co</v>
+      </c>
+      <c r="D636" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E636" t="str">
+        <v>Co</v>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B637" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C637" t="str">
+        <v>Cov</v>
+      </c>
+      <c r="D637" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E637" t="str">
+        <v>Cov</v>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B638" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C638" t="str">
+        <v>Cove</v>
+      </c>
+      <c r="D638" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E638" t="str">
+        <v>Cove</v>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B639" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C639" t="str">
+        <v>Coveo</v>
+      </c>
+      <c r="D639" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E639" t="str">
+        <v>Coveo</v>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B640" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C640" t="str">
+        <v xml:space="preserve">Coveo </v>
+      </c>
+      <c r="D640" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E640" t="str">
+        <v xml:space="preserve">Coveo </v>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B641" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C641" t="str">
+        <v>Coveo R</v>
+      </c>
+      <c r="D641" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E641" t="str">
+        <v>Coveo R</v>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B642" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C642" t="str">
+        <v>Coveo RE</v>
+      </c>
+      <c r="D642" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E642" t="str">
+        <v>Coveo RE</v>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B643" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C643" t="str">
+        <v>Coveo R</v>
+      </c>
+      <c r="D643" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E643" t="str">
+        <v>Coveo R</v>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B644" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C644" t="str">
+        <v xml:space="preserve">Coveo </v>
+      </c>
+      <c r="D644" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E644" t="str">
+        <v xml:space="preserve">Coveo </v>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B645" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C645" t="str">
+        <v>Coveo R</v>
+      </c>
+      <c r="D645" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E645" t="str">
+        <v>Coveo R</v>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B646" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C646" t="str">
+        <v>Coveo RS</v>
+      </c>
+      <c r="D646" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E646" t="str">
+        <v>Coveo RS</v>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B647" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C647" t="str">
+        <v>Coveo RSW</v>
+      </c>
+      <c r="D647" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E647" t="str">
+        <v>Coveo RSW</v>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B648" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C648" t="str">
+        <v>Coveo RSW(</v>
+      </c>
+      <c r="D648" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E648" t="str">
+        <v>Coveo RSW(</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E617"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E648"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 10 notes, 0 done (2026-08-17 15:51)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -451,7 +451,7 @@
         <v>T-31URD46</v>
       </c>
       <c r="B2" t="str">
-        <v>Coveo RSW(</v>
+        <v>Coveo RSW(Spain) recommendation Setup</v>
       </c>
       <c r="C2" t="str">
         <v/>
@@ -852,7 +852,7 @@
         <v>Last saved</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-17 15:50</v>
+        <v>2026-08-17 15:51</v>
       </c>
     </row>
   </sheetData>
@@ -958,7 +958,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E648"/>
+  <dimension ref="A1:E679"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -11983,9 +11983,536 @@
         <v>Coveo RSW(</v>
       </c>
     </row>
+    <row r="649">
+      <c r="A649" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B649" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C649" t="str">
+        <v>Coveo RSW(E</v>
+      </c>
+      <c r="D649" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E649" t="str">
+        <v>Coveo RSW(E</v>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B650" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C650" t="str">
+        <v>Coveo RSW(ES</v>
+      </c>
+      <c r="D650" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E650" t="str">
+        <v>Coveo RSW(ES</v>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B651" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C651" t="str">
+        <v>Coveo RSW(E</v>
+      </c>
+      <c r="D651" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E651" t="str">
+        <v>Coveo RSW(E</v>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B652" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C652" t="str">
+        <v>Coveo RSW(</v>
+      </c>
+      <c r="D652" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E652" t="str">
+        <v>Coveo RSW(</v>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B653" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C653" t="str">
+        <v>Coveo RSW(S</v>
+      </c>
+      <c r="D653" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E653" t="str">
+        <v>Coveo RSW(S</v>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B654" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C654" t="str">
+        <v>Coveo RSW(Sp</v>
+      </c>
+      <c r="D654" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E654" t="str">
+        <v>Coveo RSW(Sp</v>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B655" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C655" t="str">
+        <v>Coveo RSW(Spa</v>
+      </c>
+      <c r="D655" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E655" t="str">
+        <v>Coveo RSW(Spa</v>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B656" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C656" t="str">
+        <v>Coveo RSW(Spai</v>
+      </c>
+      <c r="D656" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E656" t="str">
+        <v>Coveo RSW(Spai</v>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B657" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C657" t="str">
+        <v>Coveo RSW(Spain</v>
+      </c>
+      <c r="D657" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E657" t="str">
+        <v>Coveo RSW(Spain</v>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B658" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C658" t="str">
+        <v>Coveo RSW(Spain)</v>
+      </c>
+      <c r="D658" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E658" t="str">
+        <v>Coveo RSW(Spain)</v>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B659" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C659" t="str">
+        <v xml:space="preserve">Coveo RSW(Spain) </v>
+      </c>
+      <c r="D659" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E659" t="str">
+        <v xml:space="preserve">Coveo RSW(Spain) </v>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B660" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C660" t="str">
+        <v>Coveo RSW(Spain) r</v>
+      </c>
+      <c r="D660" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E660" t="str">
+        <v>Coveo RSW(Spain) r</v>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B661" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C661" t="str">
+        <v>Coveo RSW(Spain) re</v>
+      </c>
+      <c r="D661" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E661" t="str">
+        <v>Coveo RSW(Spain) re</v>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B662" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C662" t="str">
+        <v>Coveo RSW(Spain) rec</v>
+      </c>
+      <c r="D662" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E662" t="str">
+        <v>Coveo RSW(Spain) rec</v>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B663" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C663" t="str">
+        <v>Coveo RSW(Spain) reco</v>
+      </c>
+      <c r="D663" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E663" t="str">
+        <v>Coveo RSW(Spain) reco</v>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B664" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C664" t="str">
+        <v>Coveo RSW(Spain) recom</v>
+      </c>
+      <c r="D664" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E664" t="str">
+        <v>Coveo RSW(Spain) recom</v>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B665" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C665" t="str">
+        <v>Coveo RSW(Spain) recomm</v>
+      </c>
+      <c r="D665" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E665" t="str">
+        <v>Coveo RSW(Spain) recomm</v>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B666" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C666" t="str">
+        <v>Coveo RSW(Spain) recomme</v>
+      </c>
+      <c r="D666" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E666" t="str">
+        <v>Coveo RSW(Spain) recomme</v>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B667" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C667" t="str">
+        <v>Coveo RSW(Spain) recommen</v>
+      </c>
+      <c r="D667" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E667" t="str">
+        <v>Coveo RSW(Spain) recommen</v>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B668" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C668" t="str">
+        <v>Coveo RSW(Spain) recommend</v>
+      </c>
+      <c r="D668" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E668" t="str">
+        <v>Coveo RSW(Spain) recommend</v>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B669" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C669" t="str">
+        <v>Coveo RSW(Spain) recommenda</v>
+      </c>
+      <c r="D669" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E669" t="str">
+        <v>Coveo RSW(Spain) recommenda</v>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B670" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C670" t="str">
+        <v>Coveo RSW(Spain) recommendat</v>
+      </c>
+      <c r="D670" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E670" t="str">
+        <v>Coveo RSW(Spain) recommendat</v>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B671" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C671" t="str">
+        <v>Coveo RSW(Spain) recommendati</v>
+      </c>
+      <c r="D671" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E671" t="str">
+        <v>Coveo RSW(Spain) recommendati</v>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B672" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C672" t="str">
+        <v>Coveo RSW(Spain) recommendatio</v>
+      </c>
+      <c r="D672" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E672" t="str">
+        <v>Coveo RSW(Spain) recommendatio</v>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B673" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C673" t="str">
+        <v>Coveo RSW(Spain) recommendation</v>
+      </c>
+      <c r="D673" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E673" t="str">
+        <v>Coveo RSW(Spain) recommendation</v>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B674" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C674" t="str">
+        <v xml:space="preserve">Coveo RSW(Spain) recommendation </v>
+      </c>
+      <c r="D674" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E674" t="str">
+        <v xml:space="preserve">Coveo RSW(Spain) recommendation </v>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B675" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C675" t="str">
+        <v>Coveo RSW(Spain) recommendation S</v>
+      </c>
+      <c r="D675" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E675" t="str">
+        <v>Coveo RSW(Spain) recommendation S</v>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B676" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C676" t="str">
+        <v>Coveo RSW(Spain) recommendation Se</v>
+      </c>
+      <c r="D676" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E676" t="str">
+        <v>Coveo RSW(Spain) recommendation Se</v>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B677" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C677" t="str">
+        <v>Coveo RSW(Spain) recommendation Set</v>
+      </c>
+      <c r="D677" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E677" t="str">
+        <v>Coveo RSW(Spain) recommendation Set</v>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B678" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C678" t="str">
+        <v>Coveo RSW(Spain) recommendation Setu</v>
+      </c>
+      <c r="D678" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E678" t="str">
+        <v>Coveo RSW(Spain) recommendation Setu</v>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="str">
+        <v>2026-08-17 15:50</v>
+      </c>
+      <c r="B679" t="str">
+        <v>T-31URD46</v>
+      </c>
+      <c r="C679" t="str">
+        <v>Coveo RSW(Spain) recommendation Setup</v>
+      </c>
+      <c r="D679" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E679" t="str">
+        <v>Coveo RSW(Spain) recommendation Setup</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E648"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E679"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 10 notes, 1 done (2026-08-17 16:51)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -586,22 +586,22 @@
         <v/>
       </c>
       <c r="D6" t="str">
-        <v>To do</v>
+        <v>Done</v>
       </c>
       <c r="E6">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="F6" t="str">
-        <v/>
+        <v>2026-08-17</v>
       </c>
       <c r="G6" t="str">
         <v>2026-08-17</v>
       </c>
       <c r="H6" t="str">
-        <v/>
+        <v>2026-08-17</v>
       </c>
       <c r="I6" t="str">
-        <v>2026-08-17 15:25</v>
+        <v>2026-08-17 16:51</v>
       </c>
       <c r="J6" t="str">
         <v>--p6</v>
@@ -805,7 +805,7 @@
         <v>To do</v>
       </c>
       <c r="B3">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4">
@@ -821,7 +821,7 @@
         <v>Done</v>
       </c>
       <c r="B5">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -829,7 +829,7 @@
         <v>Overall progress %</v>
       </c>
       <c r="B6">
-        <v>12</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7">
@@ -853,7 +853,7 @@
         <v>Last saved</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-17 15:51</v>
+        <v>2026-08-17 16:51</v>
       </c>
     </row>
   </sheetData>
@@ -959,7 +959,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E707"/>
+  <dimension ref="A1:E709"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -12987,9 +12987,43 @@
         <v>for  Julia before 14.7 UAT</v>
       </c>
     </row>
+    <row r="708">
+      <c r="A708" t="str">
+        <v>2026-08-17 16:51</v>
+      </c>
+      <c r="B708" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C708" t="str">
+        <v xml:space="preserve">CPD - Follow Up for TBD to mathieu </v>
+      </c>
+      <c r="D708" t="str">
+        <v>Due date set</v>
+      </c>
+      <c r="E708" t="str">
+        <v>2026-08-17</v>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" t="str">
+        <v>2026-08-17 16:51</v>
+      </c>
+      <c r="B709" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="C709" t="str">
+        <v xml:space="preserve">CPD - Follow Up for TBD to mathieu </v>
+      </c>
+      <c r="D709" t="str">
+        <v>Status changed</v>
+      </c>
+      <c r="E709" t="str">
+        <v>To do → Done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E707"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E709"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 10 notes, 1 done (2026-08-17 16:52)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -658,7 +658,7 @@
         <v>0</v>
       </c>
       <c r="F8" t="str">
-        <v/>
+        <v>2026-08-21</v>
       </c>
       <c r="G8" t="str">
         <v>2026-08-17</v>
@@ -667,7 +667,7 @@
         <v/>
       </c>
       <c r="I8" t="str">
-        <v>2026-08-17 15:22</v>
+        <v>2026-08-17 16:52</v>
       </c>
       <c r="J8" t="str">
         <v>--p4</v>
@@ -853,7 +853,7 @@
         <v>Last saved</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-17 16:51</v>
+        <v>2026-08-17 16:52</v>
       </c>
     </row>
   </sheetData>
@@ -959,7 +959,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E709"/>
+  <dimension ref="A1:E710"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -13021,9 +13021,26 @@
         <v>To do → Done</v>
       </c>
     </row>
+    <row r="710">
+      <c r="A710" t="str">
+        <v>2026-08-17 16:52</v>
+      </c>
+      <c r="B710" t="str">
+        <v>T-20UNS57</v>
+      </c>
+      <c r="C710" t="str">
+        <v xml:space="preserve">DF--4191 - New Version Recommendation Model Migration </v>
+      </c>
+      <c r="D710" t="str">
+        <v>Due date set</v>
+      </c>
+      <c r="E710" t="str">
+        <v>2026-08-21</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E709"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E710"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 10 notes, 1 done (2026-08-17 17:05)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -845,7 +845,7 @@
         <v>In bin</v>
       </c>
       <c r="B8">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -853,7 +853,7 @@
         <v>Last saved</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-17 16:52</v>
+        <v>2026-08-17 17:05</v>
       </c>
     </row>
   </sheetData>
@@ -917,37 +917,37 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>T-2D24I52</v>
+        <v/>
       </c>
       <c r="B2" t="str">
-        <v xml:space="preserve">TASK -- Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+        <v/>
       </c>
       <c r="C2" t="str">
         <v/>
       </c>
       <c r="D2" t="str">
-        <v>To do</v>
-      </c>
-      <c r="E2">
-        <v>0</v>
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v/>
       </c>
       <c r="F2" t="str">
         <v/>
       </c>
       <c r="G2" t="str">
-        <v>2026-08-17</v>
+        <v/>
       </c>
       <c r="H2" t="str">
         <v/>
       </c>
       <c r="I2" t="str">
-        <v>2026-08-17 15:31</v>
+        <v/>
       </c>
       <c r="J2" t="str">
-        <v>--p4</v>
+        <v/>
       </c>
       <c r="K2" t="str">
-        <v>2026-08-17 15:31</v>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -959,7 +959,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E711"/>
+  <dimension ref="A1:E712"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -13055,9 +13055,26 @@
         <v>0% → 50%</v>
       </c>
     </row>
+    <row r="712">
+      <c r="A712" t="str">
+        <v>2026-08-17 17:05</v>
+      </c>
+      <c r="B712" t="str">
+        <v>T-2D24I52</v>
+      </c>
+      <c r="C712" t="str">
+        <v xml:space="preserve">TASK -- Coveo Global Configuration API Deprecation Confirmation and Confirm Coveo for Production </v>
+      </c>
+      <c r="D712" t="str">
+        <v>Deleted permanently</v>
+      </c>
+      <c r="E712" t="str">
+        <v>binned 2026-08-17 15:31</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E711"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E712"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 10 notes, 1 done (2026-08-17 17:36)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -554,7 +554,7 @@
         <v/>
       </c>
       <c r="D5" t="str">
-        <v>In progress</v>
+        <v>To do</v>
       </c>
       <c r="E5">
         <v>70</v>
@@ -569,7 +569,7 @@
         <v/>
       </c>
       <c r="I5" t="str">
-        <v>2026-08-17 15:27</v>
+        <v>2026-08-17 17:36</v>
       </c>
       <c r="J5" t="str">
         <v>--p1</v>
@@ -805,7 +805,7 @@
         <v>To do</v>
       </c>
       <c r="B3">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4">
@@ -813,7 +813,7 @@
         <v>In progress</v>
       </c>
       <c r="B4">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -853,7 +853,7 @@
         <v>Last saved</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-17 17:05</v>
+        <v>2026-08-17 17:36</v>
       </c>
     </row>
   </sheetData>
@@ -959,7 +959,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E712"/>
+  <dimension ref="A1:E713"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -13072,9 +13072,26 @@
         <v>binned 2026-08-17 15:31</v>
       </c>
     </row>
+    <row r="713">
+      <c r="A713" t="str">
+        <v>2026-08-17 17:36</v>
+      </c>
+      <c r="B713" t="str">
+        <v>T-27I6K43</v>
+      </c>
+      <c r="C713" t="str">
+        <v>Coveo CPD Keys and Configuration</v>
+      </c>
+      <c r="D713" t="str">
+        <v>Status changed</v>
+      </c>
+      <c r="E713" t="str">
+        <v>In progress → To do</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E712"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E713"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 10 notes, 2 done (2026-08-17 17:37)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -554,10 +554,10 @@
         <v/>
       </c>
       <c r="D5" t="str">
-        <v>To do</v>
+        <v>Done</v>
       </c>
       <c r="E5">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="F5" t="str">
         <v>2026-08-17</v>
@@ -566,7 +566,7 @@
         <v>2026-08-17</v>
       </c>
       <c r="H5" t="str">
-        <v/>
+        <v>2026-08-17</v>
       </c>
       <c r="I5" t="str">
         <v>2026-08-17 17:36</v>
@@ -805,7 +805,7 @@
         <v>To do</v>
       </c>
       <c r="B3">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4">
@@ -821,7 +821,7 @@
         <v>Done</v>
       </c>
       <c r="B5">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -829,7 +829,7 @@
         <v>Overall progress %</v>
       </c>
       <c r="B6">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7">
@@ -853,7 +853,7 @@
         <v>Last saved</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-17 17:36</v>
+        <v>2026-08-17 17:37</v>
       </c>
     </row>
   </sheetData>
@@ -959,7 +959,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E713"/>
+  <dimension ref="A1:E714"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -13089,9 +13089,26 @@
         <v>In progress → To do</v>
       </c>
     </row>
+    <row r="714">
+      <c r="A714" t="str">
+        <v>2026-08-17 17:36</v>
+      </c>
+      <c r="B714" t="str">
+        <v>T-27I6K43</v>
+      </c>
+      <c r="C714" t="str">
+        <v>Coveo CPD Keys and Configuration</v>
+      </c>
+      <c r="D714" t="str">
+        <v>Status changed</v>
+      </c>
+      <c r="E714" t="str">
+        <v>To do → Done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E713"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E714"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 11 notes, 2 done (2026-08-17 18:11)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J12"/>
   <cols>
     <col min="1" max="1" width="11.83203125" customWidth="1"/>
     <col min="2" max="2" width="34.83203125" customWidth="1"/>
@@ -446,49 +446,49 @@
         <v>Colour</v>
       </c>
     </row>
-    <row r="2" xml:space="preserve">
+    <row r="2">
       <c r="A2" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Request AO team to add CPD Live endpoint to liquibase</v>
+      </c>
+      <c r="C2" t="str">
+        <v/>
+      </c>
+      <c r="D2" t="str">
+        <v>In progress</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
+      <c r="I2" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="J2" t="str">
+        <v>--p5</v>
+      </c>
+    </row>
+    <row r="3" xml:space="preserve">
+      <c r="A3" t="str">
         <v>T-31URD46</v>
       </c>
-      <c r="B2" t="str">
+      <c r="B3" t="str">
         <v>Coveo RSW(Spain) recommendation Setup</v>
       </c>
-      <c r="C2" t="str" xml:space="preserve">
+      <c r="C3" t="str" xml:space="preserve">
         <v xml:space="preserve">for 
 Julia before 14.7 UAT</v>
       </c>
-      <c r="D2" t="str">
-        <v>To do</v>
-      </c>
-      <c r="E2">
-        <v>0</v>
-      </c>
-      <c r="F2" t="str">
-        <v/>
-      </c>
-      <c r="G2" t="str">
-        <v>2026-08-17</v>
-      </c>
-      <c r="H2" t="str">
-        <v/>
-      </c>
-      <c r="I2" t="str">
-        <v>2026-08-17 15:51</v>
-      </c>
-      <c r="J2" t="str">
-        <v>--p4</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>T-292O348</v>
-      </c>
-      <c r="B3" t="str">
-        <v>SonarQube Resolve</v>
-      </c>
-      <c r="C3" t="str">
-        <v/>
-      </c>
       <c r="D3" t="str">
         <v>To do</v>
       </c>
@@ -505,18 +505,18 @@
         <v/>
       </c>
       <c r="I3" t="str">
-        <v>2026-08-17 15:31</v>
+        <v>2026-08-17 15:51</v>
       </c>
       <c r="J3" t="str">
-        <v>--p3</v>
+        <v>--p4</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>T-28A0V57</v>
+        <v>T-292O348</v>
       </c>
       <c r="B4" t="str">
-        <v>Coveo - CPD explanation to Mohan</v>
+        <v>SonarQube Resolve</v>
       </c>
       <c r="C4" t="str">
         <v/>
@@ -537,50 +537,50 @@
         <v/>
       </c>
       <c r="I4" t="str">
-        <v>2026-08-17 15:27</v>
+        <v>2026-08-17 15:31</v>
       </c>
       <c r="J4" t="str">
-        <v>--p2</v>
+        <v>--p3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>T-27I6K43</v>
+        <v>T-28A0V57</v>
       </c>
       <c r="B5" t="str">
-        <v>Coveo CPD Keys and Configuration</v>
+        <v>Coveo - CPD explanation to Mohan</v>
       </c>
       <c r="C5" t="str">
         <v/>
       </c>
       <c r="D5" t="str">
-        <v>Done</v>
+        <v>To do</v>
       </c>
       <c r="E5">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="F5" t="str">
-        <v>2026-08-17</v>
+        <v/>
       </c>
       <c r="G5" t="str">
         <v>2026-08-17</v>
       </c>
       <c r="H5" t="str">
-        <v>2026-08-17</v>
+        <v/>
       </c>
       <c r="I5" t="str">
-        <v>2026-08-17 17:36</v>
+        <v>2026-08-17 15:27</v>
       </c>
       <c r="J5" t="str">
-        <v>--p1</v>
+        <v>--p2</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>T-24W7H31</v>
+        <v>T-27I6K43</v>
       </c>
       <c r="B6" t="str">
-        <v xml:space="preserve">CPD - Follow Up for TBD to mathieu </v>
+        <v>Coveo CPD Keys and Configuration</v>
       </c>
       <c r="C6" t="str">
         <v/>
@@ -601,88 +601,88 @@
         <v>2026-08-17</v>
       </c>
       <c r="I6" t="str">
+        <v>2026-08-17 17:36</v>
+      </c>
+      <c r="J6" t="str">
+        <v>--p1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="B7" t="str">
+        <v xml:space="preserve">CPD - Follow Up for TBD to mathieu </v>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+      <c r="D7" t="str">
+        <v>Done</v>
+      </c>
+      <c r="E7">
+        <v>100</v>
+      </c>
+      <c r="F7" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="G7" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H7" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="I7" t="str">
         <v>2026-08-17 16:51</v>
       </c>
-      <c r="J6" t="str">
+      <c r="J7" t="str">
         <v>--p6</v>
       </c>
     </row>
-    <row r="7" xml:space="preserve">
-      <c r="A7" t="str">
-        <v>T-22JLI81</v>
-      </c>
-      <c r="B7" t="str">
+    <row r="8" xml:space="preserve">
+      <c r="A8" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="B8" t="str">
         <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation mail and Confirm Coveo for Production </v>
       </c>
-      <c r="C7" t="str" xml:space="preserve">
+      <c r="C8" t="str" xml:space="preserve">
         <v xml:space="preserve">For 
 RSP, RGG, RSW, BOCT</v>
       </c>
-      <c r="D7" t="str">
+      <c r="D8" t="str">
         <v>In progress</v>
       </c>
-      <c r="E7">
+      <c r="E8">
         <v>50</v>
       </c>
-      <c r="F7" t="str">
+      <c r="F8" t="str">
         <v>2026-08-21</v>
       </c>
-      <c r="G7" t="str">
+      <c r="G8" t="str">
         <v>2026-08-17</v>
       </c>
-      <c r="H7" t="str">
+      <c r="H8" t="str">
         <v/>
       </c>
-      <c r="I7" t="str">
+      <c r="I8" t="str">
         <v>2026-08-17 16:52</v>
       </c>
-      <c r="J7" t="str">
+      <c r="J8" t="str">
         <v>--p5</v>
       </c>
     </row>
-    <row r="8" xml:space="preserve">
-      <c r="A8" t="str">
+    <row r="9" xml:space="preserve">
+      <c r="A9" t="str">
         <v>T-20UNS57</v>
       </c>
-      <c r="B8" t="str">
+      <c r="B9" t="str">
         <v xml:space="preserve">DF--4191 - New Version Recommendation Model Migration </v>
       </c>
-      <c r="C8" t="str" xml:space="preserve">
+      <c r="C9" t="str" xml:space="preserve">
         <v xml:space="preserve">For 
 RGG and RSW (DE and CH store)</v>
       </c>
-      <c r="D8" t="str">
-        <v>To do</v>
-      </c>
-      <c r="E8">
-        <v>0</v>
-      </c>
-      <c r="F8" t="str">
-        <v>2026-08-21</v>
-      </c>
-      <c r="G8" t="str">
-        <v>2026-08-17</v>
-      </c>
-      <c r="H8" t="str">
-        <v/>
-      </c>
-      <c r="I8" t="str">
-        <v>2026-08-17 16:52</v>
-      </c>
-      <c r="J8" t="str">
-        <v>--p4</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>T-1ZZXI87</v>
-      </c>
-      <c r="B9" t="str">
-        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
-      </c>
-      <c r="C9" t="str">
-        <v xml:space="preserve">For grant </v>
-      </c>
       <c r="D9" t="str">
         <v>To do</v>
       </c>
@@ -690,7 +690,7 @@
         <v>0</v>
       </c>
       <c r="F9" t="str">
-        <v/>
+        <v>2026-08-21</v>
       </c>
       <c r="G9" t="str">
         <v>2026-08-17</v>
@@ -699,21 +699,21 @@
         <v/>
       </c>
       <c r="I9" t="str">
-        <v>2026-08-17 15:21</v>
+        <v>2026-08-17 16:52</v>
       </c>
       <c r="J9" t="str">
-        <v>--p3</v>
+        <v>--p4</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>T-1YYRK56</v>
+        <v>T-1ZZXI87</v>
       </c>
       <c r="B10" t="str">
-        <v>Coveo RSP - Recommendation Go-Live for BOC AU store</v>
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
       </c>
       <c r="C10" t="str">
-        <v>for Grant</v>
+        <v xml:space="preserve">For grant </v>
       </c>
       <c r="D10" t="str">
         <v>To do</v>
@@ -731,21 +731,21 @@
         <v/>
       </c>
       <c r="I10" t="str">
-        <v>2026-08-17 15:20</v>
+        <v>2026-08-17 15:21</v>
       </c>
       <c r="J10" t="str">
-        <v>--p2</v>
+        <v>--p3</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>T-1X4UW94</v>
+        <v>T-1YYRK56</v>
       </c>
       <c r="B11" t="str">
-        <v>Coveo RSP- QPM for V2 calls</v>
+        <v>Coveo RSP - Recommendation Go-Live for BOC AU store</v>
       </c>
       <c r="C11" t="str">
-        <v/>
+        <v>for Grant</v>
       </c>
       <c r="D11" t="str">
         <v>To do</v>
@@ -754,7 +754,7 @@
         <v>0</v>
       </c>
       <c r="F11" t="str">
-        <v>2026-08-14</v>
+        <v/>
       </c>
       <c r="G11" t="str">
         <v>2026-08-17</v>
@@ -763,15 +763,47 @@
         <v/>
       </c>
       <c r="I11" t="str">
+        <v>2026-08-17 15:20</v>
+      </c>
+      <c r="J11" t="str">
+        <v>--p2</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Coveo RSP- QPM for V2 calls</v>
+      </c>
+      <c r="C12" t="str">
+        <v/>
+      </c>
+      <c r="D12" t="str">
+        <v>To do</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12" t="str">
+        <v>2026-08-14</v>
+      </c>
+      <c r="G12" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H12" t="str">
+        <v/>
+      </c>
+      <c r="I12" t="str">
         <v>2026-08-17 17:37</v>
       </c>
-      <c r="J11" t="str">
+      <c r="J12" t="str">
         <v>--p1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J12"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -797,7 +829,7 @@
         <v>Total notes</v>
       </c>
       <c r="B2">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3">
@@ -813,7 +845,7 @@
         <v>In progress</v>
       </c>
       <c r="B4">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -829,7 +861,7 @@
         <v>Overall progress %</v>
       </c>
       <c r="B6">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7">
@@ -853,7 +885,7 @@
         <v>Last saved</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-17 17:37</v>
+        <v>2026-08-17 18:11</v>
       </c>
     </row>
   </sheetData>
@@ -959,7 +991,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E716"/>
+  <dimension ref="A1:E777"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -13140,9 +13172,1046 @@
         <v>50% → 0%</v>
       </c>
     </row>
+    <row r="717">
+      <c r="A717" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B717" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C717" t="str">
+        <v>(untitled)</v>
+      </c>
+      <c r="D717" t="str">
+        <v>Created</v>
+      </c>
+      <c r="E717" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B718" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C718" t="str">
+        <v>R</v>
+      </c>
+      <c r="D718" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E718" t="str">
+        <v>R</v>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B719" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C719" t="str">
+        <v>Re</v>
+      </c>
+      <c r="D719" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E719" t="str">
+        <v>Re</v>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B720" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C720" t="str">
+        <v>Req</v>
+      </c>
+      <c r="D720" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E720" t="str">
+        <v>Req</v>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B721" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C721" t="str">
+        <v>Requ</v>
+      </c>
+      <c r="D721" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E721" t="str">
+        <v>Requ</v>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B722" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C722" t="str">
+        <v>Reque</v>
+      </c>
+      <c r="D722" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E722" t="str">
+        <v>Reque</v>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B723" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C723" t="str">
+        <v>Reques</v>
+      </c>
+      <c r="D723" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E723" t="str">
+        <v>Reques</v>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B724" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C724" t="str">
+        <v>Request</v>
+      </c>
+      <c r="D724" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E724" t="str">
+        <v>Request</v>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B725" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C725" t="str">
+        <v xml:space="preserve">Request </v>
+      </c>
+      <c r="D725" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E725" t="str">
+        <v xml:space="preserve">Request </v>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B726" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C726" t="str">
+        <v>Request A</v>
+      </c>
+      <c r="D726" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E726" t="str">
+        <v>Request A</v>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B727" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C727" t="str">
+        <v>Request AO</v>
+      </c>
+      <c r="D727" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E727" t="str">
+        <v>Request AO</v>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B728" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C728" t="str">
+        <v xml:space="preserve">Request AO </v>
+      </c>
+      <c r="D728" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E728" t="str">
+        <v xml:space="preserve">Request AO </v>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B729" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C729" t="str">
+        <v>Request AO t</v>
+      </c>
+      <c r="D729" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E729" t="str">
+        <v>Request AO t</v>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B730" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C730" t="str">
+        <v>Request AO te</v>
+      </c>
+      <c r="D730" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E730" t="str">
+        <v>Request AO te</v>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B731" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C731" t="str">
+        <v>Request AO tea</v>
+      </c>
+      <c r="D731" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E731" t="str">
+        <v>Request AO tea</v>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B732" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C732" t="str">
+        <v>Request AO team</v>
+      </c>
+      <c r="D732" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E732" t="str">
+        <v>Request AO team</v>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B733" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C733" t="str">
+        <v xml:space="preserve">Request AO team </v>
+      </c>
+      <c r="D733" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E733" t="str">
+        <v xml:space="preserve">Request AO team </v>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B734" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C734" t="str">
+        <v>Request AO team t</v>
+      </c>
+      <c r="D734" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E734" t="str">
+        <v>Request AO team t</v>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B735" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C735" t="str">
+        <v>Request AO team to</v>
+      </c>
+      <c r="D735" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E735" t="str">
+        <v>Request AO team to</v>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B736" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C736" t="str">
+        <v xml:space="preserve">Request AO team to </v>
+      </c>
+      <c r="D736" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E736" t="str">
+        <v xml:space="preserve">Request AO team to </v>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B737" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C737" t="str">
+        <v>Request AO team to a</v>
+      </c>
+      <c r="D737" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E737" t="str">
+        <v>Request AO team to a</v>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B738" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C738" t="str">
+        <v>Request AO team to ad</v>
+      </c>
+      <c r="D738" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E738" t="str">
+        <v>Request AO team to ad</v>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B739" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C739" t="str">
+        <v>Request AO team to add</v>
+      </c>
+      <c r="D739" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E739" t="str">
+        <v>Request AO team to add</v>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B740" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C740" t="str">
+        <v xml:space="preserve">Request AO team to add </v>
+      </c>
+      <c r="D740" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E740" t="str">
+        <v xml:space="preserve">Request AO team to add </v>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B741" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C741" t="str">
+        <v>Request AO team to add C</v>
+      </c>
+      <c r="D741" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E741" t="str">
+        <v>Request AO team to add C</v>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B742" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C742" t="str">
+        <v>Request AO team to add CP</v>
+      </c>
+      <c r="D742" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E742" t="str">
+        <v>Request AO team to add CP</v>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B743" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C743" t="str">
+        <v>Request AO team to add CPD</v>
+      </c>
+      <c r="D743" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E743" t="str">
+        <v>Request AO team to add CPD</v>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B744" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C744" t="str">
+        <v xml:space="preserve">Request AO team to add CPD </v>
+      </c>
+      <c r="D744" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E744" t="str">
+        <v xml:space="preserve">Request AO team to add CPD </v>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B745" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C745" t="str">
+        <v>Request AO team to add CPD L</v>
+      </c>
+      <c r="D745" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E745" t="str">
+        <v>Request AO team to add CPD L</v>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B746" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C746" t="str">
+        <v>Request AO team to add CPD Li</v>
+      </c>
+      <c r="D746" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E746" t="str">
+        <v>Request AO team to add CPD Li</v>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B747" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C747" t="str">
+        <v>Request AO team to add CPD Liv</v>
+      </c>
+      <c r="D747" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E747" t="str">
+        <v>Request AO team to add CPD Liv</v>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B748" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C748" t="str">
+        <v>Request AO team to add CPD Live</v>
+      </c>
+      <c r="D748" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E748" t="str">
+        <v>Request AO team to add CPD Live</v>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B749" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C749" t="str">
+        <v xml:space="preserve">Request AO team to add CPD Live </v>
+      </c>
+      <c r="D749" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E749" t="str">
+        <v xml:space="preserve">Request AO team to add CPD Live </v>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B750" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C750" t="str">
+        <v>Request AO team to add CPD Live o</v>
+      </c>
+      <c r="D750" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E750" t="str">
+        <v>Request AO team to add CPD Live o</v>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B751" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C751" t="str">
+        <v>Request AO team to add CPD Live on</v>
+      </c>
+      <c r="D751" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E751" t="str">
+        <v>Request AO team to add CPD Live on</v>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B752" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C752" t="str">
+        <v>Request AO team to add CPD Live ond</v>
+      </c>
+      <c r="D752" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E752" t="str">
+        <v>Request AO team to add CPD Live ond</v>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B753" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C753" t="str">
+        <v>Request AO team to add CPD Live on</v>
+      </c>
+      <c r="D753" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E753" t="str">
+        <v>Request AO team to add CPD Live on</v>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B754" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C754" t="str">
+        <v>Request AO team to add CPD Live o</v>
+      </c>
+      <c r="D754" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E754" t="str">
+        <v>Request AO team to add CPD Live o</v>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B755" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C755" t="str">
+        <v xml:space="preserve">Request AO team to add CPD Live </v>
+      </c>
+      <c r="D755" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E755" t="str">
+        <v xml:space="preserve">Request AO team to add CPD Live </v>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B756" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C756" t="str">
+        <v>Request AO team to add CPD Live e</v>
+      </c>
+      <c r="D756" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E756" t="str">
+        <v>Request AO team to add CPD Live e</v>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B757" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C757" t="str">
+        <v>Request AO team to add CPD Live en</v>
+      </c>
+      <c r="D757" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E757" t="str">
+        <v>Request AO team to add CPD Live en</v>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B758" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C758" t="str">
+        <v>Request AO team to add CPD Live end</v>
+      </c>
+      <c r="D758" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E758" t="str">
+        <v>Request AO team to add CPD Live end</v>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B759" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C759" t="str">
+        <v>Request AO team to add CPD Live endp</v>
+      </c>
+      <c r="D759" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E759" t="str">
+        <v>Request AO team to add CPD Live endp</v>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B760" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C760" t="str">
+        <v>Request AO team to add CPD Live endpo</v>
+      </c>
+      <c r="D760" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E760" t="str">
+        <v>Request AO team to add CPD Live endpo</v>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B761" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C761" t="str">
+        <v>Request AO team to add CPD Live endpoi</v>
+      </c>
+      <c r="D761" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E761" t="str">
+        <v>Request AO team to add CPD Live endpoi</v>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B762" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C762" t="str">
+        <v>Request AO team to add CPD Live endpoin</v>
+      </c>
+      <c r="D762" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E762" t="str">
+        <v>Request AO team to add CPD Live endpoin</v>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B763" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C763" t="str">
+        <v>Request AO team to add CPD Live endpoint</v>
+      </c>
+      <c r="D763" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E763" t="str">
+        <v>Request AO team to add CPD Live endpoint</v>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B764" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C764" t="str">
+        <v xml:space="preserve">Request AO team to add CPD Live endpoint </v>
+      </c>
+      <c r="D764" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E764" t="str">
+        <v xml:space="preserve">Request AO team to add CPD Live endpoint </v>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B765" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C765" t="str">
+        <v>Request AO team to add CPD Live endpoint t</v>
+      </c>
+      <c r="D765" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E765" t="str">
+        <v>Request AO team to add CPD Live endpoint t</v>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B766" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C766" t="str">
+        <v>Request AO team to add CPD Live endpoint to</v>
+      </c>
+      <c r="D766" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E766" t="str">
+        <v>Request AO team to add CPD Live endpoint to</v>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B767" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C767" t="str">
+        <v xml:space="preserve">Request AO team to add CPD Live endpoint to </v>
+      </c>
+      <c r="D767" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E767" t="str">
+        <v xml:space="preserve">Request AO team to add CPD Live endpoint to </v>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B768" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C768" t="str">
+        <v>Request AO team to add CPD Live endpoint to l</v>
+      </c>
+      <c r="D768" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E768" t="str">
+        <v>Request AO team to add CPD Live endpoint to l</v>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B769" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C769" t="str">
+        <v>Request AO team to add CPD Live endpoint to li</v>
+      </c>
+      <c r="D769" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E769" t="str">
+        <v>Request AO team to add CPD Live endpoint to li</v>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B770" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C770" t="str">
+        <v>Request AO team to add CPD Live endpoint to liq</v>
+      </c>
+      <c r="D770" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E770" t="str">
+        <v>Request AO team to add CPD Live endpoint to liq</v>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B771" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C771" t="str">
+        <v>Request AO team to add CPD Live endpoint to liqu</v>
+      </c>
+      <c r="D771" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E771" t="str">
+        <v>Request AO team to add CPD Live endpoint to liqu</v>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B772" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C772" t="str">
+        <v>Request AO team to add CPD Live endpoint to liqui</v>
+      </c>
+      <c r="D772" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E772" t="str">
+        <v>Request AO team to add CPD Live endpoint to liqui</v>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B773" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C773" t="str">
+        <v>Request AO team to add CPD Live endpoint to liquib</v>
+      </c>
+      <c r="D773" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E773" t="str">
+        <v>Request AO team to add CPD Live endpoint to liquib</v>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B774" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C774" t="str">
+        <v>Request AO team to add CPD Live endpoint to liquiba</v>
+      </c>
+      <c r="D774" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E774" t="str">
+        <v>Request AO team to add CPD Live endpoint to liquiba</v>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B775" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C775" t="str">
+        <v>Request AO team to add CPD Live endpoint to liquibas</v>
+      </c>
+      <c r="D775" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E775" t="str">
+        <v>Request AO team to add CPD Live endpoint to liquibas</v>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B776" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C776" t="str">
+        <v>Request AO team to add CPD Live endpoint to liquibase</v>
+      </c>
+      <c r="D776" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E776" t="str">
+        <v>Request AO team to add CPD Live endpoint to liquibase</v>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" t="str">
+        <v>2026-08-17 18:11</v>
+      </c>
+      <c r="B777" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C777" t="str">
+        <v>Request AO team to add CPD Live endpoint to liquibase</v>
+      </c>
+      <c r="D777" t="str">
+        <v>Status changed</v>
+      </c>
+      <c r="E777" t="str">
+        <v>To do → In progress</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E716"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E777"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 11 notes, 3 done (2026-08-18 12:09)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -457,22 +457,22 @@
         <v/>
       </c>
       <c r="D2" t="str">
-        <v>In progress</v>
+        <v>Done</v>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="F2" t="str">
-        <v/>
+        <v>2026-08-17</v>
       </c>
       <c r="G2" t="str">
         <v>2026-08-17</v>
       </c>
       <c r="H2" t="str">
-        <v/>
+        <v>2026-08-18</v>
       </c>
       <c r="I2" t="str">
-        <v>2026-08-17 18:11</v>
+        <v>2026-08-18 12:09</v>
       </c>
       <c r="J2" t="str">
         <v>--p5</v>
@@ -845,7 +845,7 @@
         <v>In progress</v>
       </c>
       <c r="B4">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -853,7 +853,7 @@
         <v>Done</v>
       </c>
       <c r="B5">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -861,7 +861,7 @@
         <v>Overall progress %</v>
       </c>
       <c r="B6">
-        <v>23</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7">
@@ -885,7 +885,7 @@
         <v>Last saved</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-17 18:11</v>
+        <v>2026-08-18 12:09</v>
       </c>
     </row>
   </sheetData>
@@ -991,7 +991,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E777"/>
+  <dimension ref="A1:E779"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -14209,9 +14209,43 @@
         <v>To do → In progress</v>
       </c>
     </row>
+    <row r="778">
+      <c r="A778" t="str">
+        <v>2026-08-18 12:09</v>
+      </c>
+      <c r="B778" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C778" t="str">
+        <v>Request AO team to add CPD Live endpoint to liquibase</v>
+      </c>
+      <c r="D778" t="str">
+        <v>Due date set</v>
+      </c>
+      <c r="E778" t="str">
+        <v>2026-08-17</v>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" t="str">
+        <v>2026-08-18 12:09</v>
+      </c>
+      <c r="B779" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="C779" t="str">
+        <v>Request AO team to add CPD Live endpoint to liquibase</v>
+      </c>
+      <c r="D779" t="str">
+        <v>Status changed</v>
+      </c>
+      <c r="E779" t="str">
+        <v>In progress → Done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E777"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E779"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 11 notes, 2 done (2026-08-18 12:09)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -586,10 +586,10 @@
         <v/>
       </c>
       <c r="D6" t="str">
-        <v>Done</v>
+        <v>To do</v>
       </c>
       <c r="E6">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="F6" t="str">
         <v>2026-08-17</v>
@@ -598,10 +598,10 @@
         <v>2026-08-17</v>
       </c>
       <c r="H6" t="str">
-        <v>2026-08-17</v>
+        <v/>
       </c>
       <c r="I6" t="str">
-        <v>2026-08-17 17:36</v>
+        <v>2026-08-18 12:09</v>
       </c>
       <c r="J6" t="str">
         <v>--p1</v>
@@ -837,7 +837,7 @@
         <v>To do</v>
       </c>
       <c r="B3">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4">
@@ -853,7 +853,7 @@
         <v>Done</v>
       </c>
       <c r="B5">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -861,7 +861,7 @@
         <v>Overall progress %</v>
       </c>
       <c r="B6">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7">
@@ -869,7 +869,7 @@
         <v>Overdue</v>
       </c>
       <c r="B7">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
@@ -991,7 +991,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E779"/>
+  <dimension ref="A1:E780"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -14243,9 +14243,26 @@
         <v>In progress → Done</v>
       </c>
     </row>
+    <row r="780">
+      <c r="A780" t="str">
+        <v>2026-08-18 12:09</v>
+      </c>
+      <c r="B780" t="str">
+        <v>T-27I6K43</v>
+      </c>
+      <c r="C780" t="str">
+        <v>Coveo CPD Keys and Configuration</v>
+      </c>
+      <c r="D780" t="str">
+        <v>Status changed</v>
+      </c>
+      <c r="E780" t="str">
+        <v>Done → To do</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E779"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E780"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 12 notes, 2 done (2026-08-18 12:10)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J13"/>
   <cols>
     <col min="1" max="1" width="11.83203125" customWidth="1"/>
     <col min="2" max="2" width="34.83203125" customWidth="1"/>
@@ -448,79 +448,79 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>T-8399X61</v>
+        <v>T-AMG4458</v>
       </c>
       <c r="B2" t="str">
-        <v>Request AO team to add CPD Live endpoint to liquibase</v>
+        <v xml:space="preserve">Coveo CPD Observation </v>
       </c>
       <c r="C2" t="str">
         <v/>
       </c>
       <c r="D2" t="str">
+        <v>To do</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v>2026-08-18</v>
+      </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
+      <c r="I2" t="str">
+        <v>2026-08-18 12:10</v>
+      </c>
+      <c r="J2" t="str">
+        <v>--p6</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Request AO team to add CPD Live endpoint to liquibase</v>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
         <v>Done</v>
       </c>
-      <c r="E2">
+      <c r="E3">
         <v>100</v>
       </c>
-      <c r="F2" t="str">
+      <c r="F3" t="str">
         <v>2026-08-17</v>
       </c>
-      <c r="G2" t="str">
+      <c r="G3" t="str">
         <v>2026-08-17</v>
       </c>
-      <c r="H2" t="str">
+      <c r="H3" t="str">
         <v>2026-08-18</v>
       </c>
-      <c r="I2" t="str">
+      <c r="I3" t="str">
         <v>2026-08-18 12:09</v>
       </c>
-      <c r="J2" t="str">
+      <c r="J3" t="str">
         <v>--p5</v>
       </c>
     </row>
-    <row r="3" xml:space="preserve">
-      <c r="A3" t="str">
+    <row r="4" xml:space="preserve">
+      <c r="A4" t="str">
         <v>T-31URD46</v>
       </c>
-      <c r="B3" t="str">
+      <c r="B4" t="str">
         <v>Coveo RSW(Spain) recommendation Setup</v>
       </c>
-      <c r="C3" t="str" xml:space="preserve">
+      <c r="C4" t="str" xml:space="preserve">
         <v xml:space="preserve">for 
 Julia before 14.7 UAT</v>
       </c>
-      <c r="D3" t="str">
-        <v>To do</v>
-      </c>
-      <c r="E3">
-        <v>0</v>
-      </c>
-      <c r="F3" t="str">
-        <v/>
-      </c>
-      <c r="G3" t="str">
-        <v>2026-08-17</v>
-      </c>
-      <c r="H3" t="str">
-        <v/>
-      </c>
-      <c r="I3" t="str">
-        <v>2026-08-17 15:51</v>
-      </c>
-      <c r="J3" t="str">
-        <v>--p4</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>T-292O348</v>
-      </c>
-      <c r="B4" t="str">
-        <v>SonarQube Resolve</v>
-      </c>
-      <c r="C4" t="str">
-        <v/>
-      </c>
       <c r="D4" t="str">
         <v>To do</v>
       </c>
@@ -537,18 +537,18 @@
         <v/>
       </c>
       <c r="I4" t="str">
-        <v>2026-08-17 15:31</v>
+        <v>2026-08-17 15:51</v>
       </c>
       <c r="J4" t="str">
-        <v>--p3</v>
+        <v>--p4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>T-28A0V57</v>
+        <v>T-292O348</v>
       </c>
       <c r="B5" t="str">
-        <v>Coveo - CPD explanation to Mohan</v>
+        <v>SonarQube Resolve</v>
       </c>
       <c r="C5" t="str">
         <v/>
@@ -569,30 +569,30 @@
         <v/>
       </c>
       <c r="I5" t="str">
-        <v>2026-08-17 15:27</v>
+        <v>2026-08-17 15:31</v>
       </c>
       <c r="J5" t="str">
-        <v>--p2</v>
+        <v>--p3</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>T-27I6K43</v>
+        <v>T-28A0V57</v>
       </c>
       <c r="B6" t="str">
-        <v>Coveo CPD Keys and Configuration</v>
+        <v>Coveo - CPD explanation to Mohan</v>
       </c>
       <c r="C6" t="str">
         <v/>
       </c>
       <c r="D6" t="str">
-        <v>In progress</v>
+        <v>To do</v>
       </c>
       <c r="E6">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="F6" t="str">
-        <v>2026-08-17</v>
+        <v/>
       </c>
       <c r="G6" t="str">
         <v>2026-08-17</v>
@@ -601,27 +601,27 @@
         <v/>
       </c>
       <c r="I6" t="str">
-        <v>2026-08-18 12:09</v>
+        <v>2026-08-17 15:27</v>
       </c>
       <c r="J6" t="str">
-        <v>--p1</v>
+        <v>--p2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>T-24W7H31</v>
+        <v>T-27I6K43</v>
       </c>
       <c r="B7" t="str">
-        <v xml:space="preserve">CPD - Follow Up for TBD to mathieu </v>
+        <v>Coveo CPD Keys and Configuration</v>
       </c>
       <c r="C7" t="str">
         <v/>
       </c>
       <c r="D7" t="str">
-        <v>Done</v>
+        <v>In progress</v>
       </c>
       <c r="E7">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="F7" t="str">
         <v>2026-08-17</v>
@@ -630,91 +630,91 @@
         <v>2026-08-17</v>
       </c>
       <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="str">
+        <v>2026-08-18 12:09</v>
+      </c>
+      <c r="J7" t="str">
+        <v>--p1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="B8" t="str">
+        <v xml:space="preserve">CPD - Follow Up for TBD to mathieu </v>
+      </c>
+      <c r="C8" t="str">
+        <v/>
+      </c>
+      <c r="D8" t="str">
+        <v>Done</v>
+      </c>
+      <c r="E8">
+        <v>100</v>
+      </c>
+      <c r="F8" t="str">
         <v>2026-08-17</v>
       </c>
-      <c r="I7" t="str">
+      <c r="G8" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H8" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="I8" t="str">
         <v>2026-08-17 16:51</v>
       </c>
-      <c r="J7" t="str">
+      <c r="J8" t="str">
         <v>--p6</v>
       </c>
     </row>
-    <row r="8" xml:space="preserve">
-      <c r="A8" t="str">
-        <v>T-22JLI81</v>
-      </c>
-      <c r="B8" t="str">
+    <row r="9" xml:space="preserve">
+      <c r="A9" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="B9" t="str">
         <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation mail and Confirm Coveo for Production </v>
       </c>
-      <c r="C8" t="str" xml:space="preserve">
+      <c r="C9" t="str" xml:space="preserve">
         <v xml:space="preserve">For 
 RSP, RGG, RSW, BOCT</v>
       </c>
-      <c r="D8" t="str">
+      <c r="D9" t="str">
         <v>In progress</v>
       </c>
-      <c r="E8">
+      <c r="E9">
         <v>50</v>
       </c>
-      <c r="F8" t="str">
+      <c r="F9" t="str">
         <v>2026-08-21</v>
       </c>
-      <c r="G8" t="str">
+      <c r="G9" t="str">
         <v>2026-08-17</v>
       </c>
-      <c r="H8" t="str">
+      <c r="H9" t="str">
         <v/>
       </c>
-      <c r="I8" t="str">
+      <c r="I9" t="str">
         <v>2026-08-17 16:52</v>
       </c>
-      <c r="J8" t="str">
+      <c r="J9" t="str">
         <v>--p5</v>
       </c>
     </row>
-    <row r="9" xml:space="preserve">
-      <c r="A9" t="str">
+    <row r="10" xml:space="preserve">
+      <c r="A10" t="str">
         <v>T-20UNS57</v>
       </c>
-      <c r="B9" t="str">
+      <c r="B10" t="str">
         <v xml:space="preserve">DF--4191 - New Version Recommendation Model Migration </v>
       </c>
-      <c r="C9" t="str" xml:space="preserve">
+      <c r="C10" t="str" xml:space="preserve">
         <v xml:space="preserve">For 
 RGG and RSW (DE and CH store)</v>
       </c>
-      <c r="D9" t="str">
-        <v>To do</v>
-      </c>
-      <c r="E9">
-        <v>0</v>
-      </c>
-      <c r="F9" t="str">
-        <v>2026-08-21</v>
-      </c>
-      <c r="G9" t="str">
-        <v>2026-08-17</v>
-      </c>
-      <c r="H9" t="str">
-        <v/>
-      </c>
-      <c r="I9" t="str">
-        <v>2026-08-17 16:52</v>
-      </c>
-      <c r="J9" t="str">
-        <v>--p4</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>T-1ZZXI87</v>
-      </c>
-      <c r="B10" t="str">
-        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
-      </c>
-      <c r="C10" t="str">
-        <v xml:space="preserve">For grant </v>
-      </c>
       <c r="D10" t="str">
         <v>To do</v>
       </c>
@@ -722,7 +722,7 @@
         <v>0</v>
       </c>
       <c r="F10" t="str">
-        <v/>
+        <v>2026-08-21</v>
       </c>
       <c r="G10" t="str">
         <v>2026-08-17</v>
@@ -731,21 +731,21 @@
         <v/>
       </c>
       <c r="I10" t="str">
-        <v>2026-08-17 15:21</v>
+        <v>2026-08-17 16:52</v>
       </c>
       <c r="J10" t="str">
-        <v>--p3</v>
+        <v>--p4</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>T-1YYRK56</v>
+        <v>T-1ZZXI87</v>
       </c>
       <c r="B11" t="str">
-        <v>Coveo RSP - Recommendation Go-Live for BOC AU store</v>
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
       </c>
       <c r="C11" t="str">
-        <v>for Grant</v>
+        <v xml:space="preserve">For grant </v>
       </c>
       <c r="D11" t="str">
         <v>To do</v>
@@ -763,21 +763,21 @@
         <v/>
       </c>
       <c r="I11" t="str">
-        <v>2026-08-17 15:20</v>
+        <v>2026-08-17 15:21</v>
       </c>
       <c r="J11" t="str">
-        <v>--p2</v>
+        <v>--p3</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>T-1X4UW94</v>
+        <v>T-1YYRK56</v>
       </c>
       <c r="B12" t="str">
-        <v>Coveo RSP- QPM for V2 calls</v>
+        <v>Coveo RSP - Recommendation Go-Live for BOC AU store</v>
       </c>
       <c r="C12" t="str">
-        <v/>
+        <v>for Grant</v>
       </c>
       <c r="D12" t="str">
         <v>To do</v>
@@ -786,7 +786,7 @@
         <v>0</v>
       </c>
       <c r="F12" t="str">
-        <v>2026-08-14</v>
+        <v/>
       </c>
       <c r="G12" t="str">
         <v>2026-08-17</v>
@@ -795,15 +795,47 @@
         <v/>
       </c>
       <c r="I12" t="str">
+        <v>2026-08-17 15:20</v>
+      </c>
+      <c r="J12" t="str">
+        <v>--p2</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Coveo RSP- QPM for V2 calls</v>
+      </c>
+      <c r="C13" t="str">
+        <v/>
+      </c>
+      <c r="D13" t="str">
+        <v>To do</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13" t="str">
+        <v>2026-08-14</v>
+      </c>
+      <c r="G13" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H13" t="str">
+        <v/>
+      </c>
+      <c r="I13" t="str">
         <v>2026-08-17 17:37</v>
       </c>
-      <c r="J12" t="str">
+      <c r="J13" t="str">
         <v>--p1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J13"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -829,7 +861,7 @@
         <v>Total notes</v>
       </c>
       <c r="B2">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3">
@@ -837,7 +869,7 @@
         <v>To do</v>
       </c>
       <c r="B3">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4">
@@ -861,7 +893,7 @@
         <v>Overall progress %</v>
       </c>
       <c r="B6">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7">
@@ -885,7 +917,7 @@
         <v>Last saved</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-18 12:09</v>
+        <v>2026-08-18 12:10</v>
       </c>
     </row>
   </sheetData>
@@ -991,7 +1023,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E781"/>
+  <dimension ref="A1:E804"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -14277,9 +14309,400 @@
         <v>To do → In progress</v>
       </c>
     </row>
+    <row r="782">
+      <c r="A782" t="str">
+        <v>2026-08-18 12:10</v>
+      </c>
+      <c r="B782" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C782" t="str">
+        <v>(untitled)</v>
+      </c>
+      <c r="D782" t="str">
+        <v>Created</v>
+      </c>
+      <c r="E782" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" t="str">
+        <v>2026-08-18 12:10</v>
+      </c>
+      <c r="B783" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C783" t="str">
+        <v>C</v>
+      </c>
+      <c r="D783" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E783" t="str">
+        <v>C</v>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" t="str">
+        <v>2026-08-18 12:10</v>
+      </c>
+      <c r="B784" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C784" t="str">
+        <v>Co</v>
+      </c>
+      <c r="D784" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E784" t="str">
+        <v>Co</v>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" t="str">
+        <v>2026-08-18 12:10</v>
+      </c>
+      <c r="B785" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C785" t="str">
+        <v>Cov</v>
+      </c>
+      <c r="D785" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E785" t="str">
+        <v>Cov</v>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" t="str">
+        <v>2026-08-18 12:10</v>
+      </c>
+      <c r="B786" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C786" t="str">
+        <v>Cove</v>
+      </c>
+      <c r="D786" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E786" t="str">
+        <v>Cove</v>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" t="str">
+        <v>2026-08-18 12:10</v>
+      </c>
+      <c r="B787" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C787" t="str">
+        <v>Coveo</v>
+      </c>
+      <c r="D787" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E787" t="str">
+        <v>Coveo</v>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" t="str">
+        <v>2026-08-18 12:10</v>
+      </c>
+      <c r="B788" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C788" t="str">
+        <v xml:space="preserve">Coveo </v>
+      </c>
+      <c r="D788" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E788" t="str">
+        <v xml:space="preserve">Coveo </v>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" t="str">
+        <v>2026-08-18 12:10</v>
+      </c>
+      <c r="B789" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C789" t="str">
+        <v>Coveo C</v>
+      </c>
+      <c r="D789" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E789" t="str">
+        <v>Coveo C</v>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" t="str">
+        <v>2026-08-18 12:10</v>
+      </c>
+      <c r="B790" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C790" t="str">
+        <v>Coveo CP</v>
+      </c>
+      <c r="D790" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E790" t="str">
+        <v>Coveo CP</v>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" t="str">
+        <v>2026-08-18 12:10</v>
+      </c>
+      <c r="B791" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C791" t="str">
+        <v>Coveo CPD</v>
+      </c>
+      <c r="D791" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E791" t="str">
+        <v>Coveo CPD</v>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" t="str">
+        <v>2026-08-18 12:10</v>
+      </c>
+      <c r="B792" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C792" t="str">
+        <v xml:space="preserve">Coveo CPD </v>
+      </c>
+      <c r="D792" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E792" t="str">
+        <v xml:space="preserve">Coveo CPD </v>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" t="str">
+        <v>2026-08-18 12:10</v>
+      </c>
+      <c r="B793" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C793" t="str">
+        <v>Coveo CPD O</v>
+      </c>
+      <c r="D793" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E793" t="str">
+        <v>Coveo CPD O</v>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" t="str">
+        <v>2026-08-18 12:10</v>
+      </c>
+      <c r="B794" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C794" t="str">
+        <v>Coveo CPD Ob</v>
+      </c>
+      <c r="D794" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E794" t="str">
+        <v>Coveo CPD Ob</v>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" t="str">
+        <v>2026-08-18 12:10</v>
+      </c>
+      <c r="B795" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C795" t="str">
+        <v>Coveo CPD Obs</v>
+      </c>
+      <c r="D795" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E795" t="str">
+        <v>Coveo CPD Obs</v>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" t="str">
+        <v>2026-08-18 12:10</v>
+      </c>
+      <c r="B796" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C796" t="str">
+        <v>Coveo CPD Obse</v>
+      </c>
+      <c r="D796" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E796" t="str">
+        <v>Coveo CPD Obse</v>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" t="str">
+        <v>2026-08-18 12:10</v>
+      </c>
+      <c r="B797" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C797" t="str">
+        <v>Coveo CPD Obser</v>
+      </c>
+      <c r="D797" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E797" t="str">
+        <v>Coveo CPD Obser</v>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" t="str">
+        <v>2026-08-18 12:10</v>
+      </c>
+      <c r="B798" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C798" t="str">
+        <v>Coveo CPD Observ</v>
+      </c>
+      <c r="D798" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E798" t="str">
+        <v>Coveo CPD Observ</v>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" t="str">
+        <v>2026-08-18 12:10</v>
+      </c>
+      <c r="B799" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C799" t="str">
+        <v>Coveo CPD Observa</v>
+      </c>
+      <c r="D799" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E799" t="str">
+        <v>Coveo CPD Observa</v>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" t="str">
+        <v>2026-08-18 12:10</v>
+      </c>
+      <c r="B800" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C800" t="str">
+        <v>Coveo CPD Observat</v>
+      </c>
+      <c r="D800" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E800" t="str">
+        <v>Coveo CPD Observat</v>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" t="str">
+        <v>2026-08-18 12:10</v>
+      </c>
+      <c r="B801" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C801" t="str">
+        <v>Coveo CPD Observati</v>
+      </c>
+      <c r="D801" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E801" t="str">
+        <v>Coveo CPD Observati</v>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" t="str">
+        <v>2026-08-18 12:10</v>
+      </c>
+      <c r="B802" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C802" t="str">
+        <v>Coveo CPD Observatio</v>
+      </c>
+      <c r="D802" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E802" t="str">
+        <v>Coveo CPD Observatio</v>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" t="str">
+        <v>2026-08-18 12:10</v>
+      </c>
+      <c r="B803" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C803" t="str">
+        <v>Coveo CPD Observation</v>
+      </c>
+      <c r="D803" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E803" t="str">
+        <v>Coveo CPD Observation</v>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" t="str">
+        <v>2026-08-18 12:10</v>
+      </c>
+      <c r="B804" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C804" t="str">
+        <v xml:space="preserve">Coveo CPD Observation </v>
+      </c>
+      <c r="D804" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E804" t="str">
+        <v xml:space="preserve">Coveo CPD Observation </v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E781"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E804"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 13 notes, 2 done (2026-08-18 15:05)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J14"/>
   <cols>
     <col min="1" max="1" width="11.83203125" customWidth="1"/>
     <col min="2" max="2" width="34.83203125" customWidth="1"/>
@@ -448,22 +448,22 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>T-AMG4458</v>
+        <v>T-GVGGA16</v>
       </c>
       <c r="B2" t="str">
-        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+        <v/>
       </c>
       <c r="C2" t="str">
         <v/>
       </c>
       <c r="D2" t="str">
-        <v>In progress</v>
+        <v>To do</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-08-17</v>
+        <v/>
       </c>
       <c r="G2" t="str">
         <v>2026-08-18</v>
@@ -472,87 +472,87 @@
         <v/>
       </c>
       <c r="I2" t="str">
-        <v>2026-08-18 12:10</v>
+        <v>2026-08-18 15:05</v>
       </c>
       <c r="J2" t="str">
-        <v>--p6</v>
+        <v>--p1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>T-8399X61</v>
+        <v>T-AMG4458</v>
       </c>
       <c r="B3" t="str">
-        <v>Request AO team to add CPD Live endpoint to liquibase</v>
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
       </c>
       <c r="C3" t="str">
         <v/>
       </c>
       <c r="D3" t="str">
-        <v>Done</v>
+        <v>In progress</v>
       </c>
       <c r="E3">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="F3" t="str">
         <v>2026-08-17</v>
       </c>
       <c r="G3" t="str">
+        <v>2026-08-18</v>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
+        <v>2026-08-18 12:10</v>
+      </c>
+      <c r="J3" t="str">
+        <v>--p6</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Request AO team to add CPD Live endpoint to liquibase</v>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v>Done</v>
+      </c>
+      <c r="E4">
+        <v>100</v>
+      </c>
+      <c r="F4" t="str">
         <v>2026-08-17</v>
       </c>
-      <c r="H3" t="str">
+      <c r="G4" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H4" t="str">
         <v>2026-08-18</v>
       </c>
-      <c r="I3" t="str">
+      <c r="I4" t="str">
         <v>2026-08-18 12:09</v>
       </c>
-      <c r="J3" t="str">
+      <c r="J4" t="str">
         <v>--p5</v>
       </c>
     </row>
-    <row r="4" xml:space="preserve">
-      <c r="A4" t="str">
+    <row r="5" xml:space="preserve">
+      <c r="A5" t="str">
         <v>T-31URD46</v>
       </c>
-      <c r="B4" t="str">
+      <c r="B5" t="str">
         <v>Coveo RSW(Spain) recommendation Setup</v>
       </c>
-      <c r="C4" t="str" xml:space="preserve">
+      <c r="C5" t="str" xml:space="preserve">
         <v xml:space="preserve">for 
 Julia before 14.7 UAT</v>
       </c>
-      <c r="D4" t="str">
-        <v>To do</v>
-      </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-      <c r="F4" t="str">
-        <v/>
-      </c>
-      <c r="G4" t="str">
-        <v>2026-08-17</v>
-      </c>
-      <c r="H4" t="str">
-        <v/>
-      </c>
-      <c r="I4" t="str">
-        <v>2026-08-17 15:51</v>
-      </c>
-      <c r="J4" t="str">
-        <v>--p4</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>T-292O348</v>
-      </c>
-      <c r="B5" t="str">
-        <v>SonarQube Resolve</v>
-      </c>
-      <c r="C5" t="str">
-        <v/>
-      </c>
       <c r="D5" t="str">
         <v>To do</v>
       </c>
@@ -569,18 +569,18 @@
         <v/>
       </c>
       <c r="I5" t="str">
-        <v>2026-08-17 15:31</v>
+        <v>2026-08-17 15:51</v>
       </c>
       <c r="J5" t="str">
-        <v>--p3</v>
+        <v>--p4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>T-28A0V57</v>
+        <v>T-292O348</v>
       </c>
       <c r="B6" t="str">
-        <v>Coveo - CPD explanation to Mohan</v>
+        <v>SonarQube Resolve</v>
       </c>
       <c r="C6" t="str">
         <v/>
@@ -601,30 +601,30 @@
         <v/>
       </c>
       <c r="I6" t="str">
-        <v>2026-08-17 15:27</v>
+        <v>2026-08-17 15:31</v>
       </c>
       <c r="J6" t="str">
-        <v>--p2</v>
+        <v>--p3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>T-27I6K43</v>
+        <v>T-28A0V57</v>
       </c>
       <c r="B7" t="str">
-        <v>Coveo CPD Keys and Configuration</v>
+        <v>Coveo - CPD explanation to Mohan</v>
       </c>
       <c r="C7" t="str">
         <v/>
       </c>
       <c r="D7" t="str">
-        <v>In progress</v>
+        <v>To do</v>
       </c>
       <c r="E7">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="F7" t="str">
-        <v>2026-08-17</v>
+        <v/>
       </c>
       <c r="G7" t="str">
         <v>2026-08-17</v>
@@ -633,27 +633,27 @@
         <v/>
       </c>
       <c r="I7" t="str">
-        <v>2026-08-18 12:09</v>
+        <v>2026-08-17 15:27</v>
       </c>
       <c r="J7" t="str">
-        <v>--p1</v>
+        <v>--p2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>T-24W7H31</v>
+        <v>T-27I6K43</v>
       </c>
       <c r="B8" t="str">
-        <v xml:space="preserve">CPD - Follow Up for TBD to mathieu </v>
+        <v>Coveo CPD Keys and Configuration</v>
       </c>
       <c r="C8" t="str">
         <v/>
       </c>
       <c r="D8" t="str">
-        <v>Done</v>
+        <v>In progress</v>
       </c>
       <c r="E8">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="F8" t="str">
         <v>2026-08-17</v>
@@ -662,91 +662,91 @@
         <v>2026-08-17</v>
       </c>
       <c r="H8" t="str">
+        <v/>
+      </c>
+      <c r="I8" t="str">
+        <v>2026-08-18 12:09</v>
+      </c>
+      <c r="J8" t="str">
+        <v>--p1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="B9" t="str">
+        <v xml:space="preserve">CPD - Follow Up for TBD to mathieu </v>
+      </c>
+      <c r="C9" t="str">
+        <v/>
+      </c>
+      <c r="D9" t="str">
+        <v>Done</v>
+      </c>
+      <c r="E9">
+        <v>100</v>
+      </c>
+      <c r="F9" t="str">
         <v>2026-08-17</v>
       </c>
-      <c r="I8" t="str">
+      <c r="G9" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H9" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="I9" t="str">
         <v>2026-08-17 16:51</v>
       </c>
-      <c r="J8" t="str">
+      <c r="J9" t="str">
         <v>--p6</v>
       </c>
     </row>
-    <row r="9" xml:space="preserve">
-      <c r="A9" t="str">
-        <v>T-22JLI81</v>
-      </c>
-      <c r="B9" t="str">
+    <row r="10" xml:space="preserve">
+      <c r="A10" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="B10" t="str">
         <v xml:space="preserve">Coveo Global Configuration API Deprecation Confirmation mail and Confirm Coveo for Production </v>
       </c>
-      <c r="C9" t="str" xml:space="preserve">
+      <c r="C10" t="str" xml:space="preserve">
         <v xml:space="preserve">For 
 RSP, RGG, RSW, BOCT</v>
       </c>
-      <c r="D9" t="str">
+      <c r="D10" t="str">
         <v>In progress</v>
       </c>
-      <c r="E9">
+      <c r="E10">
         <v>50</v>
       </c>
-      <c r="F9" t="str">
+      <c r="F10" t="str">
         <v>2026-08-21</v>
       </c>
-      <c r="G9" t="str">
+      <c r="G10" t="str">
         <v>2026-08-17</v>
       </c>
-      <c r="H9" t="str">
+      <c r="H10" t="str">
         <v/>
       </c>
-      <c r="I9" t="str">
+      <c r="I10" t="str">
         <v>2026-08-17 16:52</v>
       </c>
-      <c r="J9" t="str">
+      <c r="J10" t="str">
         <v>--p5</v>
       </c>
     </row>
-    <row r="10" xml:space="preserve">
-      <c r="A10" t="str">
+    <row r="11" xml:space="preserve">
+      <c r="A11" t="str">
         <v>T-20UNS57</v>
       </c>
-      <c r="B10" t="str">
+      <c r="B11" t="str">
         <v xml:space="preserve">DF--4191 - New Version Recommendation Model Migration </v>
       </c>
-      <c r="C10" t="str" xml:space="preserve">
+      <c r="C11" t="str" xml:space="preserve">
         <v xml:space="preserve">For 
 RGG and RSW (DE and CH store)</v>
       </c>
-      <c r="D10" t="str">
-        <v>To do</v>
-      </c>
-      <c r="E10">
-        <v>0</v>
-      </c>
-      <c r="F10" t="str">
-        <v>2026-08-21</v>
-      </c>
-      <c r="G10" t="str">
-        <v>2026-08-17</v>
-      </c>
-      <c r="H10" t="str">
-        <v/>
-      </c>
-      <c r="I10" t="str">
-        <v>2026-08-17 16:52</v>
-      </c>
-      <c r="J10" t="str">
-        <v>--p4</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>T-1ZZXI87</v>
-      </c>
-      <c r="B11" t="str">
-        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
-      </c>
-      <c r="C11" t="str">
-        <v xml:space="preserve">For grant </v>
-      </c>
       <c r="D11" t="str">
         <v>To do</v>
       </c>
@@ -754,7 +754,7 @@
         <v>0</v>
       </c>
       <c r="F11" t="str">
-        <v/>
+        <v>2026-08-21</v>
       </c>
       <c r="G11" t="str">
         <v>2026-08-17</v>
@@ -763,21 +763,21 @@
         <v/>
       </c>
       <c r="I11" t="str">
-        <v>2026-08-17 15:21</v>
+        <v>2026-08-17 16:52</v>
       </c>
       <c r="J11" t="str">
-        <v>--p3</v>
+        <v>--p4</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>T-1YYRK56</v>
+        <v>T-1ZZXI87</v>
       </c>
       <c r="B12" t="str">
-        <v>Coveo RSP - Recommendation Go-Live for BOC AU store</v>
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
       </c>
       <c r="C12" t="str">
-        <v>for Grant</v>
+        <v xml:space="preserve">For grant </v>
       </c>
       <c r="D12" t="str">
         <v>To do</v>
@@ -795,21 +795,21 @@
         <v/>
       </c>
       <c r="I12" t="str">
-        <v>2026-08-17 15:20</v>
+        <v>2026-08-17 15:21</v>
       </c>
       <c r="J12" t="str">
-        <v>--p2</v>
+        <v>--p3</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>T-1X4UW94</v>
+        <v>T-1YYRK56</v>
       </c>
       <c r="B13" t="str">
-        <v>Coveo RSP- QPM for V2 calls</v>
+        <v>Coveo RSP - Recommendation Go-Live for BOC AU store</v>
       </c>
       <c r="C13" t="str">
-        <v/>
+        <v>for Grant</v>
       </c>
       <c r="D13" t="str">
         <v>To do</v>
@@ -818,7 +818,7 @@
         <v>0</v>
       </c>
       <c r="F13" t="str">
-        <v>2026-08-14</v>
+        <v/>
       </c>
       <c r="G13" t="str">
         <v>2026-08-17</v>
@@ -827,15 +827,47 @@
         <v/>
       </c>
       <c r="I13" t="str">
+        <v>2026-08-17 15:20</v>
+      </c>
+      <c r="J13" t="str">
+        <v>--p2</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Coveo RSP- QPM for V2 calls</v>
+      </c>
+      <c r="C14" t="str">
+        <v/>
+      </c>
+      <c r="D14" t="str">
+        <v>To do</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+      <c r="F14" t="str">
+        <v>2026-08-14</v>
+      </c>
+      <c r="G14" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H14" t="str">
+        <v/>
+      </c>
+      <c r="I14" t="str">
         <v>2026-08-17 17:37</v>
       </c>
-      <c r="J13" t="str">
+      <c r="J14" t="str">
         <v>--p1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J14"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -861,7 +893,7 @@
         <v>Total notes</v>
       </c>
       <c r="B2">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3">
@@ -869,7 +901,7 @@
         <v>To do</v>
       </c>
       <c r="B3">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4">
@@ -893,7 +925,7 @@
         <v>Overall progress %</v>
       </c>
       <c r="B6">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7">
@@ -917,7 +949,7 @@
         <v>Last saved</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-18 12:10</v>
+        <v>2026-08-18 15:05</v>
       </c>
     </row>
   </sheetData>
@@ -1023,7 +1055,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E833"/>
+  <dimension ref="A1:E836"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -15193,9 +15225,60 @@
         <v>2026-08-17</v>
       </c>
     </row>
+    <row r="834">
+      <c r="A834" t="str">
+        <v>2026-08-18 15:05</v>
+      </c>
+      <c r="B834" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C834" t="str">
+        <v>(untitled)</v>
+      </c>
+      <c r="D834" t="str">
+        <v>Created</v>
+      </c>
+      <c r="E834" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" t="str">
+        <v>2026-08-18 15:05</v>
+      </c>
+      <c r="B835" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C835" t="str">
+        <v>C</v>
+      </c>
+      <c r="D835" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E835" t="str">
+        <v>C</v>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" t="str">
+        <v>2026-08-18 15:05</v>
+      </c>
+      <c r="B836" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C836" t="str">
+        <v>(untitled)</v>
+      </c>
+      <c r="D836" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E836" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E833"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E836"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 13 notes, 2 done (2026-08-18 15:06)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -451,7 +451,7 @@
         <v>T-GVGGA16</v>
       </c>
       <c r="B2" t="str">
-        <v xml:space="preserve">LIN-40309 QS model </v>
+        <v>LIN-40309 QS model for CPD</v>
       </c>
       <c r="C2" t="str">
         <v/>
@@ -949,7 +949,7 @@
         <v>Last saved</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-18 15:05</v>
+        <v>2026-08-18 15:06</v>
       </c>
     </row>
   </sheetData>
@@ -1055,7 +1055,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E849"/>
+  <dimension ref="A1:E856"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -15497,9 +15497,128 @@
         <v xml:space="preserve">LIN-40309 QS model </v>
       </c>
     </row>
+    <row r="850">
+      <c r="A850" t="str">
+        <v>2026-08-18 15:05</v>
+      </c>
+      <c r="B850" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C850" t="str">
+        <v>LIN-40309 QS model f</v>
+      </c>
+      <c r="D850" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E850" t="str">
+        <v>LIN-40309 QS model f</v>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" t="str">
+        <v>2026-08-18 15:05</v>
+      </c>
+      <c r="B851" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C851" t="str">
+        <v>LIN-40309 QS model fo</v>
+      </c>
+      <c r="D851" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E851" t="str">
+        <v>LIN-40309 QS model fo</v>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" t="str">
+        <v>2026-08-18 15:05</v>
+      </c>
+      <c r="B852" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C852" t="str">
+        <v>LIN-40309 QS model for</v>
+      </c>
+      <c r="D852" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E852" t="str">
+        <v>LIN-40309 QS model for</v>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" t="str">
+        <v>2026-08-18 15:05</v>
+      </c>
+      <c r="B853" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C853" t="str">
+        <v xml:space="preserve">LIN-40309 QS model for </v>
+      </c>
+      <c r="D853" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E853" t="str">
+        <v xml:space="preserve">LIN-40309 QS model for </v>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" t="str">
+        <v>2026-08-18 15:05</v>
+      </c>
+      <c r="B854" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C854" t="str">
+        <v>LIN-40309 QS model for C</v>
+      </c>
+      <c r="D854" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E854" t="str">
+        <v>LIN-40309 QS model for C</v>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" t="str">
+        <v>2026-08-18 15:05</v>
+      </c>
+      <c r="B855" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C855" t="str">
+        <v>LIN-40309 QS model for CP</v>
+      </c>
+      <c r="D855" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E855" t="str">
+        <v>LIN-40309 QS model for CP</v>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" t="str">
+        <v>2026-08-18 15:05</v>
+      </c>
+      <c r="B856" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C856" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D856" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E856" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E849"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E856"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 13 notes, 2 done (2026-08-18 15:07)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -487,7 +487,7 @@
         <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
       </c>
       <c r="C3" t="str">
-        <v/>
+        <v>Sent mail to Mathieu, regarding product carasol</v>
       </c>
       <c r="D3" t="str">
         <v>In progress</v>
@@ -505,7 +505,7 @@
         <v/>
       </c>
       <c r="I3" t="str">
-        <v>2026-08-18 12:10</v>
+        <v>2026-08-18 15:07</v>
       </c>
       <c r="J3" t="str">
         <v>--p6</v>
@@ -950,7 +950,7 @@
         <v>Last saved</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-18 15:06</v>
+        <v>2026-08-18 15:07</v>
       </c>
     </row>
   </sheetData>
@@ -1056,7 +1056,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E880"/>
+  <dimension ref="A1:E940"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -16025,9 +16025,1029 @@
         <v xml:space="preserve">return only queries </v>
       </c>
     </row>
+    <row r="881">
+      <c r="A881" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B881" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C881" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D881" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E881" t="str">
+        <v>S</v>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B882" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C882" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D882" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E882" t="str">
+        <v>Se</v>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B883" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C883" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D883" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E883" t="str">
+        <v>Sen</v>
+      </c>
+    </row>
+    <row r="884">
+      <c r="A884" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B884" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C884" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D884" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E884" t="str">
+        <v>Sent</v>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B885" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C885" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D885" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E885" t="str">
+        <v xml:space="preserve">Sent </v>
+      </c>
+    </row>
+    <row r="886">
+      <c r="A886" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B886" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C886" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D886" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E886" t="str">
+        <v>Sent m</v>
+      </c>
+    </row>
+    <row r="887">
+      <c r="A887" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B887" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C887" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D887" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E887" t="str">
+        <v>Sent ma</v>
+      </c>
+    </row>
+    <row r="888">
+      <c r="A888" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B888" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C888" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D888" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E888" t="str">
+        <v>Sent mai</v>
+      </c>
+    </row>
+    <row r="889">
+      <c r="A889" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B889" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C889" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D889" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E889" t="str">
+        <v>Sent mail</v>
+      </c>
+    </row>
+    <row r="890">
+      <c r="A890" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B890" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C890" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D890" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E890" t="str">
+        <v xml:space="preserve">Sent mail </v>
+      </c>
+    </row>
+    <row r="891">
+      <c r="A891" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B891" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C891" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D891" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E891" t="str">
+        <v>Sent mail t</v>
+      </c>
+    </row>
+    <row r="892">
+      <c r="A892" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B892" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C892" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D892" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E892" t="str">
+        <v>Sent mail to</v>
+      </c>
+    </row>
+    <row r="893">
+      <c r="A893" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B893" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C893" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D893" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E893" t="str">
+        <v xml:space="preserve">Sent mail to </v>
+      </c>
+    </row>
+    <row r="894">
+      <c r="A894" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B894" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C894" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D894" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E894" t="str">
+        <v>Sent mail to M</v>
+      </c>
+    </row>
+    <row r="895">
+      <c r="A895" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B895" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C895" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D895" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E895" t="str">
+        <v>Sent mail to Ma</v>
+      </c>
+    </row>
+    <row r="896">
+      <c r="A896" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B896" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C896" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D896" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E896" t="str">
+        <v>Sent mail to Mat</v>
+      </c>
+    </row>
+    <row r="897">
+      <c r="A897" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B897" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C897" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D897" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E897" t="str">
+        <v>Sent mail to Math</v>
+      </c>
+    </row>
+    <row r="898">
+      <c r="A898" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B898" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C898" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D898" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E898" t="str">
+        <v>Sent mail to Mathi</v>
+      </c>
+    </row>
+    <row r="899">
+      <c r="A899" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B899" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C899" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D899" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E899" t="str">
+        <v>Sent mail to Mathie</v>
+      </c>
+    </row>
+    <row r="900">
+      <c r="A900" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B900" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C900" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D900" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E900" t="str">
+        <v>Sent mail to Mathieu</v>
+      </c>
+    </row>
+    <row r="901">
+      <c r="A901" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B901" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C901" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D901" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E901" t="str">
+        <v xml:space="preserve">Sent mail to Mathieu </v>
+      </c>
+    </row>
+    <row r="902">
+      <c r="A902" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B902" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C902" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D902" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E902" t="str">
+        <v>Sent mail to Mathieu</v>
+      </c>
+    </row>
+    <row r="903">
+      <c r="A903" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B903" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C903" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D903" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E903" t="str">
+        <v>Sent mail to Mathieu,</v>
+      </c>
+    </row>
+    <row r="904">
+      <c r="A904" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B904" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C904" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D904" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E904" t="str">
+        <v xml:space="preserve">Sent mail to Mathieu, </v>
+      </c>
+    </row>
+    <row r="905">
+      <c r="A905" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B905" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C905" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D905" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E905" t="str">
+        <v>Sent mail to Mathieu, r</v>
+      </c>
+    </row>
+    <row r="906">
+      <c r="A906" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B906" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C906" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D906" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E906" t="str">
+        <v>Sent mail to Mathieu, re</v>
+      </c>
+    </row>
+    <row r="907">
+      <c r="A907" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B907" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C907" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D907" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E907" t="str">
+        <v>Sent mail to Mathieu, reh</v>
+      </c>
+    </row>
+    <row r="908">
+      <c r="A908" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B908" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C908" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D908" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E908" t="str">
+        <v>Sent mail to Mathieu, rehg</v>
+      </c>
+    </row>
+    <row r="909">
+      <c r="A909" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B909" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C909" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D909" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E909" t="str">
+        <v>Sent mail to Mathieu, rehga</v>
+      </c>
+    </row>
+    <row r="910">
+      <c r="A910" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B910" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C910" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D910" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E910" t="str">
+        <v>Sent mail to Mathieu, rehgar</v>
+      </c>
+    </row>
+    <row r="911">
+      <c r="A911" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B911" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C911" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D911" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E911" t="str">
+        <v>Sent mail to Mathieu, rehgard</v>
+      </c>
+    </row>
+    <row r="912">
+      <c r="A912" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B912" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C912" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D912" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E912" t="str">
+        <v>Sent mail to Mathieu, rehgardi</v>
+      </c>
+    </row>
+    <row r="913">
+      <c r="A913" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B913" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C913" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D913" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E913" t="str">
+        <v>Sent mail to Mathieu, rehgardin</v>
+      </c>
+    </row>
+    <row r="914">
+      <c r="A914" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B914" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C914" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D914" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E914" t="str">
+        <v>Sent mail to Mathieu, rehgarding</v>
+      </c>
+    </row>
+    <row r="915">
+      <c r="A915" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B915" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C915" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D915" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E915" t="str">
+        <v xml:space="preserve">Sent mail to Mathieu, rehgarding </v>
+      </c>
+    </row>
+    <row r="916">
+      <c r="A916" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B916" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C916" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D916" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E916" t="str">
+        <v>Sent mail to Mathieu, rehgarding p</v>
+      </c>
+    </row>
+    <row r="917">
+      <c r="A917" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B917" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C917" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D917" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E917" t="str">
+        <v>Sent mail to Mathieu, rehgarding pr</v>
+      </c>
+    </row>
+    <row r="918">
+      <c r="A918" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B918" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C918" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D918" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E918" t="str">
+        <v>Sent mail to Mathieu, rehgarding pro</v>
+      </c>
+    </row>
+    <row r="919">
+      <c r="A919" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B919" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C919" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D919" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E919" t="str">
+        <v>Sent mail to Mathieu, rehgarding prod</v>
+      </c>
+    </row>
+    <row r="920">
+      <c r="A920" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B920" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C920" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D920" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E920" t="str">
+        <v>Sent mail to Mathieu, rehgarding produ</v>
+      </c>
+    </row>
+    <row r="921">
+      <c r="A921" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B921" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C921" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D921" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E921" t="str">
+        <v>Sent mail to Mathieu, rehgarding produc</v>
+      </c>
+    </row>
+    <row r="922">
+      <c r="A922" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B922" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C922" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D922" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E922" t="str">
+        <v>Sent mail to Mathieu, rehgarding product</v>
+      </c>
+    </row>
+    <row r="923">
+      <c r="A923" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B923" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C923" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D923" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E923" t="str">
+        <v xml:space="preserve">Sent mail to Mathieu, rehgarding product </v>
+      </c>
+    </row>
+    <row r="924">
+      <c r="A924" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B924" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C924" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D924" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E924" t="str">
+        <v>Sent mail to Mathieu, rehgarding product c</v>
+      </c>
+    </row>
+    <row r="925">
+      <c r="A925" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B925" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C925" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D925" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E925" t="str">
+        <v>Sent mail to Mathieu, rehgarding product ca</v>
+      </c>
+    </row>
+    <row r="926">
+      <c r="A926" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B926" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C926" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D926" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E926" t="str">
+        <v>Sent mail to Mathieu, rehgarding product car</v>
+      </c>
+    </row>
+    <row r="927">
+      <c r="A927" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B927" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C927" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D927" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E927" t="str">
+        <v>Sent mail to Mathieu, rehgarding product cara</v>
+      </c>
+    </row>
+    <row r="928">
+      <c r="A928" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B928" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C928" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D928" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E928" t="str">
+        <v>Sent mail to Mathieu, rehgarding product caras</v>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B929" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C929" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D929" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E929" t="str">
+        <v>Sent mail to Mathieu, rehgarding product caraso</v>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" t="str">
+        <v>2026-08-18 15:06</v>
+      </c>
+      <c r="B930" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C930" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D930" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E930" t="str">
+        <v>Sent mail to Mathieu, rehgarding product carasol</v>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" t="str">
+        <v>2026-08-18 15:07</v>
+      </c>
+      <c r="B931" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C931" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D931" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E931" t="str">
+        <v>Sent mail to Mathieu, rproduct carasol</v>
+      </c>
+    </row>
+    <row r="932">
+      <c r="A932" t="str">
+        <v>2026-08-18 15:07</v>
+      </c>
+      <c r="B932" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C932" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D932" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E932" t="str">
+        <v>Sent mail to Mathieu, reproduct carasol</v>
+      </c>
+    </row>
+    <row r="933">
+      <c r="A933" t="str">
+        <v>2026-08-18 15:07</v>
+      </c>
+      <c r="B933" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C933" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D933" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E933" t="str">
+        <v>Sent mail to Mathieu, regproduct carasol</v>
+      </c>
+    </row>
+    <row r="934">
+      <c r="A934" t="str">
+        <v>2026-08-18 15:07</v>
+      </c>
+      <c r="B934" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C934" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D934" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E934" t="str">
+        <v>Sent mail to Mathieu, regaproduct carasol</v>
+      </c>
+    </row>
+    <row r="935">
+      <c r="A935" t="str">
+        <v>2026-08-18 15:07</v>
+      </c>
+      <c r="B935" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C935" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D935" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E935" t="str">
+        <v>Sent mail to Mathieu, regarproduct carasol</v>
+      </c>
+    </row>
+    <row r="936">
+      <c r="A936" t="str">
+        <v>2026-08-18 15:07</v>
+      </c>
+      <c r="B936" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C936" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D936" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E936" t="str">
+        <v>Sent mail to Mathieu, regardproduct carasol</v>
+      </c>
+    </row>
+    <row r="937">
+      <c r="A937" t="str">
+        <v>2026-08-18 15:07</v>
+      </c>
+      <c r="B937" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C937" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D937" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E937" t="str">
+        <v>Sent mail to Mathieu, regardiproduct carasol</v>
+      </c>
+    </row>
+    <row r="938">
+      <c r="A938" t="str">
+        <v>2026-08-18 15:07</v>
+      </c>
+      <c r="B938" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C938" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D938" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E938" t="str">
+        <v>Sent mail to Mathieu, regardinproduct carasol</v>
+      </c>
+    </row>
+    <row r="939">
+      <c r="A939" t="str">
+        <v>2026-08-18 15:07</v>
+      </c>
+      <c r="B939" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C939" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D939" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E939" t="str">
+        <v>Sent mail to Mathieu, regardingproduct carasol</v>
+      </c>
+    </row>
+    <row r="940">
+      <c r="A940" t="str">
+        <v>2026-08-18 15:07</v>
+      </c>
+      <c r="B940" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C940" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D940" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E940" t="str">
+        <v>Sent mail to Mathieu, regarding product carasol</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E880"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E940"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 13 notes, 2 done (2026-08-18 15:08)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -649,8 +649,7 @@
       </c>
       <c r="C8" t="str" xml:space="preserve">
         <v xml:space="preserve">Created 42 keys with liquibase 
-still pending...
-</v>
+still pending...</v>
       </c>
       <c r="D8" t="str">
         <v>In progress</v>
@@ -668,7 +667,7 @@
         <v/>
       </c>
       <c r="I8" t="str">
-        <v>2026-08-18 15:07</v>
+        <v>2026-08-18 15:08</v>
       </c>
       <c r="J8" t="str">
         <v>--p1</v>
@@ -952,7 +951,7 @@
         <v>Last saved</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-18 15:07</v>
+        <v>2026-08-18 15:08</v>
       </c>
     </row>
   </sheetData>
@@ -1058,7 +1057,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E990"/>
+  <dimension ref="A1:E991"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -17897,9 +17896,26 @@
         <v xml:space="preserve">Created 42 keys with liquibase  still pending... </v>
       </c>
     </row>
+    <row r="991">
+      <c r="A991" t="str">
+        <v>2026-08-18 15:08</v>
+      </c>
+      <c r="B991" t="str">
+        <v>T-27I6K43</v>
+      </c>
+      <c r="C991" t="str">
+        <v>Coveo CPD Keys and Configuration</v>
+      </c>
+      <c r="D991" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E991" t="str">
+        <v>Created 42 keys with liquibase  still pending...</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E990"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E991"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 13 notes, 2 done (2026-08-18 15:09)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -715,7 +715,7 @@
       <c r="C10" t="str" xml:space="preserve">
         <v xml:space="preserve">For 
 RSP, RGG, RSW, BOCT
-To send Send Confirmation mail and Confirm Coveo for Production </v>
+To send Send Confirmation mail and Confirm Coveo for Production enablement</v>
       </c>
       <c r="D10" t="str">
         <v>In progress</v>
@@ -733,7 +733,7 @@
         <v/>
       </c>
       <c r="I10" t="str">
-        <v>2026-08-18 15:08</v>
+        <v>2026-08-18 15:09</v>
       </c>
       <c r="J10" t="str">
         <v>--p5</v>
@@ -952,7 +952,7 @@
         <v>Last saved</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-18 15:08</v>
+        <v>2026-08-18 15:09</v>
       </c>
     </row>
   </sheetData>
@@ -1058,7 +1058,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E1021"/>
+  <dimension ref="A1:E1037"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -18424,9 +18424,281 @@
         <v>For  RSP, RGG, RSW, BOCT To send Send Confirmation mail and Confirm Coveo for Pr</v>
       </c>
     </row>
+    <row r="1022">
+      <c r="A1022" t="str">
+        <v>2026-08-18 15:09</v>
+      </c>
+      <c r="B1022" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C1022" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation </v>
+      </c>
+      <c r="D1022" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1022" t="str">
+        <v>For  RSP, RGG, RSW, BOCT To send Send Confirmation mail and Confirm Coveo for Pr</v>
+      </c>
+    </row>
+    <row r="1023">
+      <c r="A1023" t="str">
+        <v>2026-08-18 15:09</v>
+      </c>
+      <c r="B1023" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C1023" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation </v>
+      </c>
+      <c r="D1023" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1023" t="str">
+        <v>For  RSP, RGG, RSW, BOCT To send Send Confirmation mail and Confirm Coveo for Pr</v>
+      </c>
+    </row>
+    <row r="1024">
+      <c r="A1024" t="str">
+        <v>2026-08-18 15:09</v>
+      </c>
+      <c r="B1024" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C1024" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation </v>
+      </c>
+      <c r="D1024" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1024" t="str">
+        <v>For  RSP, RGG, RSW, BOCT To send Send Confirmation mail and Confirm Coveo for Pr</v>
+      </c>
+    </row>
+    <row r="1025">
+      <c r="A1025" t="str">
+        <v>2026-08-18 15:09</v>
+      </c>
+      <c r="B1025" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C1025" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation </v>
+      </c>
+      <c r="D1025" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1025" t="str">
+        <v>For  RSP, RGG, RSW, BOCT To send Send Confirmation mail and Confirm Coveo for Pr</v>
+      </c>
+    </row>
+    <row r="1026">
+      <c r="A1026" t="str">
+        <v>2026-08-18 15:09</v>
+      </c>
+      <c r="B1026" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C1026" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation </v>
+      </c>
+      <c r="D1026" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1026" t="str">
+        <v>For  RSP, RGG, RSW, BOCT To send Send Confirmation mail and Confirm Coveo for Pr</v>
+      </c>
+    </row>
+    <row r="1027">
+      <c r="A1027" t="str">
+        <v>2026-08-18 15:09</v>
+      </c>
+      <c r="B1027" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C1027" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation </v>
+      </c>
+      <c r="D1027" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1027" t="str">
+        <v>For  RSP, RGG, RSW, BOCT To send Send Confirmation mail and Confirm Coveo for Pr</v>
+      </c>
+    </row>
+    <row r="1028">
+      <c r="A1028" t="str">
+        <v>2026-08-18 15:09</v>
+      </c>
+      <c r="B1028" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C1028" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation </v>
+      </c>
+      <c r="D1028" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1028" t="str">
+        <v>For  RSP, RGG, RSW, BOCT To send Send Confirmation mail and Confirm Coveo for Pr</v>
+      </c>
+    </row>
+    <row r="1029">
+      <c r="A1029" t="str">
+        <v>2026-08-18 15:09</v>
+      </c>
+      <c r="B1029" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C1029" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation </v>
+      </c>
+      <c r="D1029" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1029" t="str">
+        <v>For  RSP, RGG, RSW, BOCT To send Send Confirmation mail and Confirm Coveo for Pr</v>
+      </c>
+    </row>
+    <row r="1030">
+      <c r="A1030" t="str">
+        <v>2026-08-18 15:09</v>
+      </c>
+      <c r="B1030" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C1030" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation </v>
+      </c>
+      <c r="D1030" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1030" t="str">
+        <v>For  RSP, RGG, RSW, BOCT To send Send Confirmation mail and Confirm Coveo for Pr</v>
+      </c>
+    </row>
+    <row r="1031">
+      <c r="A1031" t="str">
+        <v>2026-08-18 15:09</v>
+      </c>
+      <c r="B1031" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C1031" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation </v>
+      </c>
+      <c r="D1031" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1031" t="str">
+        <v>For  RSP, RGG, RSW, BOCT To send Send Confirmation mail and Confirm Coveo for Pr</v>
+      </c>
+    </row>
+    <row r="1032">
+      <c r="A1032" t="str">
+        <v>2026-08-18 15:09</v>
+      </c>
+      <c r="B1032" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C1032" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation </v>
+      </c>
+      <c r="D1032" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1032" t="str">
+        <v>For  RSP, RGG, RSW, BOCT To send Send Confirmation mail and Confirm Coveo for Pr</v>
+      </c>
+    </row>
+    <row r="1033">
+      <c r="A1033" t="str">
+        <v>2026-08-18 15:09</v>
+      </c>
+      <c r="B1033" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C1033" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation </v>
+      </c>
+      <c r="D1033" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1033" t="str">
+        <v>For  RSP, RGG, RSW, BOCT To send Send Confirmation mail and Confirm Coveo for Pr</v>
+      </c>
+    </row>
+    <row r="1034">
+      <c r="A1034" t="str">
+        <v>2026-08-18 15:09</v>
+      </c>
+      <c r="B1034" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C1034" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation </v>
+      </c>
+      <c r="D1034" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1034" t="str">
+        <v>For  RSP, RGG, RSW, BOCT To send Send Confirmation mail and Confirm Coveo for Pr</v>
+      </c>
+    </row>
+    <row r="1035">
+      <c r="A1035" t="str">
+        <v>2026-08-18 15:09</v>
+      </c>
+      <c r="B1035" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C1035" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation </v>
+      </c>
+      <c r="D1035" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1035" t="str">
+        <v>For  RSP, RGG, RSW, BOCT To send Send Confirmation mail and Confirm Coveo for Pr</v>
+      </c>
+    </row>
+    <row r="1036">
+      <c r="A1036" t="str">
+        <v>2026-08-18 15:09</v>
+      </c>
+      <c r="B1036" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C1036" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation </v>
+      </c>
+      <c r="D1036" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1036" t="str">
+        <v>For  RSP, RGG, RSW, BOCT To send Send Confirmation mail and Confirm Coveo for Pr</v>
+      </c>
+    </row>
+    <row r="1037">
+      <c r="A1037" t="str">
+        <v>2026-08-18 15:09</v>
+      </c>
+      <c r="B1037" t="str">
+        <v>T-22JLI81</v>
+      </c>
+      <c r="C1037" t="str">
+        <v xml:space="preserve">Coveo Global Configuration API Deprecation </v>
+      </c>
+      <c r="D1037" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1037" t="str">
+        <v>For  RSP, RGG, RSW, BOCT To send Send Confirmation mail and Confirm Coveo for Pr</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E1021"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E1037"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 13 notes, 3 done (2026-08-19 10:41)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -619,10 +619,10 @@
         <v/>
       </c>
       <c r="D7" t="str">
-        <v>To do</v>
+        <v>Done</v>
       </c>
       <c r="E7">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="F7" t="str">
         <v/>
@@ -631,10 +631,10 @@
         <v>2026-08-17</v>
       </c>
       <c r="H7" t="str">
-        <v/>
+        <v>2026-08-19</v>
       </c>
       <c r="I7" t="str">
-        <v>2026-08-17 15:27</v>
+        <v>2026-08-19 10:41</v>
       </c>
       <c r="J7" t="str">
         <v>--p2</v>
@@ -904,7 +904,7 @@
         <v>To do</v>
       </c>
       <c r="B3">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4">
@@ -920,7 +920,7 @@
         <v>Done</v>
       </c>
       <c r="B5">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -928,7 +928,7 @@
         <v>Overall progress %</v>
       </c>
       <c r="B6">
-        <v>26</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7">
@@ -936,7 +936,7 @@
         <v>Overdue</v>
       </c>
       <c r="B7">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
@@ -952,7 +952,7 @@
         <v>Last saved</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-18 15:09</v>
+        <v>2026-08-19 10:41</v>
       </c>
     </row>
   </sheetData>
@@ -1058,7 +1058,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E1037"/>
+  <dimension ref="A1:E1038"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -18696,9 +18696,26 @@
         <v>For  RSP, RGG, RSW, BOCT To send Send Confirmation mail and Confirm Coveo for Pr</v>
       </c>
     </row>
+    <row r="1038">
+      <c r="A1038" t="str">
+        <v>2026-08-19 10:41</v>
+      </c>
+      <c r="B1038" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="C1038" t="str">
+        <v>Coveo - CPD explanation to Mohan</v>
+      </c>
+      <c r="D1038" t="str">
+        <v>Status changed</v>
+      </c>
+      <c r="E1038" t="str">
+        <v>To do → Done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E1037"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E1038"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 13 notes, 3 done (2026-08-19 10:47)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -479,15 +479,16 @@
         <v>--p1</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" xml:space="preserve">
       <c r="A3" t="str">
         <v>T-AMG4458</v>
       </c>
       <c r="B3" t="str">
         <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
       </c>
-      <c r="C3" t="str">
-        <v>Sent mail to Mathieu, regarding product carousel</v>
+      <c r="C3" t="str" xml:space="preserve">
+        <v xml:space="preserve">Mode detection Confirmed 
+Datasheets mapping </v>
       </c>
       <c r="D3" t="str">
         <v>In progress</v>
@@ -505,7 +506,7 @@
         <v/>
       </c>
       <c r="I3" t="str">
-        <v>2026-08-18 15:07</v>
+        <v>2026-08-19 10:47</v>
       </c>
       <c r="J3" t="str">
         <v>--p6</v>
@@ -952,7 +953,7 @@
         <v>Last saved</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-19 10:41</v>
+        <v>2026-08-19 10:47</v>
       </c>
     </row>
   </sheetData>
@@ -1058,7 +1059,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E1039"/>
+  <dimension ref="A1:E1088"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -18730,9 +18731,842 @@
         <v>2026-08-18</v>
       </c>
     </row>
+    <row r="1040">
+      <c r="A1040" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1040" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1040" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1040" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1040" t="str">
+        <v>M</v>
+      </c>
+    </row>
+    <row r="1041">
+      <c r="A1041" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1041" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1041" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1041" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1041" t="str">
+        <v>Mo</v>
+      </c>
+    </row>
+    <row r="1042">
+      <c r="A1042" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1042" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1042" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1042" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1042" t="str">
+        <v>Mod</v>
+      </c>
+    </row>
+    <row r="1043">
+      <c r="A1043" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1043" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1043" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1043" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1043" t="str">
+        <v>Mode</v>
+      </c>
+    </row>
+    <row r="1044">
+      <c r="A1044" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1044" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1044" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1044" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1044" t="str">
+        <v>Model</v>
+      </c>
+    </row>
+    <row r="1045">
+      <c r="A1045" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1045" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1045" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1045" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1045" t="str">
+        <v xml:space="preserve">Model </v>
+      </c>
+    </row>
+    <row r="1046">
+      <c r="A1046" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1046" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1046" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1046" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1046" t="str">
+        <v>Model</v>
+      </c>
+    </row>
+    <row r="1047">
+      <c r="A1047" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1047" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1047" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1047" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1047" t="str">
+        <v>Mode</v>
+      </c>
+    </row>
+    <row r="1048">
+      <c r="A1048" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1048" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1048" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1048" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1048" t="str">
+        <v xml:space="preserve">Mode </v>
+      </c>
+    </row>
+    <row r="1049">
+      <c r="A1049" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1049" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1049" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1049" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1049" t="str">
+        <v>Mode d</v>
+      </c>
+    </row>
+    <row r="1050">
+      <c r="A1050" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1050" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1050" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1050" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1050" t="str">
+        <v>Mode de</v>
+      </c>
+    </row>
+    <row r="1051">
+      <c r="A1051" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1051" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1051" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1051" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1051" t="str">
+        <v>Mode det</v>
+      </c>
+    </row>
+    <row r="1052">
+      <c r="A1052" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1052" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1052" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1052" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1052" t="str">
+        <v>Mode dete</v>
+      </c>
+    </row>
+    <row r="1053">
+      <c r="A1053" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1053" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1053" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1053" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1053" t="str">
+        <v>Mode detec</v>
+      </c>
+    </row>
+    <row r="1054">
+      <c r="A1054" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1054" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1054" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1054" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1054" t="str">
+        <v>Mode detect</v>
+      </c>
+    </row>
+    <row r="1055">
+      <c r="A1055" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1055" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1055" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1055" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1055" t="str">
+        <v>Mode detecti</v>
+      </c>
+    </row>
+    <row r="1056">
+      <c r="A1056" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1056" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1056" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1056" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1056" t="str">
+        <v>Mode detectio</v>
+      </c>
+    </row>
+    <row r="1057">
+      <c r="A1057" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1057" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1057" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1057" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1057" t="str">
+        <v>Mode detection</v>
+      </c>
+    </row>
+    <row r="1058">
+      <c r="A1058" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1058" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1058" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1058" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1058" t="str">
+        <v xml:space="preserve">Mode detection </v>
+      </c>
+    </row>
+    <row r="1059">
+      <c r="A1059" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1059" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1059" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1059" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1059" t="str">
+        <v>Mode detection C</v>
+      </c>
+    </row>
+    <row r="1060">
+      <c r="A1060" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1060" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1060" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1060" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1060" t="str">
+        <v>Mode detection Co</v>
+      </c>
+    </row>
+    <row r="1061">
+      <c r="A1061" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1061" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1061" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1061" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1061" t="str">
+        <v>Mode detection Con</v>
+      </c>
+    </row>
+    <row r="1062">
+      <c r="A1062" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1062" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1062" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1062" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1062" t="str">
+        <v>Mode detection Conf</v>
+      </c>
+    </row>
+    <row r="1063">
+      <c r="A1063" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1063" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1063" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1063" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1063" t="str">
+        <v>Mode detection Confi</v>
+      </c>
+    </row>
+    <row r="1064">
+      <c r="A1064" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1064" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1064" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1064" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1064" t="str">
+        <v>Mode detection Confir</v>
+      </c>
+    </row>
+    <row r="1065">
+      <c r="A1065" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1065" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1065" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1065" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1065" t="str">
+        <v>Mode detection Confirm</v>
+      </c>
+    </row>
+    <row r="1066">
+      <c r="A1066" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1066" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1066" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1066" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1066" t="str">
+        <v>Mode detection Confirme</v>
+      </c>
+    </row>
+    <row r="1067">
+      <c r="A1067" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1067" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1067" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1067" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1067" t="str">
+        <v>Mode detection Confirmed</v>
+      </c>
+    </row>
+    <row r="1068">
+      <c r="A1068" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1068" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1068" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1068" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1068" t="str">
+        <v xml:space="preserve">Mode detection Confirmed </v>
+      </c>
+    </row>
+    <row r="1069">
+      <c r="A1069" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1069" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1069" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1069" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1069" t="str">
+        <v xml:space="preserve">Mode detection Confirmed  </v>
+      </c>
+    </row>
+    <row r="1070">
+      <c r="A1070" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1070" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1070" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1070" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1070" t="str">
+        <v>Mode detection Confirmed  D</v>
+      </c>
+    </row>
+    <row r="1071">
+      <c r="A1071" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1071" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1071" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1071" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1071" t="str">
+        <v>Mode detection Confirmed  Da</v>
+      </c>
+    </row>
+    <row r="1072">
+      <c r="A1072" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1072" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1072" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1072" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1072" t="str">
+        <v>Mode detection Confirmed  Dat</v>
+      </c>
+    </row>
+    <row r="1073">
+      <c r="A1073" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1073" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1073" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1073" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1073" t="str">
+        <v>Mode detection Confirmed  Data</v>
+      </c>
+    </row>
+    <row r="1074">
+      <c r="A1074" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1074" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1074" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1074" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1074" t="str">
+        <v>Mode detection Confirmed  Datas</v>
+      </c>
+    </row>
+    <row r="1075">
+      <c r="A1075" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1075" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1075" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1075" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1075" t="str">
+        <v>Mode detection Confirmed  Datash</v>
+      </c>
+    </row>
+    <row r="1076">
+      <c r="A1076" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1076" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1076" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1076" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1076" t="str">
+        <v>Mode detection Confirmed  Datashe</v>
+      </c>
+    </row>
+    <row r="1077">
+      <c r="A1077" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1077" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1077" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1077" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1077" t="str">
+        <v>Mode detection Confirmed  Datashee</v>
+      </c>
+    </row>
+    <row r="1078">
+      <c r="A1078" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1078" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1078" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1078" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1078" t="str">
+        <v>Mode detection Confirmed  Datasheet</v>
+      </c>
+    </row>
+    <row r="1079">
+      <c r="A1079" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1079" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1079" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1079" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1079" t="str">
+        <v>Mode detection Confirmed  Datasheets</v>
+      </c>
+    </row>
+    <row r="1080">
+      <c r="A1080" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1080" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1080" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1080" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1080" t="str">
+        <v xml:space="preserve">Mode detection Confirmed  Datasheets </v>
+      </c>
+    </row>
+    <row r="1081">
+      <c r="A1081" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1081" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1081" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1081" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1081" t="str">
+        <v>Mode detection Confirmed  Datasheets m</v>
+      </c>
+    </row>
+    <row r="1082">
+      <c r="A1082" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1082" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1082" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1082" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1082" t="str">
+        <v>Mode detection Confirmed  Datasheets ma</v>
+      </c>
+    </row>
+    <row r="1083">
+      <c r="A1083" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1083" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1083" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1083" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1083" t="str">
+        <v>Mode detection Confirmed  Datasheets map</v>
+      </c>
+    </row>
+    <row r="1084">
+      <c r="A1084" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1084" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1084" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1084" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1084" t="str">
+        <v>Mode detection Confirmed  Datasheets mapp</v>
+      </c>
+    </row>
+    <row r="1085">
+      <c r="A1085" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1085" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1085" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1085" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1085" t="str">
+        <v>Mode detection Confirmed  Datasheets mappi</v>
+      </c>
+    </row>
+    <row r="1086">
+      <c r="A1086" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1086" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1086" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1086" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1086" t="str">
+        <v>Mode detection Confirmed  Datasheets mappin</v>
+      </c>
+    </row>
+    <row r="1087">
+      <c r="A1087" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1087" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1087" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1087" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1087" t="str">
+        <v>Mode detection Confirmed  Datasheets mapping</v>
+      </c>
+    </row>
+    <row r="1088">
+      <c r="A1088" t="str">
+        <v>2026-08-19 10:47</v>
+      </c>
+      <c r="B1088" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1088" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1088" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1088" t="str">
+        <v xml:space="preserve">Mode detection Confirmed  Datasheets mapping </v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E1039"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E1088"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 13 notes, 3 done (2026-08-19 10:48)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -489,7 +489,7 @@
       <c r="C3" t="str" xml:space="preserve">
         <v xml:space="preserve">Mode detection Confirmed 
 Datasheets mapping 
-</v>
+guardrial rules </v>
       </c>
       <c r="D3" t="str">
         <v>In progress</v>
@@ -507,7 +507,7 @@
         <v/>
       </c>
       <c r="I3" t="str">
-        <v>2026-08-19 10:47</v>
+        <v>2026-08-19 10:48</v>
       </c>
       <c r="J3" t="str">
         <v>--p6</v>
@@ -954,7 +954,7 @@
         <v>Last saved</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-19 10:47</v>
+        <v>2026-08-19 10:48</v>
       </c>
     </row>
   </sheetData>
@@ -1060,7 +1060,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E1089"/>
+  <dimension ref="A1:E1105"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -19582,9 +19582,281 @@
         <v xml:space="preserve">Mode detection Confirmed  Datasheets mapping  </v>
       </c>
     </row>
+    <row r="1090">
+      <c r="A1090" t="str">
+        <v>2026-08-19 10:48</v>
+      </c>
+      <c r="B1090" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1090" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1090" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1090" t="str">
+        <v>Mode detection Confirmed  Datasheets mapping  g</v>
+      </c>
+    </row>
+    <row r="1091">
+      <c r="A1091" t="str">
+        <v>2026-08-19 10:48</v>
+      </c>
+      <c r="B1091" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1091" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1091" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1091" t="str">
+        <v>Mode detection Confirmed  Datasheets mapping  gu</v>
+      </c>
+    </row>
+    <row r="1092">
+      <c r="A1092" t="str">
+        <v>2026-08-19 10:48</v>
+      </c>
+      <c r="B1092" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1092" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1092" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1092" t="str">
+        <v>Mode detection Confirmed  Datasheets mapping  gua</v>
+      </c>
+    </row>
+    <row r="1093">
+      <c r="A1093" t="str">
+        <v>2026-08-19 10:48</v>
+      </c>
+      <c r="B1093" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1093" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1093" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1093" t="str">
+        <v>Mode detection Confirmed  Datasheets mapping  guar</v>
+      </c>
+    </row>
+    <row r="1094">
+      <c r="A1094" t="str">
+        <v>2026-08-19 10:48</v>
+      </c>
+      <c r="B1094" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1094" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1094" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1094" t="str">
+        <v>Mode detection Confirmed  Datasheets mapping  guard</v>
+      </c>
+    </row>
+    <row r="1095">
+      <c r="A1095" t="str">
+        <v>2026-08-19 10:48</v>
+      </c>
+      <c r="B1095" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1095" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1095" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1095" t="str">
+        <v>Mode detection Confirmed  Datasheets mapping  guardr</v>
+      </c>
+    </row>
+    <row r="1096">
+      <c r="A1096" t="str">
+        <v>2026-08-19 10:48</v>
+      </c>
+      <c r="B1096" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1096" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1096" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1096" t="str">
+        <v>Mode detection Confirmed  Datasheets mapping  guardri</v>
+      </c>
+    </row>
+    <row r="1097">
+      <c r="A1097" t="str">
+        <v>2026-08-19 10:48</v>
+      </c>
+      <c r="B1097" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1097" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1097" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1097" t="str">
+        <v>Mode detection Confirmed  Datasheets mapping  guardria</v>
+      </c>
+    </row>
+    <row r="1098">
+      <c r="A1098" t="str">
+        <v>2026-08-19 10:48</v>
+      </c>
+      <c r="B1098" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1098" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1098" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1098" t="str">
+        <v>Mode detection Confirmed  Datasheets mapping  guardrial</v>
+      </c>
+    </row>
+    <row r="1099">
+      <c r="A1099" t="str">
+        <v>2026-08-19 10:48</v>
+      </c>
+      <c r="B1099" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1099" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1099" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1099" t="str">
+        <v xml:space="preserve">Mode detection Confirmed  Datasheets mapping  guardrial </v>
+      </c>
+    </row>
+    <row r="1100">
+      <c r="A1100" t="str">
+        <v>2026-08-19 10:48</v>
+      </c>
+      <c r="B1100" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1100" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1100" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1100" t="str">
+        <v>Mode detection Confirmed  Datasheets mapping  guardrial r</v>
+      </c>
+    </row>
+    <row r="1101">
+      <c r="A1101" t="str">
+        <v>2026-08-19 10:48</v>
+      </c>
+      <c r="B1101" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1101" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1101" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1101" t="str">
+        <v>Mode detection Confirmed  Datasheets mapping  guardrial ru</v>
+      </c>
+    </row>
+    <row r="1102">
+      <c r="A1102" t="str">
+        <v>2026-08-19 10:48</v>
+      </c>
+      <c r="B1102" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1102" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1102" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1102" t="str">
+        <v>Mode detection Confirmed  Datasheets mapping  guardrial rul</v>
+      </c>
+    </row>
+    <row r="1103">
+      <c r="A1103" t="str">
+        <v>2026-08-19 10:48</v>
+      </c>
+      <c r="B1103" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1103" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1103" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1103" t="str">
+        <v>Mode detection Confirmed  Datasheets mapping  guardrial rule</v>
+      </c>
+    </row>
+    <row r="1104">
+      <c r="A1104" t="str">
+        <v>2026-08-19 10:48</v>
+      </c>
+      <c r="B1104" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1104" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1104" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1104" t="str">
+        <v>Mode detection Confirmed  Datasheets mapping  guardrial rules</v>
+      </c>
+    </row>
+    <row r="1105">
+      <c r="A1105" t="str">
+        <v>2026-08-19 10:48</v>
+      </c>
+      <c r="B1105" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1105" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1105" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1105" t="str">
+        <v xml:space="preserve">Mode detection Confirmed  Datasheets mapping  guardrial rules </v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E1089"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E1105"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 13 notes, 3 done (2026-08-19 10:49)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -489,7 +489,7 @@
       <c r="C3" t="str" xml:space="preserve">
         <v xml:space="preserve">Mode detection Confirmed 
 Datasheets mapping 
-Guardrial rules </v>
+Guardrials rules </v>
       </c>
       <c r="D3" t="str">
         <v>In progress</v>
@@ -507,7 +507,7 @@
         <v/>
       </c>
       <c r="I3" t="str">
-        <v>2026-08-19 10:48</v>
+        <v>2026-08-19 10:49</v>
       </c>
       <c r="J3" t="str">
         <v>--p6</v>
@@ -954,7 +954,7 @@
         <v>Last saved</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-19 10:48</v>
+        <v>2026-08-19 10:49</v>
       </c>
     </row>
   </sheetData>
@@ -1060,7 +1060,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E1107"/>
+  <dimension ref="A1:E1112"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -19888,9 +19888,94 @@
         <v xml:space="preserve">Mode detection Confirmed  Datasheets mapping  Guardrial rules </v>
       </c>
     </row>
+    <row r="1108">
+      <c r="A1108" t="str">
+        <v>2026-08-19 10:49</v>
+      </c>
+      <c r="B1108" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1108" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1108" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1108" t="str">
+        <v xml:space="preserve">Mode detection Confirmed  Datasheets mapping  Guardrial srules </v>
+      </c>
+    </row>
+    <row r="1109">
+      <c r="A1109" t="str">
+        <v>2026-08-19 10:49</v>
+      </c>
+      <c r="B1109" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1109" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1109" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1109" t="str">
+        <v xml:space="preserve">Mode detection Confirmed  Datasheets mapping  Guardrial rules </v>
+      </c>
+    </row>
+    <row r="1110">
+      <c r="A1110" t="str">
+        <v>2026-08-19 10:49</v>
+      </c>
+      <c r="B1110" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1110" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1110" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1110" t="str">
+        <v xml:space="preserve">Mode detection Confirmed  Datasheets mapping  Guardrialrules </v>
+      </c>
+    </row>
+    <row r="1111">
+      <c r="A1111" t="str">
+        <v>2026-08-19 10:49</v>
+      </c>
+      <c r="B1111" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1111" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1111" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1111" t="str">
+        <v xml:space="preserve">Mode detection Confirmed  Datasheets mapping  Guardrialsrules </v>
+      </c>
+    </row>
+    <row r="1112">
+      <c r="A1112" t="str">
+        <v>2026-08-19 10:49</v>
+      </c>
+      <c r="B1112" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1112" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1112" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1112" t="str">
+        <v xml:space="preserve">Mode detection Confirmed  Datasheets mapping  Guardrials rules </v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E1107"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E1112"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 13 notes, 3 done (2026-08-19 10:50)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -495,7 +495,7 @@
         <v>In progress</v>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="F3" t="str">
         <v>2026-08-17</v>
@@ -507,7 +507,7 @@
         <v/>
       </c>
       <c r="I3" t="str">
-        <v>2026-08-19 10:49</v>
+        <v>2026-08-19 10:50</v>
       </c>
       <c r="J3" t="str">
         <v>--p6</v>
@@ -930,7 +930,7 @@
         <v>Overall progress %</v>
       </c>
       <c r="B6">
-        <v>34</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7">
@@ -954,7 +954,7 @@
         <v>Last saved</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-19 10:49</v>
+        <v>2026-08-19 10:50</v>
       </c>
     </row>
   </sheetData>
@@ -1060,7 +1060,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E1122"/>
+  <dimension ref="A1:E1123"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -20143,9 +20143,26 @@
         <v>Mode detection Confirmed  Datasheets mapping  Guardrials rules  for price</v>
       </c>
     </row>
+    <row r="1123">
+      <c r="A1123" t="str">
+        <v>2026-08-19 10:50</v>
+      </c>
+      <c r="B1123" t="str">
+        <v>T-AMG4458</v>
+      </c>
+      <c r="C1123" t="str">
+        <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
+      </c>
+      <c r="D1123" t="str">
+        <v>Progress updated</v>
+      </c>
+      <c r="E1123" t="str">
+        <v>0% → 60%</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E1122"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E1123"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 14 notes, 3 done (2026-08-19 13:12)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J15"/>
   <cols>
     <col min="1" max="1" width="11.83203125" customWidth="1"/>
     <col min="2" max="2" width="34.83203125" customWidth="1"/>
@@ -446,148 +446,148 @@
         <v>Colour</v>
       </c>
     </row>
-    <row r="2" xml:space="preserve">
+    <row r="2">
       <c r="A2" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="B2" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="C2" t="str">
+        <v/>
+      </c>
+      <c r="D2" t="str">
+        <v>To do</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v>2026-08-19</v>
+      </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
+      <c r="I2" t="str">
+        <v>2026-08-19 13:12</v>
+      </c>
+      <c r="J2" t="str">
+        <v>--p2</v>
+      </c>
+    </row>
+    <row r="3" xml:space="preserve">
+      <c r="A3" t="str">
         <v>T-GVGGA16</v>
       </c>
-      <c r="B2" t="str">
+      <c r="B3" t="str">
         <v>LIN-40309 QS model for CPD</v>
       </c>
-      <c r="C2" t="str" xml:space="preserve">
+      <c r="C3" t="str" xml:space="preserve">
         <v xml:space="preserve">return only queries
 </v>
       </c>
-      <c r="D2" t="str">
+      <c r="D3" t="str">
         <v>In progress</v>
       </c>
-      <c r="E2">
+      <c r="E3">
         <v>0</v>
       </c>
-      <c r="F2" t="str">
+      <c r="F3" t="str">
         <v>2026-08-18</v>
       </c>
-      <c r="G2" t="str">
+      <c r="G3" t="str">
         <v>2026-08-18</v>
       </c>
-      <c r="H2" t="str">
+      <c r="H3" t="str">
         <v/>
       </c>
-      <c r="I2" t="str">
+      <c r="I3" t="str">
         <v>2026-08-18 15:06</v>
       </c>
-      <c r="J2" t="str">
+      <c r="J3" t="str">
         <v>--p1</v>
       </c>
     </row>
-    <row r="3" xml:space="preserve">
-      <c r="A3" t="str">
+    <row r="4" xml:space="preserve">
+      <c r="A4" t="str">
         <v>T-AMG4458</v>
       </c>
-      <c r="B3" t="str">
+      <c r="B4" t="str">
         <v xml:space="preserve">Coveo CPD Observation Checking with Coveo team </v>
       </c>
-      <c r="C3" t="str" xml:space="preserve">
+      <c r="C4" t="str" xml:space="preserve">
         <v xml:space="preserve">Mode detection Confirmed 
 Datasheets mapping 
 Guardrials rules  for price</v>
       </c>
-      <c r="D3" t="str">
+      <c r="D4" t="str">
         <v>In progress</v>
       </c>
-      <c r="E3">
+      <c r="E4">
         <v>60</v>
-      </c>
-      <c r="F3" t="str">
-        <v>2026-08-17</v>
-      </c>
-      <c r="G3" t="str">
-        <v>2026-08-18</v>
-      </c>
-      <c r="H3" t="str">
-        <v/>
-      </c>
-      <c r="I3" t="str">
-        <v>2026-08-19 10:50</v>
-      </c>
-      <c r="J3" t="str">
-        <v>--p6</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>T-8399X61</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Request AO team to add CPD Live endpoint to liquibase</v>
-      </c>
-      <c r="C4" t="str">
-        <v/>
-      </c>
-      <c r="D4" t="str">
-        <v>Done</v>
-      </c>
-      <c r="E4">
-        <v>100</v>
       </c>
       <c r="F4" t="str">
         <v>2026-08-17</v>
       </c>
       <c r="G4" t="str">
+        <v>2026-08-18</v>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v>2026-08-19 10:50</v>
+      </c>
+      <c r="J4" t="str">
+        <v>--p6</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>T-8399X61</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Request AO team to add CPD Live endpoint to liquibase</v>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v>Done</v>
+      </c>
+      <c r="E5">
+        <v>100</v>
+      </c>
+      <c r="F5" t="str">
         <v>2026-08-17</v>
       </c>
-      <c r="H4" t="str">
+      <c r="G5" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H5" t="str">
         <v>2026-08-18</v>
       </c>
-      <c r="I4" t="str">
+      <c r="I5" t="str">
         <v>2026-08-18 12:09</v>
       </c>
-      <c r="J4" t="str">
+      <c r="J5" t="str">
         <v>--p5</v>
       </c>
     </row>
-    <row r="5" xml:space="preserve">
-      <c r="A5" t="str">
+    <row r="6" xml:space="preserve">
+      <c r="A6" t="str">
         <v>T-31URD46</v>
       </c>
-      <c r="B5" t="str">
+      <c r="B6" t="str">
         <v>Coveo RSW(Spain) recommendation Setup</v>
       </c>
-      <c r="C5" t="str" xml:space="preserve">
+      <c r="C6" t="str" xml:space="preserve">
         <v xml:space="preserve">for 
 Julia before 14.7 UAT</v>
       </c>
-      <c r="D5" t="str">
-        <v>To do</v>
-      </c>
-      <c r="E5">
-        <v>0</v>
-      </c>
-      <c r="F5" t="str">
-        <v/>
-      </c>
-      <c r="G5" t="str">
-        <v>2026-08-17</v>
-      </c>
-      <c r="H5" t="str">
-        <v/>
-      </c>
-      <c r="I5" t="str">
-        <v>2026-08-17 15:51</v>
-      </c>
-      <c r="J5" t="str">
-        <v>--p4</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>T-292O348</v>
-      </c>
-      <c r="B6" t="str">
-        <v>SonarQube Resolve</v>
-      </c>
-      <c r="C6" t="str">
-        <v/>
-      </c>
       <c r="D6" t="str">
         <v>To do</v>
       </c>
@@ -604,92 +604,92 @@
         <v/>
       </c>
       <c r="I6" t="str">
-        <v>2026-08-17 15:31</v>
+        <v>2026-08-17 15:51</v>
       </c>
       <c r="J6" t="str">
-        <v>--p3</v>
+        <v>--p4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>T-28A0V57</v>
+        <v>T-292O348</v>
       </c>
       <c r="B7" t="str">
-        <v>Coveo - CPD explanation to Mohan</v>
+        <v>SonarQube Resolve</v>
       </c>
       <c r="C7" t="str">
         <v/>
       </c>
       <c r="D7" t="str">
-        <v>Done</v>
+        <v>To do</v>
       </c>
       <c r="E7">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="F7" t="str">
-        <v>2026-08-18</v>
+        <v/>
       </c>
       <c r="G7" t="str">
         <v>2026-08-17</v>
       </c>
       <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="str">
+        <v>2026-08-17 15:31</v>
+      </c>
+      <c r="J7" t="str">
+        <v>--p3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>T-28A0V57</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Coveo - CPD explanation to Mohan</v>
+      </c>
+      <c r="C8" t="str">
+        <v/>
+      </c>
+      <c r="D8" t="str">
+        <v>Done</v>
+      </c>
+      <c r="E8">
+        <v>100</v>
+      </c>
+      <c r="F8" t="str">
+        <v>2026-08-18</v>
+      </c>
+      <c r="G8" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H8" t="str">
         <v>2026-08-19</v>
       </c>
-      <c r="I7" t="str">
+      <c r="I8" t="str">
         <v>2026-08-19 10:41</v>
       </c>
-      <c r="J7" t="str">
+      <c r="J8" t="str">
         <v>--p2</v>
       </c>
     </row>
-    <row r="8" xml:space="preserve">
-      <c r="A8" t="str">
+    <row r="9" xml:space="preserve">
+      <c r="A9" t="str">
         <v>T-27I6K43</v>
       </c>
-      <c r="B8" t="str">
+      <c r="B9" t="str">
         <v>Coveo CPD Keys and Configuration</v>
       </c>
-      <c r="C8" t="str" xml:space="preserve">
+      <c r="C9" t="str" xml:space="preserve">
         <v xml:space="preserve">Created 42 keys with liquibase 
 still pending...</v>
       </c>
-      <c r="D8" t="str">
+      <c r="D9" t="str">
         <v>In progress</v>
       </c>
-      <c r="E8">
+      <c r="E9">
         <v>90</v>
-      </c>
-      <c r="F8" t="str">
-        <v>2026-08-17</v>
-      </c>
-      <c r="G8" t="str">
-        <v>2026-08-17</v>
-      </c>
-      <c r="H8" t="str">
-        <v/>
-      </c>
-      <c r="I8" t="str">
-        <v>2026-08-18 15:08</v>
-      </c>
-      <c r="J8" t="str">
-        <v>--p1</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>T-24W7H31</v>
-      </c>
-      <c r="B9" t="str">
-        <v xml:space="preserve">CPD - Follow Up for TBD to mathieu </v>
-      </c>
-      <c r="C9" t="str">
-        <v/>
-      </c>
-      <c r="D9" t="str">
-        <v>Done</v>
-      </c>
-      <c r="E9">
-        <v>100</v>
       </c>
       <c r="F9" t="str">
         <v>2026-08-17</v>
@@ -698,92 +698,92 @@
         <v>2026-08-17</v>
       </c>
       <c r="H9" t="str">
+        <v/>
+      </c>
+      <c r="I9" t="str">
+        <v>2026-08-18 15:08</v>
+      </c>
+      <c r="J9" t="str">
+        <v>--p1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>T-24W7H31</v>
+      </c>
+      <c r="B10" t="str">
+        <v xml:space="preserve">CPD - Follow Up for TBD to mathieu </v>
+      </c>
+      <c r="C10" t="str">
+        <v/>
+      </c>
+      <c r="D10" t="str">
+        <v>Done</v>
+      </c>
+      <c r="E10">
+        <v>100</v>
+      </c>
+      <c r="F10" t="str">
         <v>2026-08-17</v>
       </c>
-      <c r="I9" t="str">
+      <c r="G10" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H10" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="I10" t="str">
         <v>2026-08-17 16:51</v>
       </c>
-      <c r="J9" t="str">
+      <c r="J10" t="str">
         <v>--p6</v>
       </c>
     </row>
-    <row r="10" xml:space="preserve">
-      <c r="A10" t="str">
+    <row r="11" xml:space="preserve">
+      <c r="A11" t="str">
         <v>T-22JLI81</v>
       </c>
-      <c r="B10" t="str">
+      <c r="B11" t="str">
         <v xml:space="preserve">Coveo Global Configuration API Deprecation </v>
       </c>
-      <c r="C10" t="str" xml:space="preserve">
+      <c r="C11" t="str" xml:space="preserve">
         <v xml:space="preserve">For 
 RSP, RGG, RSW, BOCT
 To send Send Confirmation mail and Confirm Coveo for Production enablement</v>
       </c>
-      <c r="D10" t="str">
+      <c r="D11" t="str">
         <v>In progress</v>
       </c>
-      <c r="E10">
+      <c r="E11">
         <v>50</v>
       </c>
-      <c r="F10" t="str">
+      <c r="F11" t="str">
         <v>2026-08-21</v>
       </c>
-      <c r="G10" t="str">
+      <c r="G11" t="str">
         <v>2026-08-17</v>
       </c>
-      <c r="H10" t="str">
+      <c r="H11" t="str">
         <v/>
       </c>
-      <c r="I10" t="str">
+      <c r="I11" t="str">
         <v>2026-08-18 15:09</v>
       </c>
-      <c r="J10" t="str">
+      <c r="J11" t="str">
         <v>--p5</v>
       </c>
     </row>
-    <row r="11" xml:space="preserve">
-      <c r="A11" t="str">
+    <row r="12" xml:space="preserve">
+      <c r="A12" t="str">
         <v>T-20UNS57</v>
       </c>
-      <c r="B11" t="str">
+      <c r="B12" t="str">
         <v xml:space="preserve">DF--4191 - New Version Recommendation Model Migration </v>
       </c>
-      <c r="C11" t="str" xml:space="preserve">
+      <c r="C12" t="str" xml:space="preserve">
         <v xml:space="preserve">For 
 RGG and RSW (DE and CH store)</v>
       </c>
-      <c r="D11" t="str">
-        <v>To do</v>
-      </c>
-      <c r="E11">
-        <v>0</v>
-      </c>
-      <c r="F11" t="str">
-        <v>2026-08-21</v>
-      </c>
-      <c r="G11" t="str">
-        <v>2026-08-17</v>
-      </c>
-      <c r="H11" t="str">
-        <v/>
-      </c>
-      <c r="I11" t="str">
-        <v>2026-08-17 16:52</v>
-      </c>
-      <c r="J11" t="str">
-        <v>--p4</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>T-1ZZXI87</v>
-      </c>
-      <c r="B12" t="str">
-        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
-      </c>
-      <c r="C12" t="str">
-        <v xml:space="preserve">For grant </v>
-      </c>
       <c r="D12" t="str">
         <v>To do</v>
       </c>
@@ -791,7 +791,7 @@
         <v>0</v>
       </c>
       <c r="F12" t="str">
-        <v/>
+        <v>2026-08-21</v>
       </c>
       <c r="G12" t="str">
         <v>2026-08-17</v>
@@ -800,21 +800,21 @@
         <v/>
       </c>
       <c r="I12" t="str">
-        <v>2026-08-17 15:21</v>
+        <v>2026-08-17 16:52</v>
       </c>
       <c r="J12" t="str">
-        <v>--p3</v>
+        <v>--p4</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>T-1YYRK56</v>
+        <v>T-1ZZXI87</v>
       </c>
       <c r="B13" t="str">
-        <v>Coveo RSP - Recommendation Go-Live for BOC AU store</v>
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
       </c>
       <c r="C13" t="str">
-        <v>for Grant</v>
+        <v xml:space="preserve">For grant </v>
       </c>
       <c r="D13" t="str">
         <v>To do</v>
@@ -832,21 +832,21 @@
         <v/>
       </c>
       <c r="I13" t="str">
-        <v>2026-08-17 15:20</v>
+        <v>2026-08-17 15:21</v>
       </c>
       <c r="J13" t="str">
-        <v>--p2</v>
+        <v>--p3</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>T-1X4UW94</v>
+        <v>T-1YYRK56</v>
       </c>
       <c r="B14" t="str">
-        <v>Coveo RSP- QPM for V2 calls</v>
+        <v>Coveo RSP - Recommendation Go-Live for BOC AU store</v>
       </c>
       <c r="C14" t="str">
-        <v/>
+        <v>for Grant</v>
       </c>
       <c r="D14" t="str">
         <v>To do</v>
@@ -855,7 +855,7 @@
         <v>0</v>
       </c>
       <c r="F14" t="str">
-        <v>2026-08-14</v>
+        <v/>
       </c>
       <c r="G14" t="str">
         <v>2026-08-17</v>
@@ -864,15 +864,47 @@
         <v/>
       </c>
       <c r="I14" t="str">
+        <v>2026-08-17 15:20</v>
+      </c>
+      <c r="J14" t="str">
+        <v>--p2</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>T-1X4UW94</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Coveo RSP- QPM for V2 calls</v>
+      </c>
+      <c r="C15" t="str">
+        <v/>
+      </c>
+      <c r="D15" t="str">
+        <v>To do</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15" t="str">
+        <v>2026-08-14</v>
+      </c>
+      <c r="G15" t="str">
+        <v>2026-08-17</v>
+      </c>
+      <c r="H15" t="str">
+        <v/>
+      </c>
+      <c r="I15" t="str">
         <v>2026-08-17 17:37</v>
       </c>
-      <c r="J14" t="str">
+      <c r="J15" t="str">
         <v>--p1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J15"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -898,7 +930,7 @@
         <v>Total notes</v>
       </c>
       <c r="B2">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3">
@@ -906,7 +938,7 @@
         <v>To do</v>
       </c>
       <c r="B3">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4">
@@ -930,7 +962,7 @@
         <v>Overall progress %</v>
       </c>
       <c r="B6">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7">
@@ -954,7 +986,7 @@
         <v>Last saved</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-19 10:50</v>
+        <v>2026-08-19 13:12</v>
       </c>
     </row>
   </sheetData>
@@ -1060,7 +1092,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E1123"/>
+  <dimension ref="A1:E1150"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -20160,9 +20192,468 @@
         <v>0% → 60%</v>
       </c>
     </row>
+    <row r="1124">
+      <c r="A1124" t="str">
+        <v>2026-08-19 13:12</v>
+      </c>
+      <c r="B1124" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1124" t="str">
+        <v>(untitled)</v>
+      </c>
+      <c r="D1124" t="str">
+        <v>Created</v>
+      </c>
+      <c r="E1124" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="1125">
+      <c r="A1125" t="str">
+        <v>2026-08-19 13:12</v>
+      </c>
+      <c r="B1125" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1125" t="str">
+        <v>C</v>
+      </c>
+      <c r="D1125" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E1125" t="str">
+        <v>C</v>
+      </c>
+    </row>
+    <row r="1126">
+      <c r="A1126" t="str">
+        <v>2026-08-19 13:12</v>
+      </c>
+      <c r="B1126" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1126" t="str">
+        <v>Co</v>
+      </c>
+      <c r="D1126" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E1126" t="str">
+        <v>Co</v>
+      </c>
+    </row>
+    <row r="1127">
+      <c r="A1127" t="str">
+        <v>2026-08-19 13:12</v>
+      </c>
+      <c r="B1127" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1127" t="str">
+        <v>Cov</v>
+      </c>
+      <c r="D1127" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E1127" t="str">
+        <v>Cov</v>
+      </c>
+    </row>
+    <row r="1128">
+      <c r="A1128" t="str">
+        <v>2026-08-19 13:12</v>
+      </c>
+      <c r="B1128" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1128" t="str">
+        <v>Cove</v>
+      </c>
+      <c r="D1128" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E1128" t="str">
+        <v>Cove</v>
+      </c>
+    </row>
+    <row r="1129">
+      <c r="A1129" t="str">
+        <v>2026-08-19 13:12</v>
+      </c>
+      <c r="B1129" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1129" t="str">
+        <v>Coveo</v>
+      </c>
+      <c r="D1129" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E1129" t="str">
+        <v>Coveo</v>
+      </c>
+    </row>
+    <row r="1130">
+      <c r="A1130" t="str">
+        <v>2026-08-19 13:12</v>
+      </c>
+      <c r="B1130" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1130" t="str">
+        <v xml:space="preserve">Coveo </v>
+      </c>
+      <c r="D1130" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E1130" t="str">
+        <v xml:space="preserve">Coveo </v>
+      </c>
+    </row>
+    <row r="1131">
+      <c r="A1131" t="str">
+        <v>2026-08-19 13:12</v>
+      </c>
+      <c r="B1131" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1131" t="str">
+        <v>Coveo C</v>
+      </c>
+      <c r="D1131" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E1131" t="str">
+        <v>Coveo C</v>
+      </c>
+    </row>
+    <row r="1132">
+      <c r="A1132" t="str">
+        <v>2026-08-19 13:12</v>
+      </c>
+      <c r="B1132" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1132" t="str">
+        <v>Coveo CP</v>
+      </c>
+      <c r="D1132" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E1132" t="str">
+        <v>Coveo CP</v>
+      </c>
+    </row>
+    <row r="1133">
+      <c r="A1133" t="str">
+        <v>2026-08-19 13:12</v>
+      </c>
+      <c r="B1133" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1133" t="str">
+        <v>Coveo CPD</v>
+      </c>
+      <c r="D1133" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E1133" t="str">
+        <v>Coveo CPD</v>
+      </c>
+    </row>
+    <row r="1134">
+      <c r="A1134" t="str">
+        <v>2026-08-19 13:12</v>
+      </c>
+      <c r="B1134" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1134" t="str">
+        <v xml:space="preserve">Coveo CPD </v>
+      </c>
+      <c r="D1134" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E1134" t="str">
+        <v xml:space="preserve">Coveo CPD </v>
+      </c>
+    </row>
+    <row r="1135">
+      <c r="A1135" t="str">
+        <v>2026-08-19 13:12</v>
+      </c>
+      <c r="B1135" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1135" t="str">
+        <v>Coveo CPD D</v>
+      </c>
+      <c r="D1135" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E1135" t="str">
+        <v>Coveo CPD D</v>
+      </c>
+    </row>
+    <row r="1136">
+      <c r="A1136" t="str">
+        <v>2026-08-19 13:12</v>
+      </c>
+      <c r="B1136" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1136" t="str">
+        <v>Coveo CPD De</v>
+      </c>
+      <c r="D1136" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E1136" t="str">
+        <v>Coveo CPD De</v>
+      </c>
+    </row>
+    <row r="1137">
+      <c r="A1137" t="str">
+        <v>2026-08-19 13:12</v>
+      </c>
+      <c r="B1137" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1137" t="str">
+        <v>Coveo CPD Des</v>
+      </c>
+      <c r="D1137" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E1137" t="str">
+        <v>Coveo CPD Des</v>
+      </c>
+    </row>
+    <row r="1138">
+      <c r="A1138" t="str">
+        <v>2026-08-19 13:12</v>
+      </c>
+      <c r="B1138" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1138" t="str">
+        <v>Coveo CPD Desi</v>
+      </c>
+      <c r="D1138" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E1138" t="str">
+        <v>Coveo CPD Desi</v>
+      </c>
+    </row>
+    <row r="1139">
+      <c r="A1139" t="str">
+        <v>2026-08-19 13:12</v>
+      </c>
+      <c r="B1139" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1139" t="str">
+        <v>Coveo CPD Desig</v>
+      </c>
+      <c r="D1139" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E1139" t="str">
+        <v>Coveo CPD Desig</v>
+      </c>
+    </row>
+    <row r="1140">
+      <c r="A1140" t="str">
+        <v>2026-08-19 13:12</v>
+      </c>
+      <c r="B1140" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1140" t="str">
+        <v>Coveo CPD Design</v>
+      </c>
+      <c r="D1140" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E1140" t="str">
+        <v>Coveo CPD Design</v>
+      </c>
+    </row>
+    <row r="1141">
+      <c r="A1141" t="str">
+        <v>2026-08-19 13:12</v>
+      </c>
+      <c r="B1141" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1141" t="str">
+        <v xml:space="preserve">Coveo CPD Design </v>
+      </c>
+      <c r="D1141" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E1141" t="str">
+        <v xml:space="preserve">Coveo CPD Design </v>
+      </c>
+    </row>
+    <row r="1142">
+      <c r="A1142" t="str">
+        <v>2026-08-19 13:12</v>
+      </c>
+      <c r="B1142" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1142" t="str">
+        <v>Coveo CPD Design D</v>
+      </c>
+      <c r="D1142" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E1142" t="str">
+        <v>Coveo CPD Design D</v>
+      </c>
+    </row>
+    <row r="1143">
+      <c r="A1143" t="str">
+        <v>2026-08-19 13:12</v>
+      </c>
+      <c r="B1143" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1143" t="str">
+        <v>Coveo CPD Design Do</v>
+      </c>
+      <c r="D1143" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E1143" t="str">
+        <v>Coveo CPD Design Do</v>
+      </c>
+    </row>
+    <row r="1144">
+      <c r="A1144" t="str">
+        <v>2026-08-19 13:12</v>
+      </c>
+      <c r="B1144" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1144" t="str">
+        <v>Coveo CPD Design Doc</v>
+      </c>
+      <c r="D1144" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E1144" t="str">
+        <v>Coveo CPD Design Doc</v>
+      </c>
+    </row>
+    <row r="1145">
+      <c r="A1145" t="str">
+        <v>2026-08-19 13:12</v>
+      </c>
+      <c r="B1145" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1145" t="str">
+        <v>Coveo CPD Design Docu</v>
+      </c>
+      <c r="D1145" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E1145" t="str">
+        <v>Coveo CPD Design Docu</v>
+      </c>
+    </row>
+    <row r="1146">
+      <c r="A1146" t="str">
+        <v>2026-08-19 13:12</v>
+      </c>
+      <c r="B1146" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1146" t="str">
+        <v>Coveo CPD Design Docum</v>
+      </c>
+      <c r="D1146" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E1146" t="str">
+        <v>Coveo CPD Design Docum</v>
+      </c>
+    </row>
+    <row r="1147">
+      <c r="A1147" t="str">
+        <v>2026-08-19 13:12</v>
+      </c>
+      <c r="B1147" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1147" t="str">
+        <v>Coveo CPD Design Docume</v>
+      </c>
+      <c r="D1147" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E1147" t="str">
+        <v>Coveo CPD Design Docume</v>
+      </c>
+    </row>
+    <row r="1148">
+      <c r="A1148" t="str">
+        <v>2026-08-19 13:12</v>
+      </c>
+      <c r="B1148" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1148" t="str">
+        <v>Coveo CPD Design Documen</v>
+      </c>
+      <c r="D1148" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E1148" t="str">
+        <v>Coveo CPD Design Documen</v>
+      </c>
+    </row>
+    <row r="1149">
+      <c r="A1149" t="str">
+        <v>2026-08-19 13:12</v>
+      </c>
+      <c r="B1149" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1149" t="str">
+        <v>Coveo CPD Design Document</v>
+      </c>
+      <c r="D1149" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E1149" t="str">
+        <v>Coveo CPD Design Document</v>
+      </c>
+    </row>
+    <row r="1150">
+      <c r="A1150" t="str">
+        <v>2026-08-19 13:12</v>
+      </c>
+      <c r="B1150" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1150" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1150" t="str">
+        <v>Title edited</v>
+      </c>
+      <c r="E1150" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E1123"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E1150"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 14 notes, 3 done (2026-08-20 15:31)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -849,13 +849,13 @@
         <v>for Grant</v>
       </c>
       <c r="D14" t="str">
-        <v>To do</v>
+        <v>In progress</v>
       </c>
       <c r="E14">
         <v>0</v>
       </c>
       <c r="F14" t="str">
-        <v/>
+        <v>2026-08-21</v>
       </c>
       <c r="G14" t="str">
         <v>2026-08-17</v>
@@ -864,7 +864,7 @@
         <v/>
       </c>
       <c r="I14" t="str">
-        <v>2026-08-17 15:20</v>
+        <v>2026-08-20 15:30</v>
       </c>
       <c r="J14" t="str">
         <v>--p2</v>
@@ -938,7 +938,7 @@
         <v>To do</v>
       </c>
       <c r="B3">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -946,7 +946,7 @@
         <v>In progress</v>
       </c>
       <c r="B4">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5">
@@ -986,7 +986,7 @@
         <v>Last saved</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-19 13:12</v>
+        <v>2026-08-20 15:31</v>
       </c>
     </row>
   </sheetData>
@@ -1092,7 +1092,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E1153"/>
+  <dimension ref="A1:E1156"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -20702,9 +20702,60 @@
         <v>0% → 70%</v>
       </c>
     </row>
+    <row r="1154">
+      <c r="A1154" t="str">
+        <v>2026-08-20 15:30</v>
+      </c>
+      <c r="B1154" t="str">
+        <v>T-1YYRK56</v>
+      </c>
+      <c r="C1154" t="str">
+        <v>Coveo RSP - Recommendation Go-Live for BOC AU store</v>
+      </c>
+      <c r="D1154" t="str">
+        <v>Due date set</v>
+      </c>
+      <c r="E1154" t="str">
+        <v>2026-08-20</v>
+      </c>
+    </row>
+    <row r="1155">
+      <c r="A1155" t="str">
+        <v>2026-08-20 15:30</v>
+      </c>
+      <c r="B1155" t="str">
+        <v>T-1YYRK56</v>
+      </c>
+      <c r="C1155" t="str">
+        <v>Coveo RSP - Recommendation Go-Live for BOC AU store</v>
+      </c>
+      <c r="D1155" t="str">
+        <v>Due date set</v>
+      </c>
+      <c r="E1155" t="str">
+        <v>2026-08-21</v>
+      </c>
+    </row>
+    <row r="1156">
+      <c r="A1156" t="str">
+        <v>2026-08-20 15:30</v>
+      </c>
+      <c r="B1156" t="str">
+        <v>T-1YYRK56</v>
+      </c>
+      <c r="C1156" t="str">
+        <v>Coveo RSP - Recommendation Go-Live for BOC AU store</v>
+      </c>
+      <c r="D1156" t="str">
+        <v>Status changed</v>
+      </c>
+      <c r="E1156" t="str">
+        <v>To do → In progress</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E1153"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E1156"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 14 notes, 3 done (2026-08-20 15:32)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -806,15 +806,16 @@
         <v>--p4</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" xml:space="preserve">
       <c r="A13" t="str">
         <v>T-1ZZXI87</v>
       </c>
       <c r="B13" t="str">
         <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
       </c>
-      <c r="C13" t="str">
-        <v xml:space="preserve">For grant </v>
+      <c r="C13" t="str" xml:space="preserve">
+        <v xml:space="preserve">Grant approved it...
+need to plan for 14.8</v>
       </c>
       <c r="D13" t="str">
         <v>To do</v>
@@ -832,7 +833,7 @@
         <v/>
       </c>
       <c r="I13" t="str">
-        <v>2026-08-17 15:21</v>
+        <v>2026-08-20 15:31</v>
       </c>
       <c r="J13" t="str">
         <v>--p3</v>
@@ -986,7 +987,7 @@
         <v>Last saved</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-20 15:31</v>
+        <v>2026-08-20 15:32</v>
       </c>
     </row>
   </sheetData>
@@ -1092,7 +1093,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E1200"/>
+  <dimension ref="A1:E1278"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -21501,9 +21502,1335 @@
         <v>Needs to send estimation to Grant</v>
       </c>
     </row>
+    <row r="1201">
+      <c r="A1201" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1201" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1201" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1201" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1201" t="str">
+        <v>For grant</v>
+      </c>
+    </row>
+    <row r="1202">
+      <c r="A1202" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1202" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1202" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1202" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1202" t="str">
+        <v>For gran</v>
+      </c>
+    </row>
+    <row r="1203">
+      <c r="A1203" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1203" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1203" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1203" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1203" t="str">
+        <v>For gra</v>
+      </c>
+    </row>
+    <row r="1204">
+      <c r="A1204" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1204" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1204" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1204" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1204" t="str">
+        <v>For gr</v>
+      </c>
+    </row>
+    <row r="1205">
+      <c r="A1205" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1205" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1205" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1205" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1205" t="str">
+        <v>For g</v>
+      </c>
+    </row>
+    <row r="1206">
+      <c r="A1206" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1206" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1206" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1206" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1206" t="str">
+        <v xml:space="preserve">For </v>
+      </c>
+    </row>
+    <row r="1207">
+      <c r="A1207" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1207" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1207" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1207" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1207" t="str">
+        <v>For</v>
+      </c>
+    </row>
+    <row r="1208">
+      <c r="A1208" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1208" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1208" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1208" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1208" t="str">
+        <v>Fo</v>
+      </c>
+    </row>
+    <row r="1209">
+      <c r="A1209" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1209" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1209" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1209" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1209" t="str">
+        <v>F</v>
+      </c>
+    </row>
+    <row r="1210">
+      <c r="A1210" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1210" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1210" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1210" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1210" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="1211">
+      <c r="A1211" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1211" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1211" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1211" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1211" t="str">
+        <v>G</v>
+      </c>
+    </row>
+    <row r="1212">
+      <c r="A1212" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1212" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1212" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1212" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1212" t="str">
+        <v>Gr</v>
+      </c>
+    </row>
+    <row r="1213">
+      <c r="A1213" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1213" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1213" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1213" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1213" t="str">
+        <v>Gra</v>
+      </c>
+    </row>
+    <row r="1214">
+      <c r="A1214" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1214" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1214" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1214" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1214" t="str">
+        <v>Gran</v>
+      </c>
+    </row>
+    <row r="1215">
+      <c r="A1215" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1215" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1215" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1215" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1215" t="str">
+        <v>Grant</v>
+      </c>
+    </row>
+    <row r="1216">
+      <c r="A1216" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1216" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1216" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1216" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1216" t="str">
+        <v xml:space="preserve">Grant </v>
+      </c>
+    </row>
+    <row r="1217">
+      <c r="A1217" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1217" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1217" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1217" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1217" t="str">
+        <v>Grant s</v>
+      </c>
+    </row>
+    <row r="1218">
+      <c r="A1218" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1218" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1218" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1218" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1218" t="str">
+        <v>Grant sh</v>
+      </c>
+    </row>
+    <row r="1219">
+      <c r="A1219" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1219" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1219" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1219" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1219" t="str">
+        <v>Grant sha</v>
+      </c>
+    </row>
+    <row r="1220">
+      <c r="A1220" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1220" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1220" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1220" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1220" t="str">
+        <v>Grant shar</v>
+      </c>
+    </row>
+    <row r="1221">
+      <c r="A1221" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1221" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1221" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1221" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1221" t="str">
+        <v>Grant share</v>
+      </c>
+    </row>
+    <row r="1222">
+      <c r="A1222" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1222" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1222" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1222" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1222" t="str">
+        <v>Grant shared</v>
+      </c>
+    </row>
+    <row r="1223">
+      <c r="A1223" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1223" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1223" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1223" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1223" t="str">
+        <v>Grant share</v>
+      </c>
+    </row>
+    <row r="1224">
+      <c r="A1224" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1224" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1224" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1224" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1224" t="str">
+        <v>Grant shar</v>
+      </c>
+    </row>
+    <row r="1225">
+      <c r="A1225" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1225" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1225" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1225" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1225" t="str">
+        <v>Grant sha</v>
+      </c>
+    </row>
+    <row r="1226">
+      <c r="A1226" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1226" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1226" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1226" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1226" t="str">
+        <v>Grant sh</v>
+      </c>
+    </row>
+    <row r="1227">
+      <c r="A1227" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1227" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1227" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1227" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1227" t="str">
+        <v>Grant s</v>
+      </c>
+    </row>
+    <row r="1228">
+      <c r="A1228" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1228" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1228" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1228" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1228" t="str">
+        <v xml:space="preserve">Grant </v>
+      </c>
+    </row>
+    <row r="1229">
+      <c r="A1229" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1229" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1229" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1229" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1229" t="str">
+        <v>Grant a</v>
+      </c>
+    </row>
+    <row r="1230">
+      <c r="A1230" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1230" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1230" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1230" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1230" t="str">
+        <v>Grant ap</v>
+      </c>
+    </row>
+    <row r="1231">
+      <c r="A1231" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1231" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1231" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1231" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1231" t="str">
+        <v>Grant app</v>
+      </c>
+    </row>
+    <row r="1232">
+      <c r="A1232" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1232" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1232" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1232" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1232" t="str">
+        <v>Grant appr</v>
+      </c>
+    </row>
+    <row r="1233">
+      <c r="A1233" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1233" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1233" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1233" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1233" t="str">
+        <v>Grant appro</v>
+      </c>
+    </row>
+    <row r="1234">
+      <c r="A1234" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1234" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1234" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1234" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1234" t="str">
+        <v>Grant approv</v>
+      </c>
+    </row>
+    <row r="1235">
+      <c r="A1235" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1235" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1235" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1235" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1235" t="str">
+        <v>Grant approve</v>
+      </c>
+    </row>
+    <row r="1236">
+      <c r="A1236" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1236" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1236" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1236" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1236" t="str">
+        <v>Grant approved</v>
+      </c>
+    </row>
+    <row r="1237">
+      <c r="A1237" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1237" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1237" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1237" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1237" t="str">
+        <v xml:space="preserve">Grant approved </v>
+      </c>
+    </row>
+    <row r="1238">
+      <c r="A1238" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1238" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1238" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1238" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1238" t="str">
+        <v>Grant approved i</v>
+      </c>
+    </row>
+    <row r="1239">
+      <c r="A1239" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1239" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1239" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1239" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1239" t="str">
+        <v>Grant approved it</v>
+      </c>
+    </row>
+    <row r="1240">
+      <c r="A1240" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1240" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1240" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1240" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1240" t="str">
+        <v xml:space="preserve">Grant approved it </v>
+      </c>
+    </row>
+    <row r="1241">
+      <c r="A1241" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1241" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1241" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1241" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1241" t="str">
+        <v>Grant approved it</v>
+      </c>
+    </row>
+    <row r="1242">
+      <c r="A1242" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1242" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1242" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1242" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1242" t="str">
+        <v>Grant approved it.</v>
+      </c>
+    </row>
+    <row r="1243">
+      <c r="A1243" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1243" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1243" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1243" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1243" t="str">
+        <v>Grant approved it..</v>
+      </c>
+    </row>
+    <row r="1244">
+      <c r="A1244" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1244" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1244" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1244" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1244" t="str">
+        <v>Grant approved it...</v>
+      </c>
+    </row>
+    <row r="1245">
+      <c r="A1245" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1245" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1245" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1245" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1245" t="str">
+        <v xml:space="preserve">Grant approved it... </v>
+      </c>
+    </row>
+    <row r="1246">
+      <c r="A1246" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1246" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1246" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1246" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1246" t="str">
+        <v>Grant approved it... n</v>
+      </c>
+    </row>
+    <row r="1247">
+      <c r="A1247" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1247" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1247" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1247" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1247" t="str">
+        <v>Grant approved it... ne</v>
+      </c>
+    </row>
+    <row r="1248">
+      <c r="A1248" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1248" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1248" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1248" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1248" t="str">
+        <v>Grant approved it... nee</v>
+      </c>
+    </row>
+    <row r="1249">
+      <c r="A1249" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1249" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1249" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1249" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1249" t="str">
+        <v>Grant approved it... need</v>
+      </c>
+    </row>
+    <row r="1250">
+      <c r="A1250" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1250" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1250" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1250" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1250" t="str">
+        <v xml:space="preserve">Grant approved it... need </v>
+      </c>
+    </row>
+    <row r="1251">
+      <c r="A1251" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1251" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1251" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1251" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1251" t="str">
+        <v>Grant approved it... need t</v>
+      </c>
+    </row>
+    <row r="1252">
+      <c r="A1252" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1252" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1252" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1252" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1252" t="str">
+        <v>Grant approved it... need to</v>
+      </c>
+    </row>
+    <row r="1253">
+      <c r="A1253" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1253" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1253" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1253" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1253" t="str">
+        <v xml:space="preserve">Grant approved it... need to </v>
+      </c>
+    </row>
+    <row r="1254">
+      <c r="A1254" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1254" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1254" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1254" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1254" t="str">
+        <v>Grant approved it... need to p</v>
+      </c>
+    </row>
+    <row r="1255">
+      <c r="A1255" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1255" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1255" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1255" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1255" t="str">
+        <v>Grant approved it... need to pa</v>
+      </c>
+    </row>
+    <row r="1256">
+      <c r="A1256" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1256" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1256" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1256" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1256" t="str">
+        <v>Grant approved it... need to pal</v>
+      </c>
+    </row>
+    <row r="1257">
+      <c r="A1257" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1257" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1257" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1257" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1257" t="str">
+        <v>Grant approved it... need to paln</v>
+      </c>
+    </row>
+    <row r="1258">
+      <c r="A1258" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1258" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1258" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1258" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1258" t="str">
+        <v xml:space="preserve">Grant approved it... need to paln </v>
+      </c>
+    </row>
+    <row r="1259">
+      <c r="A1259" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1259" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1259" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1259" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1259" t="str">
+        <v>Grant approved it... need to paln</v>
+      </c>
+    </row>
+    <row r="1260">
+      <c r="A1260" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1260" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1260" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1260" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1260" t="str">
+        <v>Grant approved it... need to pal</v>
+      </c>
+    </row>
+    <row r="1261">
+      <c r="A1261" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1261" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1261" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1261" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1261" t="str">
+        <v>Grant approved it... need to pa</v>
+      </c>
+    </row>
+    <row r="1262">
+      <c r="A1262" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1262" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1262" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1262" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1262" t="str">
+        <v>Grant approved it... need to paa</v>
+      </c>
+    </row>
+    <row r="1263">
+      <c r="A1263" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1263" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1263" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1263" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1263" t="str">
+        <v>Grant approved it... need to pa</v>
+      </c>
+    </row>
+    <row r="1264">
+      <c r="A1264" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1264" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1264" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1264" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1264" t="str">
+        <v>Grant approved it... need to p</v>
+      </c>
+    </row>
+    <row r="1265">
+      <c r="A1265" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1265" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1265" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1265" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1265" t="str">
+        <v>Grant approved it... need to pl</v>
+      </c>
+    </row>
+    <row r="1266">
+      <c r="A1266" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1266" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1266" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1266" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1266" t="str">
+        <v>Grant approved it... need to pla</v>
+      </c>
+    </row>
+    <row r="1267">
+      <c r="A1267" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1267" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1267" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1267" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1267" t="str">
+        <v>Grant approved it... need to plan</v>
+      </c>
+    </row>
+    <row r="1268">
+      <c r="A1268" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1268" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1268" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1268" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1268" t="str">
+        <v xml:space="preserve">Grant approved it... need to plan </v>
+      </c>
+    </row>
+    <row r="1269">
+      <c r="A1269" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1269" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1269" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1269" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1269" t="str">
+        <v>Grant approved it... need to plan f</v>
+      </c>
+    </row>
+    <row r="1270">
+      <c r="A1270" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1270" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1270" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1270" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1270" t="str">
+        <v>Grant approved it... need to plan fo</v>
+      </c>
+    </row>
+    <row r="1271">
+      <c r="A1271" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1271" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1271" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1271" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1271" t="str">
+        <v>Grant approved it... need to plan for</v>
+      </c>
+    </row>
+    <row r="1272">
+      <c r="A1272" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1272" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1272" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1272" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1272" t="str">
+        <v xml:space="preserve">Grant approved it... need to plan for </v>
+      </c>
+    </row>
+    <row r="1273">
+      <c r="A1273" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1273" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1273" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1273" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1273" t="str">
+        <v>Grant approved it... need to plan for 1</v>
+      </c>
+    </row>
+    <row r="1274">
+      <c r="A1274" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1274" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1274" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1274" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1274" t="str">
+        <v>Grant approved it... need to plan for 14</v>
+      </c>
+    </row>
+    <row r="1275">
+      <c r="A1275" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1275" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1275" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1275" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1275" t="str">
+        <v>Grant approved it... need to plan for 14.</v>
+      </c>
+    </row>
+    <row r="1276">
+      <c r="A1276" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1276" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1276" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1276" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1276" t="str">
+        <v>Grant approved it... need to plan for 14.6</v>
+      </c>
+    </row>
+    <row r="1277">
+      <c r="A1277" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1277" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1277" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1277" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1277" t="str">
+        <v>Grant approved it... need to plan for 14.</v>
+      </c>
+    </row>
+    <row r="1278">
+      <c r="A1278" t="str">
+        <v>2026-08-20 15:31</v>
+      </c>
+      <c r="B1278" t="str">
+        <v>T-1ZZXI87</v>
+      </c>
+      <c r="C1278" t="str">
+        <v xml:space="preserve">Coveo - RSP   AU SPW store </v>
+      </c>
+      <c r="D1278" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1278" t="str">
+        <v>Grant approved it... need to plan for 14.8</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E1200"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E1278"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 14 notes, 4 done (2026-08-20 15:32)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -454,25 +454,25 @@
         <v xml:space="preserve">Coveo CPD Design Document </v>
       </c>
       <c r="C2" t="str">
-        <v/>
+        <v>Design doc done and Explained to Team</v>
       </c>
       <c r="D2" t="str">
-        <v>In progress</v>
+        <v>Done</v>
       </c>
       <c r="E2">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-08-18</v>
+        <v>2026-08-19</v>
       </c>
       <c r="G2" t="str">
         <v>2026-08-19</v>
       </c>
       <c r="H2" t="str">
-        <v/>
+        <v>2026-08-20</v>
       </c>
       <c r="I2" t="str">
-        <v>2026-08-19 13:12</v>
+        <v>2026-08-20 15:32</v>
       </c>
       <c r="J2" t="str">
         <v>--p2</v>
@@ -947,7 +947,7 @@
         <v>In progress</v>
       </c>
       <c r="B4">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
@@ -955,7 +955,7 @@
         <v>Done</v>
       </c>
       <c r="B5">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -963,7 +963,7 @@
         <v>Overall progress %</v>
       </c>
       <c r="B6">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7">
@@ -971,7 +971,7 @@
         <v>Overdue</v>
       </c>
       <c r="B7">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
@@ -1093,7 +1093,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E1278"/>
+  <dimension ref="A1:E1355"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -22828,9 +22828,1318 @@
         <v>Grant approved it... need to plan for 14.8</v>
       </c>
     </row>
+    <row r="1279">
+      <c r="A1279" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1279" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1279" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1279" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1279" t="str">
+        <v>D</v>
+      </c>
+    </row>
+    <row r="1280">
+      <c r="A1280" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1280" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1280" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1280" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1280" t="str">
+        <v>Di</v>
+      </c>
+    </row>
+    <row r="1281">
+      <c r="A1281" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1281" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1281" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1281" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1281" t="str">
+        <v>D</v>
+      </c>
+    </row>
+    <row r="1282">
+      <c r="A1282" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1282" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1282" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1282" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1282" t="str">
+        <v>De</v>
+      </c>
+    </row>
+    <row r="1283">
+      <c r="A1283" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1283" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1283" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1283" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1283" t="str">
+        <v>Des</v>
+      </c>
+    </row>
+    <row r="1284">
+      <c r="A1284" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1284" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1284" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1284" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1284" t="str">
+        <v>Desi</v>
+      </c>
+    </row>
+    <row r="1285">
+      <c r="A1285" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1285" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1285" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1285" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1285" t="str">
+        <v>Desig</v>
+      </c>
+    </row>
+    <row r="1286">
+      <c r="A1286" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1286" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1286" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1286" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1286" t="str">
+        <v>Design</v>
+      </c>
+    </row>
+    <row r="1287">
+      <c r="A1287" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1287" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1287" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1287" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1287" t="str">
+        <v xml:space="preserve">Design </v>
+      </c>
+    </row>
+    <row r="1288">
+      <c r="A1288" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1288" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1288" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1288" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1288" t="str">
+        <v>Design d</v>
+      </c>
+    </row>
+    <row r="1289">
+      <c r="A1289" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1289" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1289" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1289" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1289" t="str">
+        <v>Design do</v>
+      </c>
+    </row>
+    <row r="1290">
+      <c r="A1290" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1290" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1290" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1290" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1290" t="str">
+        <v>Design don</v>
+      </c>
+    </row>
+    <row r="1291">
+      <c r="A1291" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1291" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1291" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1291" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1291" t="str">
+        <v>Design do</v>
+      </c>
+    </row>
+    <row r="1292">
+      <c r="A1292" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1292" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1292" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1292" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1292" t="str">
+        <v>Design doc</v>
+      </c>
+    </row>
+    <row r="1293">
+      <c r="A1293" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1293" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1293" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1293" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1293" t="str">
+        <v xml:space="preserve">Design doc </v>
+      </c>
+    </row>
+    <row r="1294">
+      <c r="A1294" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1294" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1294" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1294" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1294" t="str">
+        <v>Design doc d</v>
+      </c>
+    </row>
+    <row r="1295">
+      <c r="A1295" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1295" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1295" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1295" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1295" t="str">
+        <v>Design doc do</v>
+      </c>
+    </row>
+    <row r="1296">
+      <c r="A1296" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1296" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1296" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1296" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1296" t="str">
+        <v>Design doc don</v>
+      </c>
+    </row>
+    <row r="1297">
+      <c r="A1297" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1297" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1297" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1297" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1297" t="str">
+        <v>Design doc done</v>
+      </c>
+    </row>
+    <row r="1298">
+      <c r="A1298" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1298" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1298" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1298" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1298" t="str">
+        <v xml:space="preserve">Design doc done </v>
+      </c>
+    </row>
+    <row r="1299">
+      <c r="A1299" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1299" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1299" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1299" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1299" t="str">
+        <v>Design doc done a</v>
+      </c>
+    </row>
+    <row r="1300">
+      <c r="A1300" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1300" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1300" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1300" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1300" t="str">
+        <v>Design doc done an</v>
+      </c>
+    </row>
+    <row r="1301">
+      <c r="A1301" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1301" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1301" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1301" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1301" t="str">
+        <v>Design doc done and</v>
+      </c>
+    </row>
+    <row r="1302">
+      <c r="A1302" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1302" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1302" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1302" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1302" t="str">
+        <v xml:space="preserve">Design doc done and </v>
+      </c>
+    </row>
+    <row r="1303">
+      <c r="A1303" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1303" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1303" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1303" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1303" t="str">
+        <v>Design doc done and E</v>
+      </c>
+    </row>
+    <row r="1304">
+      <c r="A1304" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1304" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1304" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1304" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1304" t="str">
+        <v>Design doc done and Ex</v>
+      </c>
+    </row>
+    <row r="1305">
+      <c r="A1305" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1305" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1305" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1305" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1305" t="str">
+        <v>Design doc done and Exp</v>
+      </c>
+    </row>
+    <row r="1306">
+      <c r="A1306" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1306" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1306" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1306" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1306" t="str">
+        <v>Design doc done and Expl</v>
+      </c>
+    </row>
+    <row r="1307">
+      <c r="A1307" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1307" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1307" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1307" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1307" t="str">
+        <v>Design doc done and Expla</v>
+      </c>
+    </row>
+    <row r="1308">
+      <c r="A1308" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1308" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1308" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1308" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1308" t="str">
+        <v>Design doc done and Explai</v>
+      </c>
+    </row>
+    <row r="1309">
+      <c r="A1309" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1309" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1309" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1309" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1309" t="str">
+        <v>Design doc done and Explain</v>
+      </c>
+    </row>
+    <row r="1310">
+      <c r="A1310" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1310" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1310" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1310" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1310" t="str">
+        <v>Design doc done and Explaine</v>
+      </c>
+    </row>
+    <row r="1311">
+      <c r="A1311" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1311" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1311" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1311" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1311" t="str">
+        <v xml:space="preserve">Design doc done and Explaine </v>
+      </c>
+    </row>
+    <row r="1312">
+      <c r="A1312" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1312" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1312" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1312" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1312" t="str">
+        <v>Design doc done and Explaine d</v>
+      </c>
+    </row>
+    <row r="1313">
+      <c r="A1313" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1313" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1313" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1313" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1313" t="str">
+        <v>Design doc done and Explaine dt</v>
+      </c>
+    </row>
+    <row r="1314">
+      <c r="A1314" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1314" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1314" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1314" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1314" t="str">
+        <v>Design doc done and Explaine d</v>
+      </c>
+    </row>
+    <row r="1315">
+      <c r="A1315" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1315" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1315" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1315" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1315" t="str">
+        <v xml:space="preserve">Design doc done and Explaine </v>
+      </c>
+    </row>
+    <row r="1316">
+      <c r="A1316" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1316" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1316" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1316" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1316" t="str">
+        <v>Design doc done and Explaine</v>
+      </c>
+    </row>
+    <row r="1317">
+      <c r="A1317" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1317" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1317" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1317" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1317" t="str">
+        <v>Design doc done and Explain</v>
+      </c>
+    </row>
+    <row r="1318">
+      <c r="A1318" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1318" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1318" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1318" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1318" t="str">
+        <v>Design doc done and Explai</v>
+      </c>
+    </row>
+    <row r="1319">
+      <c r="A1319" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1319" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1319" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1319" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1319" t="str">
+        <v>Design doc done and Expla</v>
+      </c>
+    </row>
+    <row r="1320">
+      <c r="A1320" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1320" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1320" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1320" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1320" t="str">
+        <v>Design doc done and Expl</v>
+      </c>
+    </row>
+    <row r="1321">
+      <c r="A1321" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1321" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1321" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1321" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1321" t="str">
+        <v>Design doc done and Exp</v>
+      </c>
+    </row>
+    <row r="1322">
+      <c r="A1322" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1322" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1322" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1322" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1322" t="str">
+        <v>Design doc done and Expi</v>
+      </c>
+    </row>
+    <row r="1323">
+      <c r="A1323" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1323" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1323" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1323" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1323" t="str">
+        <v>Design doc done and Expin</v>
+      </c>
+    </row>
+    <row r="1324">
+      <c r="A1324" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1324" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1324" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1324" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1324" t="str">
+        <v>Design doc done and Expine</v>
+      </c>
+    </row>
+    <row r="1325">
+      <c r="A1325" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1325" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1325" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1325" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1325" t="str">
+        <v>Design doc done and Expined</v>
+      </c>
+    </row>
+    <row r="1326">
+      <c r="A1326" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1326" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1326" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1326" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1326" t="str">
+        <v xml:space="preserve">Design doc done and Expined </v>
+      </c>
+    </row>
+    <row r="1327">
+      <c r="A1327" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1327" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1327" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1327" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1327" t="str">
+        <v>Design doc done and Expined t</v>
+      </c>
+    </row>
+    <row r="1328">
+      <c r="A1328" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1328" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1328" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1328" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1328" t="str">
+        <v>Design doc done and Expined to</v>
+      </c>
+    </row>
+    <row r="1329">
+      <c r="A1329" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1329" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1329" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1329" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1329" t="str">
+        <v>Design doc done and Expined t</v>
+      </c>
+    </row>
+    <row r="1330">
+      <c r="A1330" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1330" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1330" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1330" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1330" t="str">
+        <v xml:space="preserve">Design doc done and Expined </v>
+      </c>
+    </row>
+    <row r="1331">
+      <c r="A1331" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1331" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1331" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1331" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1331" t="str">
+        <v>Design doc done and Expined</v>
+      </c>
+    </row>
+    <row r="1332">
+      <c r="A1332" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1332" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1332" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1332" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1332" t="str">
+        <v>Design doc done and Expine</v>
+      </c>
+    </row>
+    <row r="1333">
+      <c r="A1333" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1333" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1333" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1333" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1333" t="str">
+        <v>Design doc done and Expin</v>
+      </c>
+    </row>
+    <row r="1334">
+      <c r="A1334" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1334" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1334" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1334" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1334" t="str">
+        <v>Design doc done and Expi</v>
+      </c>
+    </row>
+    <row r="1335">
+      <c r="A1335" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1335" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1335" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1335" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1335" t="str">
+        <v>Design doc done and Exp</v>
+      </c>
+    </row>
+    <row r="1336">
+      <c r="A1336" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1336" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1336" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1336" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1336" t="str">
+        <v>Design doc done and Ex</v>
+      </c>
+    </row>
+    <row r="1337">
+      <c r="A1337" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1337" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1337" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1337" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1337" t="str">
+        <v>Design doc done and Exp</v>
+      </c>
+    </row>
+    <row r="1338">
+      <c r="A1338" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1338" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1338" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1338" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1338" t="str">
+        <v>Design doc done and Expl</v>
+      </c>
+    </row>
+    <row r="1339">
+      <c r="A1339" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1339" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1339" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1339" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1339" t="str">
+        <v>Design doc done and Expla</v>
+      </c>
+    </row>
+    <row r="1340">
+      <c r="A1340" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1340" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1340" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1340" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1340" t="str">
+        <v>Design doc done and Explai</v>
+      </c>
+    </row>
+    <row r="1341">
+      <c r="A1341" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1341" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1341" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1341" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1341" t="str">
+        <v>Design doc done and Explain</v>
+      </c>
+    </row>
+    <row r="1342">
+      <c r="A1342" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1342" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1342" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1342" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1342" t="str">
+        <v>Design doc done and Explaine</v>
+      </c>
+    </row>
+    <row r="1343">
+      <c r="A1343" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1343" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1343" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1343" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1343" t="str">
+        <v>Design doc done and Explained</v>
+      </c>
+    </row>
+    <row r="1344">
+      <c r="A1344" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1344" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1344" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1344" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1344" t="str">
+        <v xml:space="preserve">Design doc done and Explained </v>
+      </c>
+    </row>
+    <row r="1345">
+      <c r="A1345" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1345" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1345" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1345" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1345" t="str">
+        <v>Design doc done and Explained t</v>
+      </c>
+    </row>
+    <row r="1346">
+      <c r="A1346" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1346" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1346" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1346" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1346" t="str">
+        <v>Design doc done and Explained to</v>
+      </c>
+    </row>
+    <row r="1347">
+      <c r="A1347" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1347" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1347" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1347" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1347" t="str">
+        <v xml:space="preserve">Design doc done and Explained to </v>
+      </c>
+    </row>
+    <row r="1348">
+      <c r="A1348" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1348" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1348" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1348" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1348" t="str">
+        <v>Design doc done and Explained to T</v>
+      </c>
+    </row>
+    <row r="1349">
+      <c r="A1349" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1349" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1349" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1349" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1349" t="str">
+        <v>Design doc done and Explained to TE</v>
+      </c>
+    </row>
+    <row r="1350">
+      <c r="A1350" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1350" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1350" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1350" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1350" t="str">
+        <v>Design doc done and Explained to T</v>
+      </c>
+    </row>
+    <row r="1351">
+      <c r="A1351" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1351" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1351" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1351" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1351" t="str">
+        <v>Design doc done and Explained to Te</v>
+      </c>
+    </row>
+    <row r="1352">
+      <c r="A1352" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1352" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1352" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1352" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1352" t="str">
+        <v>Design doc done and Explained to Tea</v>
+      </c>
+    </row>
+    <row r="1353">
+      <c r="A1353" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1353" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1353" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1353" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1353" t="str">
+        <v>Design doc done and Explained to Team</v>
+      </c>
+    </row>
+    <row r="1354">
+      <c r="A1354" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1354" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1354" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1354" t="str">
+        <v>Due date set</v>
+      </c>
+      <c r="E1354" t="str">
+        <v>2026-08-19</v>
+      </c>
+    </row>
+    <row r="1355">
+      <c r="A1355" t="str">
+        <v>2026-08-20 15:32</v>
+      </c>
+      <c r="B1355" t="str">
+        <v>T-SAE6Z76</v>
+      </c>
+      <c r="C1355" t="str">
+        <v xml:space="preserve">Coveo CPD Design Document </v>
+      </c>
+      <c r="D1355" t="str">
+        <v>Status changed</v>
+      </c>
+      <c r="E1355" t="str">
+        <v>In progress → Done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E1278"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E1355"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 14 notes, 4 done (2026-08-20 15:33)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -505,7 +505,7 @@
         <v/>
       </c>
       <c r="I3" t="str">
-        <v>2026-08-18 15:06</v>
+        <v>2026-08-20 15:33</v>
       </c>
       <c r="J3" t="str">
         <v>--p1</v>
@@ -987,7 +987,7 @@
         <v>Last saved</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-20 15:32</v>
+        <v>2026-08-20 15:33</v>
       </c>
     </row>
   </sheetData>
@@ -1093,7 +1093,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E1355"/>
+  <dimension ref="A1:E1356"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -24137,9 +24137,26 @@
         <v>In progress → Done</v>
       </c>
     </row>
+    <row r="1356">
+      <c r="A1356" t="str">
+        <v>2026-08-20 15:33</v>
+      </c>
+      <c r="B1356" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1356" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1356" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1356" t="str">
+        <v xml:space="preserve">return only queries  </v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E1355"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E1356"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 14 notes, 4 done (2026-08-20 15:36)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -487,6 +487,8 @@
       </c>
       <c r="C3" t="str" xml:space="preserve">
         <v xml:space="preserve">return only queries
+Committed Keys and configuration 
+FE is pending 
 </v>
       </c>
       <c r="D3" t="str">
@@ -505,7 +507,7 @@
         <v/>
       </c>
       <c r="I3" t="str">
-        <v>2026-08-20 15:33</v>
+        <v>2026-08-20 15:36</v>
       </c>
       <c r="J3" t="str">
         <v>--p1</v>
@@ -987,7 +989,7 @@
         <v>Last saved</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-20 15:33</v>
+        <v>2026-08-20 15:36</v>
       </c>
     </row>
   </sheetData>
@@ -1093,7 +1095,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E1356"/>
+  <dimension ref="A1:E1404"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -24154,9 +24156,825 @@
         <v xml:space="preserve">return only queries  </v>
       </c>
     </row>
+    <row r="1357">
+      <c r="A1357" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1357" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1357" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1357" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1357" t="str">
+        <v xml:space="preserve">return only queries C </v>
+      </c>
+    </row>
+    <row r="1358">
+      <c r="A1358" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1358" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1358" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1358" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1358" t="str">
+        <v xml:space="preserve">return only queries Co </v>
+      </c>
+    </row>
+    <row r="1359">
+      <c r="A1359" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1359" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1359" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1359" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1359" t="str">
+        <v xml:space="preserve">return only queries Com </v>
+      </c>
+    </row>
+    <row r="1360">
+      <c r="A1360" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1360" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1360" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1360" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1360" t="str">
+        <v xml:space="preserve">return only queries Comm </v>
+      </c>
+    </row>
+    <row r="1361">
+      <c r="A1361" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1361" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1361" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1361" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1361" t="str">
+        <v xml:space="preserve">return only queries Commi </v>
+      </c>
+    </row>
+    <row r="1362">
+      <c r="A1362" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1362" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1362" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1362" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1362" t="str">
+        <v xml:space="preserve">return only queries Commit </v>
+      </c>
+    </row>
+    <row r="1363">
+      <c r="A1363" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1363" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1363" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1363" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1363" t="str">
+        <v xml:space="preserve">return only queries Committ </v>
+      </c>
+    </row>
+    <row r="1364">
+      <c r="A1364" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1364" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1364" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1364" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1364" t="str">
+        <v xml:space="preserve">return only queries Committe </v>
+      </c>
+    </row>
+    <row r="1365">
+      <c r="A1365" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1365" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1365" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1365" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1365" t="str">
+        <v xml:space="preserve">return only queries Committed </v>
+      </c>
+    </row>
+    <row r="1366">
+      <c r="A1366" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1366" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1366" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1366" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1366" t="str">
+        <v xml:space="preserve">return only queries Committed  </v>
+      </c>
+    </row>
+    <row r="1367">
+      <c r="A1367" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1367" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1367" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1367" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1367" t="str">
+        <v xml:space="preserve">return only queries Committed K </v>
+      </c>
+    </row>
+    <row r="1368">
+      <c r="A1368" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1368" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1368" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1368" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1368" t="str">
+        <v xml:space="preserve">return only queries Committed Ke </v>
+      </c>
+    </row>
+    <row r="1369">
+      <c r="A1369" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1369" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1369" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1369" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1369" t="str">
+        <v xml:space="preserve">return only queries Committed Key </v>
+      </c>
+    </row>
+    <row r="1370">
+      <c r="A1370" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1370" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1370" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1370" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1370" t="str">
+        <v xml:space="preserve">return only queries Committed Keys </v>
+      </c>
+    </row>
+    <row r="1371">
+      <c r="A1371" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1371" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1371" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1371" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1371" t="str">
+        <v xml:space="preserve">return only queries Committed Keys  </v>
+      </c>
+    </row>
+    <row r="1372">
+      <c r="A1372" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1372" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1372" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1372" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1372" t="str">
+        <v xml:space="preserve">return only queries Committed Keys a </v>
+      </c>
+    </row>
+    <row r="1373">
+      <c r="A1373" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1373" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1373" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1373" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1373" t="str">
+        <v xml:space="preserve">return only queries Committed Keys an </v>
+      </c>
+    </row>
+    <row r="1374">
+      <c r="A1374" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1374" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1374" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1374" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1374" t="str">
+        <v xml:space="preserve">return only queries Committed Keys and </v>
+      </c>
+    </row>
+    <row r="1375">
+      <c r="A1375" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1375" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1375" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1375" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1375" t="str">
+        <v xml:space="preserve">return only queries Committed Keys and  </v>
+      </c>
+    </row>
+    <row r="1376">
+      <c r="A1376" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1376" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1376" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1376" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1376" t="str">
+        <v xml:space="preserve">return only queries Committed Keys and c </v>
+      </c>
+    </row>
+    <row r="1377">
+      <c r="A1377" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1377" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1377" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1377" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1377" t="str">
+        <v xml:space="preserve">return only queries Committed Keys and co </v>
+      </c>
+    </row>
+    <row r="1378">
+      <c r="A1378" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1378" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1378" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1378" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1378" t="str">
+        <v xml:space="preserve">return only queries Committed Keys and con </v>
+      </c>
+    </row>
+    <row r="1379">
+      <c r="A1379" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1379" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1379" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1379" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1379" t="str">
+        <v xml:space="preserve">return only queries Committed Keys and conf </v>
+      </c>
+    </row>
+    <row r="1380">
+      <c r="A1380" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1380" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1380" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1380" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1380" t="str">
+        <v xml:space="preserve">return only queries Committed Keys and confi </v>
+      </c>
+    </row>
+    <row r="1381">
+      <c r="A1381" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1381" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1381" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1381" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1381" t="str">
+        <v xml:space="preserve">return only queries Committed Keys and config </v>
+      </c>
+    </row>
+    <row r="1382">
+      <c r="A1382" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1382" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1382" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1382" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1382" t="str">
+        <v xml:space="preserve">return only queries Committed Keys and configu </v>
+      </c>
+    </row>
+    <row r="1383">
+      <c r="A1383" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1383" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1383" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1383" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1383" t="str">
+        <v xml:space="preserve">return only queries Committed Keys and configur </v>
+      </c>
+    </row>
+    <row r="1384">
+      <c r="A1384" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1384" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1384" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1384" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1384" t="str">
+        <v xml:space="preserve">return only queries Committed Keys and configura </v>
+      </c>
+    </row>
+    <row r="1385">
+      <c r="A1385" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1385" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1385" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1385" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1385" t="str">
+        <v xml:space="preserve">return only queries Committed Keys and configurat </v>
+      </c>
+    </row>
+    <row r="1386">
+      <c r="A1386" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1386" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1386" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1386" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1386" t="str">
+        <v xml:space="preserve">return only queries Committed Keys and configurati </v>
+      </c>
+    </row>
+    <row r="1387">
+      <c r="A1387" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1387" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1387" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1387" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1387" t="str">
+        <v xml:space="preserve">return only queries Committed Keys and configuratio </v>
+      </c>
+    </row>
+    <row r="1388">
+      <c r="A1388" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1388" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1388" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1388" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1388" t="str">
+        <v xml:space="preserve">return only queries Committed Keys and configuration </v>
+      </c>
+    </row>
+    <row r="1389">
+      <c r="A1389" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1389" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1389" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1389" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1389" t="str">
+        <v xml:space="preserve">return only queries Committed Keys and configuration  </v>
+      </c>
+    </row>
+    <row r="1390">
+      <c r="A1390" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1390" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1390" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1390" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1390" t="str">
+        <v xml:space="preserve">return only queries Committed Keys and configuration   </v>
+      </c>
+    </row>
+    <row r="1391">
+      <c r="A1391" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1391" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1391" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1391" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1391" t="str">
+        <v xml:space="preserve">return only queries Committed Keys and configuration  F </v>
+      </c>
+    </row>
+    <row r="1392">
+      <c r="A1392" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1392" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1392" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1392" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1392" t="str">
+        <v xml:space="preserve">return only queries Committed Keys and configuration  FE </v>
+      </c>
+    </row>
+    <row r="1393">
+      <c r="A1393" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1393" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1393" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1393" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1393" t="str">
+        <v xml:space="preserve">return only queries Committed Keys and configuration  FE  </v>
+      </c>
+    </row>
+    <row r="1394">
+      <c r="A1394" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1394" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1394" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1394" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1394" t="str">
+        <v xml:space="preserve">return only queries Committed Keys and configuration  FE i </v>
+      </c>
+    </row>
+    <row r="1395">
+      <c r="A1395" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1395" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1395" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1395" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1395" t="str">
+        <v xml:space="preserve">return only queries Committed Keys and configuration  FE is </v>
+      </c>
+    </row>
+    <row r="1396">
+      <c r="A1396" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1396" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1396" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1396" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1396" t="str">
+        <v xml:space="preserve">return only queries Committed Keys and configuration  FE is  </v>
+      </c>
+    </row>
+    <row r="1397">
+      <c r="A1397" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1397" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1397" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1397" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1397" t="str">
+        <v xml:space="preserve">return only queries Committed Keys and configuration  FE is p </v>
+      </c>
+    </row>
+    <row r="1398">
+      <c r="A1398" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1398" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1398" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1398" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1398" t="str">
+        <v xml:space="preserve">return only queries Committed Keys and configuration  FE is pe </v>
+      </c>
+    </row>
+    <row r="1399">
+      <c r="A1399" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1399" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1399" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1399" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1399" t="str">
+        <v xml:space="preserve">return only queries Committed Keys and configuration  FE is pen </v>
+      </c>
+    </row>
+    <row r="1400">
+      <c r="A1400" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1400" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1400" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1400" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1400" t="str">
+        <v xml:space="preserve">return only queries Committed Keys and configuration  FE is pend </v>
+      </c>
+    </row>
+    <row r="1401">
+      <c r="A1401" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1401" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1401" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1401" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1401" t="str">
+        <v xml:space="preserve">return only queries Committed Keys and configuration  FE is pendi </v>
+      </c>
+    </row>
+    <row r="1402">
+      <c r="A1402" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1402" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1402" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1402" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1402" t="str">
+        <v xml:space="preserve">return only queries Committed Keys and configuration  FE is pendin </v>
+      </c>
+    </row>
+    <row r="1403">
+      <c r="A1403" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1403" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1403" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1403" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1403" t="str">
+        <v xml:space="preserve">return only queries Committed Keys and configuration  FE is pending </v>
+      </c>
+    </row>
+    <row r="1404">
+      <c r="A1404" t="str">
+        <v>2026-08-20 15:36</v>
+      </c>
+      <c r="B1404" t="str">
+        <v>T-GVGGA16</v>
+      </c>
+      <c r="C1404" t="str">
+        <v>LIN-40309 QS model for CPD</v>
+      </c>
+      <c r="D1404" t="str">
+        <v>Notes updated</v>
+      </c>
+      <c r="E1404" t="str">
+        <v xml:space="preserve">return only queries Committed Keys and configuration  FE is pending  </v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E1356"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E1404"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 14 notes, 4 done (2026-08-21 15:12)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -787,7 +787,7 @@
 RGG and RSW (DE and CH store)</v>
       </c>
       <c r="D12" t="str">
-        <v>To do</v>
+        <v>In progress</v>
       </c>
       <c r="E12">
         <v>0</v>
@@ -802,7 +802,7 @@
         <v/>
       </c>
       <c r="I12" t="str">
-        <v>2026-08-17 16:52</v>
+        <v>2026-08-21 15:12</v>
       </c>
       <c r="J12" t="str">
         <v>--p4</v>
@@ -941,7 +941,7 @@
         <v>To do</v>
       </c>
       <c r="B3">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -949,7 +949,7 @@
         <v>In progress</v>
       </c>
       <c r="B4">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5">
@@ -989,7 +989,7 @@
         <v>Last saved</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-20 15:36</v>
+        <v>2026-08-21 15:12</v>
       </c>
     </row>
   </sheetData>
@@ -1095,7 +1095,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E1404"/>
+  <dimension ref="A1:E1405"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -24972,9 +24972,26 @@
         <v xml:space="preserve">return only queries Committed Keys and configuration  FE is pending  </v>
       </c>
     </row>
+    <row r="1405">
+      <c r="A1405" t="str">
+        <v>2026-08-21 15:12</v>
+      </c>
+      <c r="B1405" t="str">
+        <v>T-20UNS57</v>
+      </c>
+      <c r="C1405" t="str">
+        <v xml:space="preserve">DF--4191 - New Version Recommendation Model Migration </v>
+      </c>
+      <c r="D1405" t="str">
+        <v>Status changed</v>
+      </c>
+      <c r="E1405" t="str">
+        <v>To do → In progress</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E1404"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E1405"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update board — 14 notes, 6 done (2026-08-21 15:13)
</commit_message>
<xml_diff>
--- a/data/todo-board.xlsx
+++ b/data/todo-board.xlsx
@@ -787,10 +787,10 @@
 RGG and RSW (DE and CH store)</v>
       </c>
       <c r="D12" t="str">
-        <v>In progress</v>
+        <v>Done</v>
       </c>
       <c r="E12">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="F12" t="str">
         <v>2026-08-21</v>
@@ -799,10 +799,10 @@
         <v>2026-08-17</v>
       </c>
       <c r="H12" t="str">
-        <v/>
+        <v>2026-08-21</v>
       </c>
       <c r="I12" t="str">
-        <v>2026-08-21 15:12</v>
+        <v>2026-08-21 15:13</v>
       </c>
       <c r="J12" t="str">
         <v>--p4</v>
@@ -852,10 +852,10 @@
         <v>for Grant</v>
       </c>
       <c r="D14" t="str">
-        <v>In progress</v>
+        <v>Done</v>
       </c>
       <c r="E14">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="F14" t="str">
         <v>2026-08-21</v>
@@ -864,10 +864,10 @@
         <v>2026-08-17</v>
       </c>
       <c r="H14" t="str">
-        <v/>
+        <v>2026-08-21</v>
       </c>
       <c r="I14" t="str">
-        <v>2026-08-20 15:30</v>
+        <v>2026-08-21 15:13</v>
       </c>
       <c r="J14" t="str">
         <v>--p2</v>
@@ -949,7 +949,7 @@
         <v>In progress</v>
       </c>
       <c r="B4">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -957,7 +957,7 @@
         <v>Done</v>
       </c>
       <c r="B5">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
@@ -965,7 +965,7 @@
         <v>Overall progress %</v>
       </c>
       <c r="B6">
-        <v>43</v>
+        <v>57</v>
       </c>
     </row>
     <row r="7">
@@ -989,7 +989,7 @@
         <v>Last saved</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-08-21 15:12</v>
+        <v>2026-08-21 15:13</v>
       </c>
     </row>
   </sheetData>
@@ -1095,7 +1095,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E1405"/>
+  <dimension ref="A1:E1407"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -24989,9 +24989,43 @@
         <v>To do → In progress</v>
       </c>
     </row>
+    <row r="1406">
+      <c r="A1406" t="str">
+        <v>2026-08-21 15:13</v>
+      </c>
+      <c r="B1406" t="str">
+        <v>T-1YYRK56</v>
+      </c>
+      <c r="C1406" t="str">
+        <v>Coveo RSP - Recommendation Go-Live for BOC AU store</v>
+      </c>
+      <c r="D1406" t="str">
+        <v>Status changed</v>
+      </c>
+      <c r="E1406" t="str">
+        <v>In progress → Done</v>
+      </c>
+    </row>
+    <row r="1407">
+      <c r="A1407" t="str">
+        <v>2026-08-21 15:13</v>
+      </c>
+      <c r="B1407" t="str">
+        <v>T-20UNS57</v>
+      </c>
+      <c r="C1407" t="str">
+        <v xml:space="preserve">DF--4191 - New Version Recommendation Model Migration </v>
+      </c>
+      <c r="D1407" t="str">
+        <v>Status changed</v>
+      </c>
+      <c r="E1407" t="str">
+        <v>In progress → Done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E1405"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E1407"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>